<commit_message>
var að laga persónulegu stigin, count á hverju atriði var ekki rétt
</commit_message>
<xml_diff>
--- a/03_26_schedule_results.xlsx
+++ b/03_26_schedule_results.xlsx
@@ -535,11 +535,11 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -587,11 +587,11 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J3" t="n">
@@ -607,7 +607,7 @@
         <v>40</v>
       </c>
       <c r="N3" t="n">
-        <v>420</v>
+        <v>410</v>
       </c>
     </row>
     <row r="4">
@@ -639,18 +639,18 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J4" t="n">
         <v>2</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L4" t="n">
         <v>3</v>
@@ -659,7 +659,7 @@
         <v>40</v>
       </c>
       <c r="N4" t="n">
-        <v>420</v>
+        <v>510</v>
       </c>
     </row>
     <row r="5">
@@ -691,18 +691,18 @@
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Nanna</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
         <v>3</v>
@@ -711,7 +711,7 @@
         <v>40</v>
       </c>
       <c r="N5" t="n">
-        <v>540</v>
+        <v>420</v>
       </c>
     </row>
     <row r="6">
@@ -743,18 +743,18 @@
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Össur</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L6" t="n">
         <v>3</v>
@@ -763,7 +763,7 @@
         <v>80</v>
       </c>
       <c r="N6" t="n">
-        <v>470</v>
+        <v>490</v>
       </c>
     </row>
     <row r="7">
@@ -795,18 +795,18 @@
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J7" t="n">
         <v>2</v>
       </c>
       <c r="K7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L7" t="n">
         <v>3</v>
@@ -815,7 +815,7 @@
         <v>80</v>
       </c>
       <c r="N7" t="n">
-        <v>470</v>
+        <v>460</v>
       </c>
     </row>
     <row r="8">
@@ -899,18 +899,18 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Össur</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L9" t="n">
         <v>3</v>
@@ -951,18 +951,18 @@
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L10" t="n">
         <v>3</v>
@@ -971,7 +971,7 @@
         <v>80</v>
       </c>
       <c r="N10" t="n">
-        <v>470</v>
+        <v>520</v>
       </c>
     </row>
     <row r="11">
@@ -1055,11 +1055,11 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J12" t="n">
@@ -1075,7 +1075,7 @@
         <v>40</v>
       </c>
       <c r="N12" t="n">
-        <v>340</v>
+        <v>400</v>
       </c>
     </row>
     <row r="13">
@@ -1107,15 +1107,15 @@
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Camilla</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K13" t="n">
         <v>1</v>
@@ -1127,7 +1127,7 @@
         <v>40</v>
       </c>
       <c r="N13" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
     </row>
     <row r="14">
@@ -1887,15 +1887,15 @@
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -1907,7 +1907,7 @@
         <v>80</v>
       </c>
       <c r="N28" t="n">
-        <v>440</v>
+        <v>480</v>
       </c>
     </row>
     <row r="29">
@@ -1939,11 +1939,11 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J29" t="n">
@@ -1991,18 +1991,18 @@
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Össur</t>
+          <t>Ásdís</t>
         </is>
       </c>
       <c r="J30" t="n">
         <v>3</v>
       </c>
       <c r="K30" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L30" t="n">
         <v>3.5</v>
@@ -2011,7 +2011,7 @@
         <v>50</v>
       </c>
       <c r="N30" t="n">
-        <v>540</v>
+        <v>500</v>
       </c>
     </row>
     <row r="31">
@@ -2043,18 +2043,18 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
+        <v>3</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Össur</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>3</v>
+      </c>
+      <c r="K31" t="n">
         <v>7</v>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>Harpa</t>
-        </is>
-      </c>
-      <c r="J31" t="n">
-        <v>2</v>
-      </c>
-      <c r="K31" t="n">
-        <v>2</v>
       </c>
       <c r="L31" t="n">
         <v>3.5</v>
@@ -2063,7 +2063,7 @@
         <v>50</v>
       </c>
       <c r="N31" t="n">
-        <v>390</v>
+        <v>540</v>
       </c>
     </row>
     <row r="32">
@@ -2095,18 +2095,18 @@
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Thelma</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L32" t="n">
         <v>3.5</v>
@@ -2115,7 +2115,7 @@
         <v>50</v>
       </c>
       <c r="N32" t="n">
-        <v>510</v>
+        <v>500</v>
       </c>
     </row>
     <row r="33">
@@ -2147,11 +2147,11 @@
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J33" t="n">
@@ -2167,7 +2167,7 @@
         <v>50</v>
       </c>
       <c r="N33" t="n">
-        <v>410</v>
+        <v>400</v>
       </c>
     </row>
     <row r="34">
@@ -2199,18 +2199,18 @@
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J34" t="n">
         <v>2</v>
       </c>
       <c r="K34" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L34" t="n">
         <v>3.5</v>
@@ -2219,7 +2219,7 @@
         <v>50</v>
       </c>
       <c r="N34" t="n">
-        <v>540</v>
+        <v>390</v>
       </c>
     </row>
     <row r="35">
@@ -2303,18 +2303,18 @@
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J36" t="n">
         <v>2</v>
       </c>
       <c r="K36" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L36" t="n">
         <v>3.5</v>
@@ -2323,7 +2323,7 @@
         <v>50</v>
       </c>
       <c r="N36" t="n">
-        <v>530</v>
+        <v>390</v>
       </c>
     </row>
     <row r="37">
@@ -2355,18 +2355,18 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J37" t="n">
         <v>2</v>
       </c>
       <c r="K37" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L37" t="n">
         <v>3.5</v>
@@ -2375,7 +2375,7 @@
         <v>50</v>
       </c>
       <c r="N37" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
     </row>
     <row r="38">
@@ -2407,18 +2407,18 @@
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J38" t="n">
         <v>2</v>
       </c>
       <c r="K38" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L38" t="n">
         <v>3.5</v>
@@ -2427,7 +2427,7 @@
         <v>50</v>
       </c>
       <c r="N38" t="n">
-        <v>390</v>
+        <v>530</v>
       </c>
     </row>
     <row r="39">
@@ -2459,18 +2459,18 @@
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Nanna</t>
         </is>
       </c>
       <c r="J39" t="n">
         <v>1</v>
       </c>
       <c r="K39" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L39" t="n">
         <v>3.5</v>
@@ -2479,7 +2479,7 @@
         <v>50</v>
       </c>
       <c r="N39" t="n">
-        <v>560</v>
+        <v>550</v>
       </c>
     </row>
     <row r="40">
@@ -2511,18 +2511,18 @@
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Camilla</t>
+          <t>Gunnar</t>
         </is>
       </c>
       <c r="J40" t="n">
         <v>1</v>
       </c>
       <c r="K40" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L40" t="n">
         <v>3.5</v>
@@ -2531,7 +2531,7 @@
         <v>50</v>
       </c>
       <c r="N40" t="n">
-        <v>550</v>
+        <v>560</v>
       </c>
     </row>
     <row r="41">
@@ -2563,18 +2563,18 @@
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Helgi</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K41" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L41" t="n">
         <v>4</v>
@@ -2615,18 +2615,18 @@
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J42" t="n">
         <v>2</v>
       </c>
       <c r="K42" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L42" t="n">
         <v>4</v>
@@ -2635,7 +2635,7 @@
         <v>50</v>
       </c>
       <c r="N42" t="n">
-        <v>530</v>
+        <v>560</v>
       </c>
     </row>
     <row r="43">
@@ -2990,7 +2990,7 @@
         <v>1</v>
       </c>
       <c r="K49" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L49" t="n">
         <v>4</v>
@@ -2999,7 +2999,7 @@
         <v>50</v>
       </c>
       <c r="N49" t="n">
-        <v>560</v>
+        <v>490</v>
       </c>
     </row>
     <row r="50">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Gunnar</t>
+          <t>Ólafur</t>
         </is>
       </c>
       <c r="J51" t="n">
@@ -3103,7 +3103,7 @@
         <v>50</v>
       </c>
       <c r="N51" t="n">
-        <v>560</v>
+        <v>500</v>
       </c>
     </row>
     <row r="52">
@@ -3198,7 +3198,7 @@
         <v>2</v>
       </c>
       <c r="K53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L53" t="n">
         <v>4</v>
@@ -3250,7 +3250,7 @@
         <v>2</v>
       </c>
       <c r="K54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L54" t="n">
         <v>4</v>
@@ -3291,18 +3291,18 @@
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J55" t="n">
         <v>2</v>
       </c>
       <c r="K55" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L55" t="n">
         <v>4</v>
@@ -3311,7 +3311,7 @@
         <v>50</v>
       </c>
       <c r="N55" t="n">
-        <v>560</v>
+        <v>350</v>
       </c>
     </row>
     <row r="56">
@@ -3343,18 +3343,18 @@
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J56" t="n">
         <v>2</v>
       </c>
       <c r="K56" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L56" t="n">
         <v>4</v>
@@ -3363,7 +3363,7 @@
         <v>50</v>
       </c>
       <c r="N56" t="n">
-        <v>360</v>
+        <v>560</v>
       </c>
     </row>
     <row r="57">
@@ -3395,18 +3395,18 @@
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J57" t="n">
         <v>2</v>
       </c>
       <c r="K57" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L57" t="n">
         <v>4</v>
@@ -3415,7 +3415,7 @@
         <v>50</v>
       </c>
       <c r="N57" t="n">
-        <v>560</v>
+        <v>360</v>
       </c>
     </row>
     <row r="58">
@@ -3447,18 +3447,18 @@
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J58" t="n">
         <v>2</v>
       </c>
       <c r="K58" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="L58" t="n">
         <v>4</v>
@@ -3467,7 +3467,7 @@
         <v>50</v>
       </c>
       <c r="N58" t="n">
-        <v>390</v>
+        <v>560</v>
       </c>
     </row>
     <row r="59">
@@ -3499,18 +3499,18 @@
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J59" t="n">
         <v>2</v>
       </c>
       <c r="K59" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L59" t="n">
         <v>4</v>
@@ -3519,7 +3519,7 @@
         <v>50</v>
       </c>
       <c r="N59" t="n">
-        <v>560</v>
+        <v>390</v>
       </c>
     </row>
     <row r="60">
@@ -3551,18 +3551,18 @@
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J60" t="n">
         <v>2</v>
       </c>
       <c r="K60" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L60" t="n">
         <v>4</v>
@@ -3571,7 +3571,7 @@
         <v>50</v>
       </c>
       <c r="N60" t="n">
-        <v>390</v>
+        <v>560</v>
       </c>
     </row>
     <row r="61">
@@ -3666,7 +3666,7 @@
         <v>1</v>
       </c>
       <c r="K62" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="L62" t="n">
         <v>4</v>
@@ -3675,7 +3675,7 @@
         <v>50</v>
       </c>
       <c r="N62" t="n">
-        <v>570</v>
+        <v>550</v>
       </c>
     </row>
     <row r="63">
@@ -3718,7 +3718,7 @@
         <v>2</v>
       </c>
       <c r="K63" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L63" t="n">
         <v>4</v>
@@ -3978,7 +3978,7 @@
         <v>1</v>
       </c>
       <c r="K68" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L68" t="n">
         <v>4</v>
@@ -3987,7 +3987,7 @@
         <v>70</v>
       </c>
       <c r="N68" t="n">
-        <v>510</v>
+        <v>430</v>
       </c>
     </row>
     <row r="69">
@@ -4030,7 +4030,7 @@
         <v>1</v>
       </c>
       <c r="K69" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L69" t="n">
         <v>4</v>
@@ -4071,18 +4071,18 @@
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L70" t="n">
         <v>4.5</v>
@@ -4091,7 +4091,7 @@
         <v>100</v>
       </c>
       <c r="N70" t="n">
-        <v>480</v>
+        <v>440</v>
       </c>
     </row>
     <row r="71">
@@ -4123,18 +4123,18 @@
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="n">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Bergur</t>
         </is>
       </c>
       <c r="J71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L71" t="n">
         <v>4.5</v>
@@ -4143,7 +4143,7 @@
         <v>100</v>
       </c>
       <c r="N71" t="n">
-        <v>440</v>
+        <v>480</v>
       </c>
     </row>
     <row r="72">
@@ -4175,11 +4175,11 @@
       </c>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J72" t="n">
@@ -4195,7 +4195,7 @@
         <v>100</v>
       </c>
       <c r="N72" t="n">
-        <v>480</v>
+        <v>490</v>
       </c>
     </row>
     <row r="73">
@@ -4227,11 +4227,11 @@
       </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Helgi</t>
+          <t>Ásdís</t>
         </is>
       </c>
       <c r="J73" t="n">
@@ -4247,7 +4247,7 @@
         <v>50</v>
       </c>
       <c r="N73" t="n">
-        <v>560</v>
+        <v>550</v>
       </c>
     </row>
     <row r="74">
@@ -4290,7 +4290,7 @@
         <v>2</v>
       </c>
       <c r="K74" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L74" t="n">
         <v>3.5</v>
@@ -4299,7 +4299,7 @@
         <v>50</v>
       </c>
       <c r="N74" t="n">
-        <v>410</v>
+        <v>520</v>
       </c>
     </row>
     <row r="75">
@@ -4331,18 +4331,18 @@
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J75" t="n">
         <v>2</v>
       </c>
       <c r="K75" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L75" t="n">
         <v>3.5</v>
@@ -4351,7 +4351,7 @@
         <v>50</v>
       </c>
       <c r="N75" t="n">
-        <v>390</v>
+        <v>410</v>
       </c>
     </row>
     <row r="76">
@@ -4383,18 +4383,18 @@
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K76" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L76" t="n">
         <v>3.5</v>
@@ -4403,7 +4403,7 @@
         <v>50</v>
       </c>
       <c r="N76" t="n">
-        <v>550</v>
+        <v>530</v>
       </c>
     </row>
     <row r="77">
@@ -4435,18 +4435,18 @@
       </c>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J77" t="n">
         <v>2</v>
       </c>
       <c r="K77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L77" t="n">
         <v>3.5</v>
@@ -4487,18 +4487,18 @@
       </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K78" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="L78" t="n">
         <v>3.5</v>
@@ -4507,7 +4507,7 @@
         <v>50</v>
       </c>
       <c r="N78" t="n">
-        <v>510</v>
+        <v>550</v>
       </c>
     </row>
     <row r="79">
@@ -4539,18 +4539,18 @@
       </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J79" t="n">
         <v>2</v>
       </c>
       <c r="K79" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L79" t="n">
         <v>3.5</v>
@@ -4559,7 +4559,7 @@
         <v>50</v>
       </c>
       <c r="N79" t="n">
-        <v>520</v>
+        <v>390</v>
       </c>
     </row>
     <row r="80">
@@ -4591,18 +4591,18 @@
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J80" t="n">
         <v>2</v>
       </c>
       <c r="K80" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L80" t="n">
         <v>3.5</v>
@@ -4643,18 +4643,18 @@
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J81" t="n">
         <v>2</v>
       </c>
       <c r="K81" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L81" t="n">
         <v>3.5</v>
@@ -4663,7 +4663,7 @@
         <v>50</v>
       </c>
       <c r="N81" t="n">
-        <v>520</v>
+        <v>510</v>
       </c>
     </row>
     <row r="82">
@@ -4851,11 +4851,11 @@
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Ásdís</t>
+          <t>Thelma</t>
         </is>
       </c>
       <c r="J85" t="n">
@@ -4871,7 +4871,7 @@
         <v>50</v>
       </c>
       <c r="N85" t="n">
-        <v>570</v>
+        <v>550</v>
       </c>
     </row>
     <row r="86">
@@ -4903,18 +4903,18 @@
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Thelma</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J86" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K86" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="L86" t="n">
         <v>4</v>
@@ -4923,7 +4923,7 @@
         <v>50</v>
       </c>
       <c r="N86" t="n">
-        <v>570</v>
+        <v>510</v>
       </c>
     </row>
     <row r="87">
@@ -4955,18 +4955,18 @@
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J87" t="n">
         <v>2</v>
       </c>
       <c r="K87" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L87" t="n">
         <v>4</v>
@@ -4975,7 +4975,7 @@
         <v>50</v>
       </c>
       <c r="N87" t="n">
-        <v>390</v>
+        <v>380</v>
       </c>
     </row>
     <row r="88">
@@ -5007,18 +5007,18 @@
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J88" t="n">
         <v>2</v>
       </c>
       <c r="K88" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L88" t="n">
         <v>4</v>
@@ -5059,18 +5059,18 @@
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J89" t="n">
         <v>2</v>
       </c>
       <c r="K89" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L89" t="n">
         <v>4</v>
@@ -5111,18 +5111,18 @@
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J90" t="n">
         <v>2</v>
       </c>
       <c r="K90" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L90" t="n">
         <v>4</v>
@@ -5163,18 +5163,18 @@
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J91" t="n">
         <v>2</v>
       </c>
       <c r="K91" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L91" t="n">
         <v>4</v>
@@ -5183,7 +5183,7 @@
         <v>50</v>
       </c>
       <c r="N91" t="n">
-        <v>380</v>
+        <v>370</v>
       </c>
     </row>
     <row r="92">
@@ -5215,18 +5215,18 @@
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J92" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K92" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L92" t="n">
         <v>4</v>
@@ -5235,7 +5235,7 @@
         <v>50</v>
       </c>
       <c r="N92" t="n">
-        <v>380</v>
+        <v>570</v>
       </c>
     </row>
     <row r="93">
@@ -5267,18 +5267,18 @@
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J93" t="n">
         <v>2</v>
       </c>
       <c r="K93" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L93" t="n">
         <v>4</v>
@@ -5287,7 +5287,7 @@
         <v>50</v>
       </c>
       <c r="N93" t="n">
-        <v>520</v>
+        <v>390</v>
       </c>
     </row>
     <row r="94">
@@ -5330,7 +5330,7 @@
         <v>1</v>
       </c>
       <c r="K94" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L94" t="n">
         <v>4</v>
@@ -5339,7 +5339,7 @@
         <v>50</v>
       </c>
       <c r="N94" t="n">
-        <v>560</v>
+        <v>480</v>
       </c>
     </row>
     <row r="95">
@@ -5475,18 +5475,18 @@
       </c>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J97" t="n">
         <v>2</v>
       </c>
       <c r="K97" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L97" t="n">
         <v>3</v>
@@ -5495,7 +5495,7 @@
         <v>40</v>
       </c>
       <c r="N97" t="n">
-        <v>400</v>
+        <v>560</v>
       </c>
     </row>
     <row r="98">
@@ -5527,18 +5527,18 @@
       </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J98" t="n">
         <v>2</v>
       </c>
       <c r="K98" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L98" t="n">
         <v>3</v>
@@ -5547,7 +5547,7 @@
         <v>40</v>
       </c>
       <c r="N98" t="n">
-        <v>560</v>
+        <v>400</v>
       </c>
     </row>
     <row r="99">
@@ -5579,18 +5579,18 @@
       </c>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>Ásdís</t>
+          <t>Helgi</t>
         </is>
       </c>
       <c r="J99" t="n">
         <v>3</v>
       </c>
       <c r="K99" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="L99" t="n">
         <v>3</v>
@@ -5599,7 +5599,7 @@
         <v>70</v>
       </c>
       <c r="N99" t="n">
-        <v>520</v>
+        <v>510</v>
       </c>
     </row>
     <row r="100">
@@ -5631,18 +5631,18 @@
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>Helgi</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J100" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K100" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L100" t="n">
         <v>3</v>
@@ -5651,7 +5651,7 @@
         <v>70</v>
       </c>
       <c r="N100" t="n">
-        <v>510</v>
+        <v>400</v>
       </c>
     </row>
     <row r="101">
@@ -5683,18 +5683,18 @@
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>Thelma</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J101" t="n">
+        <v>2</v>
+      </c>
+      <c r="K101" t="n">
         <v>3</v>
-      </c>
-      <c r="K101" t="n">
-        <v>9</v>
       </c>
       <c r="L101" t="n">
         <v>3</v>
@@ -5703,7 +5703,7 @@
         <v>70</v>
       </c>
       <c r="N101" t="n">
-        <v>520</v>
+        <v>490</v>
       </c>
     </row>
     <row r="102">
@@ -5735,18 +5735,18 @@
       </c>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J102" t="n">
         <v>2</v>
       </c>
       <c r="K102" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="L102" t="n">
         <v>3</v>
@@ -5755,7 +5755,7 @@
         <v>70</v>
       </c>
       <c r="N102" t="n">
-        <v>490</v>
+        <v>540</v>
       </c>
     </row>
     <row r="103">
@@ -5787,18 +5787,18 @@
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J103" t="n">
         <v>2</v>
       </c>
       <c r="K103" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="L103" t="n">
         <v>3</v>
@@ -5807,7 +5807,7 @@
         <v>70</v>
       </c>
       <c r="N103" t="n">
-        <v>490</v>
+        <v>540</v>
       </c>
     </row>
     <row r="104">
@@ -5839,18 +5839,18 @@
       </c>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J104" t="n">
         <v>2</v>
       </c>
       <c r="K104" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L104" t="n">
         <v>3</v>
@@ -5891,18 +5891,18 @@
       </c>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J105" t="n">
         <v>2</v>
       </c>
       <c r="K105" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L105" t="n">
         <v>3</v>
@@ -5911,7 +5911,7 @@
         <v>70</v>
       </c>
       <c r="N105" t="n">
-        <v>390</v>
+        <v>530</v>
       </c>
     </row>
     <row r="106">
@@ -5954,7 +5954,7 @@
         <v>1</v>
       </c>
       <c r="K106" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L106" t="n">
         <v>3</v>
@@ -5995,18 +5995,18 @@
       </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J107" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K107" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L107" t="n">
         <v>3</v>
@@ -6015,7 +6015,7 @@
         <v>70</v>
       </c>
       <c r="N107" t="n">
-        <v>510</v>
+        <v>530</v>
       </c>
     </row>
     <row r="108">
@@ -6058,7 +6058,7 @@
         <v>2</v>
       </c>
       <c r="K108" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L108" t="n">
         <v>3</v>
@@ -6151,11 +6151,11 @@
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J110" t="n">
@@ -6416,7 +6416,7 @@
         <v>2</v>
       </c>
       <c r="K115" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L115" t="n">
         <v>4</v>
@@ -6425,7 +6425,7 @@
         <v>70</v>
       </c>
       <c r="N115" t="n">
-        <v>480</v>
+        <v>470</v>
       </c>
     </row>
     <row r="116">
@@ -6468,7 +6468,7 @@
         <v>2</v>
       </c>
       <c r="K116" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="L116" t="n">
         <v>4</v>
@@ -6477,7 +6477,7 @@
         <v>70</v>
       </c>
       <c r="N116" t="n">
-        <v>470</v>
+        <v>480</v>
       </c>
     </row>
     <row r="117">
@@ -6509,18 +6509,18 @@
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J117" t="n">
         <v>2</v>
       </c>
       <c r="K117" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L117" t="n">
         <v>4</v>
@@ -6529,7 +6529,7 @@
         <v>70</v>
       </c>
       <c r="N117" t="n">
-        <v>460</v>
+        <v>470</v>
       </c>
     </row>
     <row r="118">
@@ -6561,18 +6561,18 @@
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J118" t="n">
         <v>2</v>
       </c>
       <c r="K118" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L118" t="n">
         <v>4</v>
@@ -6581,7 +6581,7 @@
         <v>70</v>
       </c>
       <c r="N118" t="n">
-        <v>480</v>
+        <v>460</v>
       </c>
     </row>
     <row r="119">
@@ -6613,18 +6613,18 @@
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J119" t="n">
         <v>2</v>
       </c>
       <c r="K119" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L119" t="n">
         <v>4</v>
@@ -6633,7 +6633,7 @@
         <v>70</v>
       </c>
       <c r="N119" t="n">
-        <v>320</v>
+        <v>470</v>
       </c>
     </row>
     <row r="120">
@@ -6665,18 +6665,18 @@
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K120" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L120" t="n">
         <v>4</v>
@@ -6685,7 +6685,7 @@
         <v>70</v>
       </c>
       <c r="N120" t="n">
-        <v>340</v>
+        <v>320</v>
       </c>
     </row>
     <row r="121">
@@ -6717,18 +6717,18 @@
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J121" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K121" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L121" t="n">
         <v>4</v>
@@ -6769,18 +6769,18 @@
       </c>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>Camilla</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J122" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K122" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="L122" t="n">
         <v>4</v>
@@ -6789,7 +6789,7 @@
         <v>70</v>
       </c>
       <c r="N122" t="n">
-        <v>500</v>
+        <v>340</v>
       </c>
     </row>
     <row r="123">
@@ -6832,7 +6832,7 @@
         <v>1</v>
       </c>
       <c r="K123" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L123" t="n">
         <v>4</v>
@@ -6884,7 +6884,7 @@
         <v>1</v>
       </c>
       <c r="K124" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L124" t="n">
         <v>4</v>
@@ -6925,18 +6925,18 @@
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="n">
+        <v>6</v>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Unnur</t>
+        </is>
+      </c>
+      <c r="J125" t="n">
+        <v>2</v>
+      </c>
+      <c r="K125" t="n">
         <v>5</v>
-      </c>
-      <c r="I125" t="inlineStr">
-        <is>
-          <t>Pétur</t>
-        </is>
-      </c>
-      <c r="J125" t="n">
-        <v>2</v>
-      </c>
-      <c r="K125" t="n">
-        <v>9</v>
       </c>
       <c r="L125" t="n">
         <v>3</v>
@@ -6977,18 +6977,18 @@
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="n">
+        <v>11</v>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Oliver</t>
+        </is>
+      </c>
+      <c r="J126" t="n">
+        <v>2</v>
+      </c>
+      <c r="K126" t="n">
         <v>9</v>
-      </c>
-      <c r="I126" t="inlineStr">
-        <is>
-          <t>Freyja</t>
-        </is>
-      </c>
-      <c r="J126" t="n">
-        <v>2</v>
-      </c>
-      <c r="K126" t="n">
-        <v>10</v>
       </c>
       <c r="L126" t="n">
         <v>3</v>
@@ -6997,7 +6997,7 @@
         <v>70</v>
       </c>
       <c r="N126" t="n">
-        <v>550</v>
+        <v>560</v>
       </c>
     </row>
     <row r="127">
@@ -7040,7 +7040,7 @@
         <v>1</v>
       </c>
       <c r="K127" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L127" t="n">
         <v>3</v>
@@ -7081,18 +7081,18 @@
       </c>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J128" t="n">
         <v>2</v>
       </c>
       <c r="K128" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L128" t="n">
         <v>3</v>
@@ -7101,7 +7101,7 @@
         <v>70</v>
       </c>
       <c r="N128" t="n">
-        <v>540</v>
+        <v>560</v>
       </c>
     </row>
     <row r="129">
@@ -7144,7 +7144,7 @@
         <v>1</v>
       </c>
       <c r="K129" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L129" t="n">
         <v>3</v>
@@ -7153,7 +7153,7 @@
         <v>70</v>
       </c>
       <c r="N129" t="n">
-        <v>510</v>
+        <v>560</v>
       </c>
     </row>
     <row r="130">
@@ -7185,18 +7185,18 @@
       </c>
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J130" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K130" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L130" t="n">
         <v>3</v>
@@ -7205,7 +7205,7 @@
         <v>70</v>
       </c>
       <c r="N130" t="n">
-        <v>530</v>
+        <v>340</v>
       </c>
     </row>
     <row r="131">
@@ -7237,18 +7237,18 @@
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J131" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L131" t="n">
         <v>3</v>
@@ -7289,18 +7289,18 @@
       </c>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J132" t="n">
         <v>2</v>
       </c>
       <c r="K132" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L132" t="n">
         <v>3</v>
@@ -7341,18 +7341,18 @@
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J133" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K133" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L133" t="n">
         <v>3</v>
@@ -7361,7 +7361,7 @@
         <v>70</v>
       </c>
       <c r="N133" t="n">
-        <v>340</v>
+        <v>550</v>
       </c>
     </row>
     <row r="134">
@@ -7393,18 +7393,18 @@
       </c>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Ólafur</t>
+          <t>Camilla</t>
         </is>
       </c>
       <c r="J134" t="n">
         <v>1</v>
       </c>
       <c r="K134" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L134" t="n">
         <v>3</v>
@@ -7413,7 +7413,7 @@
         <v>70</v>
       </c>
       <c r="N134" t="n">
-        <v>520</v>
+        <v>500</v>
       </c>
     </row>
     <row r="135">
@@ -7456,7 +7456,7 @@
         <v>2</v>
       </c>
       <c r="K135" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L135" t="n">
         <v>3</v>
@@ -7465,7 +7465,7 @@
         <v>70</v>
       </c>
       <c r="N135" t="n">
-        <v>540</v>
+        <v>550</v>
       </c>
     </row>
     <row r="136">
@@ -7497,11 +7497,11 @@
       </c>
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="n">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Bergur</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J136" t="n">
@@ -7772,21 +7772,21 @@
         <v>1</v>
       </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
+      <c r="N2" t="n">
+        <v>1</v>
+      </c>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="n">
         <v>1</v>
@@ -7809,14 +7809,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="n">
-        <v>1</v>
-      </c>
+      <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
@@ -7836,10 +7836,10 @@
       <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
         <v>1</v>
@@ -7880,7 +7880,9 @@
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
@@ -7892,9 +7894,7 @@
         <v>1</v>
       </c>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="n">
-        <v>1</v>
-      </c>
+      <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="n">
         <v>1</v>
@@ -7910,7 +7910,9 @@
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
@@ -7927,16 +7929,16 @@
       </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
+      <c r="Q6" t="n">
+        <v>1</v>
+      </c>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="n">
         <v>1</v>
       </c>
-      <c r="V6" t="n">
-        <v>1</v>
-      </c>
+      <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr"/>
     </row>
@@ -7944,37 +7946,35 @@
       <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="n">
-        <v>1</v>
-      </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="n">
-        <v>1</v>
-      </c>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="n">
         <v>1</v>
       </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
+      <c r="N7" t="n">
+        <v>1</v>
+      </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="n">
         <v>1</v>
       </c>
-      <c r="V7" t="inlineStr"/>
+      <c r="V7" t="n">
+        <v>1</v>
+      </c>
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
     </row>
@@ -7982,25 +7982,23 @@
       <c r="A8" t="n">
         <v>7</v>
       </c>
-      <c r="B8" t="inlineStr"/>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
       <c r="C8" t="inlineStr"/>
-      <c r="D8" t="n">
-        <v>1</v>
-      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
         <v>1</v>
       </c>
-      <c r="G8" t="n">
-        <v>1</v>
-      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>1</v>
       </c>
-      <c r="I8" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="n">
+        <v>1</v>
+      </c>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
@@ -8011,7 +8009,9 @@
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
+      <c r="U8" t="n">
+        <v>1</v>
+      </c>
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr"/>
@@ -8058,16 +8058,18 @@
       <c r="A10" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
       <c r="J10" t="n">
         <v>1</v>
       </c>
@@ -8077,16 +8079,16 @@
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
+      <c r="Q10" t="n">
+        <v>1</v>
+      </c>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="n">
         <v>1</v>
       </c>
-      <c r="V10" t="n">
-        <v>1</v>
-      </c>
+      <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr"/>
     </row>
@@ -8094,15 +8096,13 @@
       <c r="A11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="n">
-        <v>1</v>
-      </c>
+      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
-      <c r="D11" t="n">
-        <v>1</v>
-      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
@@ -8112,11 +8112,11 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
+      <c r="N11" t="n">
+        <v>1</v>
+      </c>
       <c r="O11" t="inlineStr"/>
-      <c r="P11" t="n">
-        <v>1</v>
-      </c>
+      <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="n">
         <v>1</v>
@@ -8140,9 +8140,7 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="n">
-        <v>1</v>
-      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
         <v>1</v>
       </c>
@@ -8162,7 +8160,9 @@
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
+      <c r="V12" t="n">
+        <v>1</v>
+      </c>
       <c r="W12" t="inlineStr"/>
       <c r="X12" t="inlineStr"/>
     </row>
@@ -8212,17 +8212,13 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="n">
-        <v>1</v>
-      </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
         <v>1</v>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" t="n">
-        <v>1</v>
-      </c>
+      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
@@ -8230,8 +8226,12 @@
         <v>1</v>
       </c>
       <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
+      <c r="R14" t="n">
+        <v>1</v>
+      </c>
+      <c r="S14" t="n">
+        <v>1</v>
+      </c>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr"/>
@@ -8248,37 +8248,39 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" t="n">
-        <v>1</v>
-      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
         <v>1</v>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
-      <c r="M15" t="n">
-        <v>1</v>
-      </c>
+      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="n">
         <v>1</v>
       </c>
       <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
+      <c r="R15" t="n">
+        <v>1</v>
+      </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
+      <c r="W15" t="n">
+        <v>1</v>
+      </c>
       <c r="X15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
         <v>15</v>
       </c>
-      <c r="B16" t="inlineStr"/>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
@@ -8298,15 +8300,13 @@
         <v>1</v>
       </c>
       <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="n">
-        <v>1</v>
-      </c>
+      <c r="R16" t="n">
+        <v>1</v>
+      </c>
+      <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
-      <c r="V16" t="n">
-        <v>1</v>
-      </c>
+      <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
       <c r="X16" t="inlineStr"/>
     </row>
@@ -8353,7 +8353,9 @@
       <c r="B18" t="n">
         <v>1</v>
       </c>
-      <c r="C18" t="inlineStr"/>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
@@ -8370,15 +8372,15 @@
         <v>1</v>
       </c>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="n">
-        <v>1</v>
-      </c>
+      <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="n">
         <v>1</v>
       </c>
-      <c r="V18" t="inlineStr"/>
+      <c r="V18" t="n">
+        <v>1</v>
+      </c>
       <c r="W18" t="inlineStr"/>
       <c r="X18" t="inlineStr"/>
     </row>
@@ -8480,13 +8482,13 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
+      <c r="R21" t="n">
+        <v>1</v>
+      </c>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
-      <c r="V21" t="n">
-        <v>1</v>
-      </c>
+      <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
       <c r="X21" t="inlineStr"/>
     </row>
@@ -8533,14 +8535,14 @@
         <v>22</v>
       </c>
       <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" t="n">
-        <v>1</v>
-      </c>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
@@ -8548,11 +8550,11 @@
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
+      <c r="P23" t="n">
+        <v>1</v>
+      </c>
       <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="n">
-        <v>1</v>
-      </c>
+      <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
@@ -8568,30 +8570,28 @@
       <c r="A24" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="n">
-        <v>1</v>
-      </c>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
+      <c r="H24" t="n">
+        <v>1</v>
+      </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="n">
         <v>1</v>
       </c>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="n">
-        <v>1</v>
-      </c>
+      <c r="M24" t="n">
+        <v>1</v>
+      </c>
+      <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr"/>
@@ -8645,26 +8645,26 @@
         <v>25</v>
       </c>
       <c r="B26" t="inlineStr"/>
-      <c r="C26" t="n">
-        <v>1</v>
-      </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" t="n">
+        <v>1</v>
+      </c>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="n">
-        <v>1</v>
-      </c>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" t="n">
-        <v>1</v>
-      </c>
+      <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
+      <c r="P26" t="n">
+        <v>1</v>
+      </c>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr"/>
@@ -8686,9 +8686,7 @@
       <c r="E27" t="n">
         <v>1</v>
       </c>
-      <c r="F27" t="n">
-        <v>1</v>
-      </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
@@ -8710,7 +8708,9 @@
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr"/>
+      <c r="V27" t="n">
+        <v>1</v>
+      </c>
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr"/>
     </row>
@@ -8720,13 +8720,13 @@
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
-      <c r="H28" t="n">
-        <v>1</v>
-      </c>
+      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="n">
         <v>1</v>
@@ -8743,10 +8743,10 @@
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr"/>
-      <c r="U28" t="n">
-        <v>1</v>
-      </c>
-      <c r="V28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="n">
+        <v>1</v>
+      </c>
       <c r="W28" t="inlineStr"/>
       <c r="X28" t="inlineStr"/>
     </row>
@@ -8754,15 +8754,15 @@
       <c r="A29" t="n">
         <v>28</v>
       </c>
-      <c r="B29" t="n">
-        <v>1</v>
-      </c>
+      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
+      <c r="H29" t="n">
+        <v>1</v>
+      </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="n">
         <v>1</v>
@@ -8797,7 +8797,9 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
+      <c r="I30" t="n">
+        <v>1</v>
+      </c>
       <c r="J30" t="n">
         <v>1</v>
       </c>
@@ -8816,9 +8818,7 @@
         <v>1</v>
       </c>
       <c r="U30" t="inlineStr"/>
-      <c r="V30" t="n">
-        <v>1</v>
-      </c>
+      <c r="V30" t="inlineStr"/>
       <c r="W30" t="inlineStr"/>
       <c r="X30" t="inlineStr"/>
     </row>
@@ -8876,7 +8876,9 @@
         <v>1</v>
       </c>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
+      <c r="L32" t="n">
+        <v>1</v>
+      </c>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
@@ -8889,9 +8891,7 @@
       <c r="V32" t="n">
         <v>1</v>
       </c>
-      <c r="W32" t="n">
-        <v>1</v>
-      </c>
+      <c r="W32" t="inlineStr"/>
       <c r="X32" t="inlineStr"/>
     </row>
     <row r="33">
@@ -8906,10 +8906,10 @@
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="n">
-        <v>1</v>
-      </c>
+      <c r="H33" t="n">
+        <v>1</v>
+      </c>
+      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
bætti við event request
bætti því við í open excek en er ekki byrjuð að gera neitt við gögnin
</commit_message>
<xml_diff>
--- a/03_26_schedule_results.xlsx
+++ b/03_26_schedule_results.xlsx
@@ -534,18 +534,18 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J2" t="n">
         <v>2</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L2" t="n">
         <v>3</v>
@@ -554,7 +554,7 @@
         <v>40</v>
       </c>
       <c r="N2" t="n">
-        <v>400</v>
+        <v>510</v>
       </c>
     </row>
     <row r="3">
@@ -586,18 +586,18 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J3" t="n">
         <v>2</v>
       </c>
       <c r="K3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
         <v>3</v>
@@ -606,7 +606,7 @@
         <v>40</v>
       </c>
       <c r="N3" t="n">
-        <v>500</v>
+        <v>420</v>
       </c>
     </row>
     <row r="4">
@@ -638,11 +638,11 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J4" t="n">
@@ -658,7 +658,7 @@
         <v>40</v>
       </c>
       <c r="N4" t="n">
-        <v>410</v>
+        <v>420</v>
       </c>
     </row>
     <row r="5">
@@ -690,15 +690,15 @@
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Nanna</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K5" t="n">
         <v>1</v>
@@ -710,7 +710,7 @@
         <v>40</v>
       </c>
       <c r="N5" t="n">
-        <v>500</v>
+        <v>540</v>
       </c>
     </row>
     <row r="6">
@@ -742,11 +742,11 @@
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J6" t="n">
@@ -762,7 +762,7 @@
         <v>80</v>
       </c>
       <c r="N6" t="n">
-        <v>460</v>
+        <v>470</v>
       </c>
     </row>
     <row r="7">
@@ -794,11 +794,11 @@
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J7" t="n">
@@ -814,7 +814,7 @@
         <v>80</v>
       </c>
       <c r="N7" t="n">
-        <v>460</v>
+        <v>470</v>
       </c>
     </row>
     <row r="8">
@@ -898,18 +898,18 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Össur</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L9" t="n">
         <v>3</v>
@@ -918,7 +918,7 @@
         <v>80</v>
       </c>
       <c r="N9" t="n">
-        <v>470</v>
+        <v>490</v>
       </c>
     </row>
     <row r="10">
@@ -950,18 +950,18 @@
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J10" t="n">
         <v>2</v>
       </c>
       <c r="K10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L10" t="n">
         <v>3</v>
@@ -1054,11 +1054,11 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Pétur</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J12" t="n">
@@ -1074,7 +1074,7 @@
         <v>40</v>
       </c>
       <c r="N12" t="n">
-        <v>400</v>
+        <v>340</v>
       </c>
     </row>
     <row r="13">
@@ -1106,11 +1106,11 @@
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J13" t="n">
@@ -1126,7 +1126,7 @@
         <v>40</v>
       </c>
       <c r="N13" t="n">
-        <v>520</v>
+        <v>530</v>
       </c>
     </row>
     <row r="14">
@@ -1366,18 +1366,18 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L18" t="n">
         <v>4</v>
@@ -1386,7 +1386,7 @@
         <v>70</v>
       </c>
       <c r="N18" t="n">
-        <v>470</v>
+        <v>450</v>
       </c>
     </row>
     <row r="19">
@@ -1418,15 +1418,15 @@
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K19" t="n">
         <v>8</v>
@@ -1438,7 +1438,7 @@
         <v>70</v>
       </c>
       <c r="N19" t="n">
-        <v>500</v>
+        <v>460</v>
       </c>
     </row>
     <row r="20">
@@ -1470,18 +1470,18 @@
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K20" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L20" t="n">
         <v>4</v>
@@ -1490,7 +1490,7 @@
         <v>70</v>
       </c>
       <c r="N20" t="n">
-        <v>510</v>
+        <v>460</v>
       </c>
     </row>
     <row r="21">
@@ -1533,7 +1533,7 @@
         <v>2</v>
       </c>
       <c r="K21" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="L21" t="n">
         <v>4</v>
@@ -1574,18 +1574,18 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K22" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L22" t="n">
         <v>4</v>
@@ -1594,7 +1594,7 @@
         <v>70</v>
       </c>
       <c r="N22" t="n">
-        <v>510</v>
+        <v>460</v>
       </c>
     </row>
     <row r="23">
@@ -1730,11 +1730,11 @@
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Camilla</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J25" t="n">
@@ -1886,15 +1886,15 @@
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -1906,7 +1906,7 @@
         <v>80</v>
       </c>
       <c r="N28" t="n">
-        <v>470</v>
+        <v>440</v>
       </c>
     </row>
     <row r="29">
@@ -1938,11 +1938,11 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Bergur</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J29" t="n">
@@ -1958,7 +1958,7 @@
         <v>90</v>
       </c>
       <c r="N29" t="n">
-        <v>470</v>
+        <v>480</v>
       </c>
     </row>
     <row r="30">
@@ -1990,18 +1990,18 @@
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
+        <v>3</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Össur</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>3</v>
+      </c>
+      <c r="K30" t="n">
         <v>7</v>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>Harpa</t>
-        </is>
-      </c>
-      <c r="J30" t="n">
-        <v>2</v>
-      </c>
-      <c r="K30" t="n">
-        <v>2</v>
       </c>
       <c r="L30" t="n">
         <v>3.5</v>
@@ -2010,7 +2010,7 @@
         <v>50</v>
       </c>
       <c r="N30" t="n">
-        <v>400</v>
+        <v>540</v>
       </c>
     </row>
     <row r="31">
@@ -2042,18 +2042,18 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J31" t="n">
         <v>2</v>
       </c>
       <c r="K31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L31" t="n">
         <v>3.5</v>
@@ -2062,7 +2062,7 @@
         <v>50</v>
       </c>
       <c r="N31" t="n">
-        <v>430</v>
+        <v>390</v>
       </c>
     </row>
     <row r="32">
@@ -2094,18 +2094,18 @@
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K32" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L32" t="n">
         <v>3.5</v>
@@ -2114,7 +2114,7 @@
         <v>50</v>
       </c>
       <c r="N32" t="n">
-        <v>550</v>
+        <v>510</v>
       </c>
     </row>
     <row r="33">
@@ -2146,18 +2146,18 @@
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J33" t="n">
         <v>2</v>
       </c>
       <c r="K33" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L33" t="n">
         <v>3.5</v>
@@ -2166,7 +2166,7 @@
         <v>50</v>
       </c>
       <c r="N33" t="n">
-        <v>550</v>
+        <v>410</v>
       </c>
     </row>
     <row r="34">
@@ -2198,18 +2198,18 @@
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K34" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="L34" t="n">
         <v>3.5</v>
@@ -2218,7 +2218,7 @@
         <v>50</v>
       </c>
       <c r="N34" t="n">
-        <v>560</v>
+        <v>540</v>
       </c>
     </row>
     <row r="35">
@@ -2250,11 +2250,11 @@
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J35" t="n">
@@ -2302,18 +2302,18 @@
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J36" t="n">
         <v>2</v>
       </c>
       <c r="K36" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L36" t="n">
         <v>3.5</v>
@@ -2322,7 +2322,7 @@
         <v>50</v>
       </c>
       <c r="N36" t="n">
-        <v>550</v>
+        <v>530</v>
       </c>
     </row>
     <row r="37">
@@ -2354,18 +2354,18 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J37" t="n">
         <v>2</v>
       </c>
       <c r="K37" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L37" t="n">
         <v>3.5</v>
@@ -2374,7 +2374,7 @@
         <v>50</v>
       </c>
       <c r="N37" t="n">
-        <v>390</v>
+        <v>530</v>
       </c>
     </row>
     <row r="38">
@@ -2406,18 +2406,18 @@
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K38" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L38" t="n">
         <v>3.5</v>
@@ -2426,7 +2426,7 @@
         <v>50</v>
       </c>
       <c r="N38" t="n">
-        <v>560</v>
+        <v>390</v>
       </c>
     </row>
     <row r="39">
@@ -2458,18 +2458,18 @@
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K39" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="L39" t="n">
         <v>3.5</v>
@@ -2478,7 +2478,7 @@
         <v>50</v>
       </c>
       <c r="N39" t="n">
-        <v>520</v>
+        <v>560</v>
       </c>
     </row>
     <row r="40">
@@ -2510,11 +2510,11 @@
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Gunnar</t>
+          <t>Camilla</t>
         </is>
       </c>
       <c r="J40" t="n">
@@ -2530,7 +2530,7 @@
         <v>50</v>
       </c>
       <c r="N40" t="n">
-        <v>560</v>
+        <v>550</v>
       </c>
     </row>
     <row r="41">
@@ -2562,18 +2562,18 @@
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J41" t="n">
         <v>2</v>
       </c>
       <c r="K41" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L41" t="n">
         <v>4</v>
@@ -2582,7 +2582,7 @@
         <v>50</v>
       </c>
       <c r="N41" t="n">
-        <v>550</v>
+        <v>560</v>
       </c>
     </row>
     <row r="42">
@@ -2614,18 +2614,18 @@
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J42" t="n">
         <v>2</v>
       </c>
       <c r="K42" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L42" t="n">
         <v>4</v>
@@ -2634,7 +2634,7 @@
         <v>50</v>
       </c>
       <c r="N42" t="n">
-        <v>330</v>
+        <v>530</v>
       </c>
     </row>
     <row r="43">
@@ -2666,18 +2666,18 @@
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J43" t="n">
         <v>2</v>
       </c>
       <c r="K43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L43" t="n">
         <v>4</v>
@@ -2718,18 +2718,18 @@
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K44" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L44" t="n">
         <v>4</v>
@@ -2770,18 +2770,18 @@
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K45" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L45" t="n">
         <v>4</v>
@@ -2822,18 +2822,18 @@
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J46" t="n">
         <v>2</v>
       </c>
       <c r="K46" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L46" t="n">
         <v>4</v>
@@ -2874,18 +2874,18 @@
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J47" t="n">
         <v>2</v>
       </c>
       <c r="K47" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L47" t="n">
         <v>4</v>
@@ -2926,18 +2926,18 @@
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J48" t="n">
         <v>2</v>
       </c>
       <c r="K48" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L48" t="n">
         <v>4</v>
@@ -2946,7 +2946,7 @@
         <v>50</v>
       </c>
       <c r="N48" t="n">
-        <v>550</v>
+        <v>330</v>
       </c>
     </row>
     <row r="49">
@@ -2978,18 +2978,18 @@
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K49" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="L49" t="n">
         <v>4</v>
@@ -2998,7 +2998,7 @@
         <v>50</v>
       </c>
       <c r="N49" t="n">
-        <v>320</v>
+        <v>560</v>
       </c>
     </row>
     <row r="50">
@@ -3030,18 +3030,18 @@
       </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Ólafur</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K50" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L50" t="n">
         <v>4</v>
@@ -3050,7 +3050,7 @@
         <v>50</v>
       </c>
       <c r="N50" t="n">
-        <v>500</v>
+        <v>320</v>
       </c>
     </row>
     <row r="51">
@@ -3082,18 +3082,18 @@
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Anna</t>
+          <t>Gunnar</t>
         </is>
       </c>
       <c r="J51" t="n">
         <v>1</v>
       </c>
       <c r="K51" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L51" t="n">
         <v>4</v>
@@ -3102,7 +3102,7 @@
         <v>50</v>
       </c>
       <c r="N51" t="n">
-        <v>500</v>
+        <v>560</v>
       </c>
     </row>
     <row r="52">
@@ -3186,18 +3186,18 @@
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Ásdís</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K53" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L53" t="n">
         <v>4</v>
@@ -3206,7 +3206,7 @@
         <v>50</v>
       </c>
       <c r="N53" t="n">
-        <v>570</v>
+        <v>360</v>
       </c>
     </row>
     <row r="54">
@@ -3238,18 +3238,18 @@
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Helgi</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J54" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K54" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L54" t="n">
         <v>4</v>
@@ -3258,7 +3258,7 @@
         <v>50</v>
       </c>
       <c r="N54" t="n">
-        <v>560</v>
+        <v>360</v>
       </c>
     </row>
     <row r="55">
@@ -3290,18 +3290,18 @@
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Thelma</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J55" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K55" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L55" t="n">
         <v>4</v>
@@ -3310,7 +3310,7 @@
         <v>50</v>
       </c>
       <c r="N55" t="n">
-        <v>570</v>
+        <v>560</v>
       </c>
     </row>
     <row r="56">
@@ -3342,18 +3342,18 @@
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Pétur</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J56" t="n">
         <v>2</v>
       </c>
       <c r="K56" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L56" t="n">
         <v>4</v>
@@ -3394,18 +3394,18 @@
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J57" t="n">
         <v>2</v>
       </c>
       <c r="K57" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L57" t="n">
         <v>4</v>
@@ -3414,7 +3414,7 @@
         <v>50</v>
       </c>
       <c r="N57" t="n">
-        <v>360</v>
+        <v>560</v>
       </c>
     </row>
     <row r="58">
@@ -3446,18 +3446,18 @@
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J58" t="n">
         <v>2</v>
       </c>
       <c r="K58" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L58" t="n">
         <v>4</v>
@@ -3466,7 +3466,7 @@
         <v>50</v>
       </c>
       <c r="N58" t="n">
-        <v>350</v>
+        <v>390</v>
       </c>
     </row>
     <row r="59">
@@ -3498,18 +3498,18 @@
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J59" t="n">
         <v>2</v>
       </c>
       <c r="K59" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L59" t="n">
         <v>4</v>
@@ -3518,7 +3518,7 @@
         <v>50</v>
       </c>
       <c r="N59" t="n">
-        <v>360</v>
+        <v>560</v>
       </c>
     </row>
     <row r="60">
@@ -3550,11 +3550,11 @@
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J60" t="n">
@@ -3665,7 +3665,7 @@
         <v>1</v>
       </c>
       <c r="K62" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L62" t="n">
         <v>4</v>
@@ -3674,7 +3674,7 @@
         <v>50</v>
       </c>
       <c r="N62" t="n">
-        <v>550</v>
+        <v>570</v>
       </c>
     </row>
     <row r="63">
@@ -3717,7 +3717,7 @@
         <v>2</v>
       </c>
       <c r="K63" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L63" t="n">
         <v>4</v>
@@ -3758,11 +3758,11 @@
       </c>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Anna</t>
         </is>
       </c>
       <c r="J64" t="n">
@@ -3778,7 +3778,7 @@
         <v>80</v>
       </c>
       <c r="N64" t="n">
-        <v>440</v>
+        <v>430</v>
       </c>
     </row>
     <row r="65">
@@ -3810,18 +3810,18 @@
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Össur</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K65" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L65" t="n">
         <v>4</v>
@@ -3830,7 +3830,7 @@
         <v>70</v>
       </c>
       <c r="N65" t="n">
-        <v>480</v>
+        <v>340</v>
       </c>
     </row>
     <row r="66">
@@ -3862,18 +3862,18 @@
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L66" t="n">
         <v>4</v>
@@ -3882,7 +3882,7 @@
         <v>70</v>
       </c>
       <c r="N66" t="n">
-        <v>340</v>
+        <v>330</v>
       </c>
     </row>
     <row r="67">
@@ -3914,18 +3914,18 @@
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K67" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L67" t="n">
         <v>4</v>
@@ -3934,7 +3934,7 @@
         <v>70</v>
       </c>
       <c r="N67" t="n">
-        <v>330</v>
+        <v>340</v>
       </c>
     </row>
     <row r="68">
@@ -3966,18 +3966,18 @@
       </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K68" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L68" t="n">
         <v>4</v>
@@ -3986,7 +3986,7 @@
         <v>70</v>
       </c>
       <c r="N68" t="n">
-        <v>340</v>
+        <v>510</v>
       </c>
     </row>
     <row r="69">
@@ -4029,7 +4029,7 @@
         <v>1</v>
       </c>
       <c r="K69" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L69" t="n">
         <v>4</v>
@@ -4070,15 +4070,15 @@
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Thelma</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K70" t="n">
         <v>1</v>
@@ -4090,7 +4090,7 @@
         <v>100</v>
       </c>
       <c r="N70" t="n">
-        <v>450</v>
+        <v>480</v>
       </c>
     </row>
     <row r="71">
@@ -4174,15 +4174,15 @@
       </c>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K72" t="n">
         <v>0</v>
@@ -4226,18 +4226,18 @@
       </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Össur</t>
+          <t>Helgi</t>
         </is>
       </c>
       <c r="J73" t="n">
         <v>3</v>
       </c>
       <c r="K73" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L73" t="n">
         <v>3.5</v>
@@ -4246,7 +4246,7 @@
         <v>50</v>
       </c>
       <c r="N73" t="n">
-        <v>530</v>
+        <v>560</v>
       </c>
     </row>
     <row r="74">
@@ -4278,11 +4278,11 @@
       </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J74" t="n">
@@ -4330,18 +4330,18 @@
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J75" t="n">
         <v>2</v>
       </c>
       <c r="K75" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L75" t="n">
         <v>3.5</v>
@@ -4350,7 +4350,7 @@
         <v>50</v>
       </c>
       <c r="N75" t="n">
-        <v>520</v>
+        <v>390</v>
       </c>
     </row>
     <row r="76">
@@ -4382,18 +4382,18 @@
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K76" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="L76" t="n">
         <v>3.5</v>
@@ -4402,7 +4402,7 @@
         <v>50</v>
       </c>
       <c r="N76" t="n">
-        <v>390</v>
+        <v>550</v>
       </c>
     </row>
     <row r="77">
@@ -4434,18 +4434,18 @@
       </c>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J77" t="n">
         <v>2</v>
       </c>
       <c r="K77" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L77" t="n">
         <v>3.5</v>
@@ -4454,7 +4454,7 @@
         <v>50</v>
       </c>
       <c r="N77" t="n">
-        <v>530</v>
+        <v>390</v>
       </c>
     </row>
     <row r="78">
@@ -4486,18 +4486,18 @@
       </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J78" t="n">
         <v>2</v>
       </c>
       <c r="K78" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L78" t="n">
         <v>3.5</v>
@@ -4506,7 +4506,7 @@
         <v>50</v>
       </c>
       <c r="N78" t="n">
-        <v>390</v>
+        <v>510</v>
       </c>
     </row>
     <row r="79">
@@ -4549,7 +4549,7 @@
         <v>2</v>
       </c>
       <c r="K79" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L79" t="n">
         <v>3.5</v>
@@ -4601,7 +4601,7 @@
         <v>2</v>
       </c>
       <c r="K80" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L80" t="n">
         <v>3.5</v>
@@ -4610,7 +4610,7 @@
         <v>50</v>
       </c>
       <c r="N80" t="n">
-        <v>520</v>
+        <v>510</v>
       </c>
     </row>
     <row r="81">
@@ -4642,18 +4642,18 @@
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Camilla</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K81" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L81" t="n">
         <v>3.5</v>
@@ -4662,7 +4662,7 @@
         <v>50</v>
       </c>
       <c r="N81" t="n">
-        <v>550</v>
+        <v>520</v>
       </c>
     </row>
     <row r="82">
@@ -4757,7 +4757,7 @@
         <v>1</v>
       </c>
       <c r="K83" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="L83" t="n">
         <v>3.5</v>
@@ -4798,11 +4798,11 @@
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Camilla</t>
         </is>
       </c>
       <c r="J84" t="n">
@@ -4850,15 +4850,15 @@
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Ásdís</t>
         </is>
       </c>
       <c r="J85" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K85" t="n">
         <v>9</v>
@@ -4902,18 +4902,18 @@
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Thelma</t>
         </is>
       </c>
       <c r="J86" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K86" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L86" t="n">
         <v>4</v>
@@ -4922,7 +4922,7 @@
         <v>50</v>
       </c>
       <c r="N86" t="n">
-        <v>520</v>
+        <v>570</v>
       </c>
     </row>
     <row r="87">
@@ -4954,18 +4954,18 @@
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J87" t="n">
         <v>2</v>
       </c>
       <c r="K87" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L87" t="n">
         <v>4</v>
@@ -4974,7 +4974,7 @@
         <v>50</v>
       </c>
       <c r="N87" t="n">
-        <v>380</v>
+        <v>390</v>
       </c>
     </row>
     <row r="88">
@@ -5006,18 +5006,18 @@
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J88" t="n">
         <v>2</v>
       </c>
       <c r="K88" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L88" t="n">
         <v>4</v>
@@ -5058,18 +5058,18 @@
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J89" t="n">
         <v>2</v>
       </c>
       <c r="K89" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L89" t="n">
         <v>4</v>
@@ -5110,18 +5110,18 @@
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J90" t="n">
         <v>2</v>
       </c>
       <c r="K90" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L90" t="n">
         <v>4</v>
@@ -5162,18 +5162,18 @@
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J91" t="n">
         <v>2</v>
       </c>
       <c r="K91" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L91" t="n">
         <v>4</v>
@@ -5182,7 +5182,7 @@
         <v>50</v>
       </c>
       <c r="N91" t="n">
-        <v>370</v>
+        <v>380</v>
       </c>
     </row>
     <row r="92">
@@ -5214,18 +5214,18 @@
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J92" t="n">
         <v>2</v>
       </c>
       <c r="K92" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L92" t="n">
         <v>4</v>
@@ -5234,7 +5234,7 @@
         <v>50</v>
       </c>
       <c r="N92" t="n">
-        <v>570</v>
+        <v>380</v>
       </c>
     </row>
     <row r="93">
@@ -5266,18 +5266,18 @@
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J93" t="n">
         <v>2</v>
       </c>
       <c r="K93" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L93" t="n">
         <v>4</v>
@@ -5286,7 +5286,7 @@
         <v>50</v>
       </c>
       <c r="N93" t="n">
-        <v>390</v>
+        <v>520</v>
       </c>
     </row>
     <row r="94">
@@ -5329,7 +5329,7 @@
         <v>1</v>
       </c>
       <c r="K94" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L94" t="n">
         <v>4</v>
@@ -5338,7 +5338,7 @@
         <v>50</v>
       </c>
       <c r="N94" t="n">
-        <v>490</v>
+        <v>560</v>
       </c>
     </row>
     <row r="95">
@@ -5474,11 +5474,11 @@
       </c>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J97" t="n">
@@ -5494,7 +5494,7 @@
         <v>40</v>
       </c>
       <c r="N97" t="n">
-        <v>380</v>
+        <v>400</v>
       </c>
     </row>
     <row r="98">
@@ -5526,11 +5526,11 @@
       </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J98" t="n">
@@ -5546,7 +5546,7 @@
         <v>40</v>
       </c>
       <c r="N98" t="n">
-        <v>500</v>
+        <v>560</v>
       </c>
     </row>
     <row r="99">
@@ -5589,7 +5589,7 @@
         <v>3</v>
       </c>
       <c r="K99" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="L99" t="n">
         <v>3</v>
@@ -5641,7 +5641,7 @@
         <v>3</v>
       </c>
       <c r="K100" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L100" t="n">
         <v>3</v>
@@ -5682,18 +5682,18 @@
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>Pétur</t>
+          <t>Thelma</t>
         </is>
       </c>
       <c r="J101" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K101" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L101" t="n">
         <v>3</v>
@@ -5702,7 +5702,7 @@
         <v>70</v>
       </c>
       <c r="N101" t="n">
-        <v>540</v>
+        <v>520</v>
       </c>
     </row>
     <row r="102">
@@ -5745,7 +5745,7 @@
         <v>2</v>
       </c>
       <c r="K102" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L102" t="n">
         <v>3</v>
@@ -5754,7 +5754,7 @@
         <v>70</v>
       </c>
       <c r="N102" t="n">
-        <v>400</v>
+        <v>490</v>
       </c>
     </row>
     <row r="103">
@@ -5797,7 +5797,7 @@
         <v>2</v>
       </c>
       <c r="K103" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="L103" t="n">
         <v>3</v>
@@ -5806,7 +5806,7 @@
         <v>70</v>
       </c>
       <c r="N103" t="n">
-        <v>540</v>
+        <v>490</v>
       </c>
     </row>
     <row r="104">
@@ -5838,11 +5838,11 @@
       </c>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J104" t="n">
@@ -5858,7 +5858,7 @@
         <v>70</v>
       </c>
       <c r="N104" t="n">
-        <v>540</v>
+        <v>530</v>
       </c>
     </row>
     <row r="105">
@@ -5890,18 +5890,18 @@
       </c>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J105" t="n">
         <v>2</v>
       </c>
       <c r="K105" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L105" t="n">
         <v>3</v>
@@ -5910,7 +5910,7 @@
         <v>70</v>
       </c>
       <c r="N105" t="n">
-        <v>530</v>
+        <v>390</v>
       </c>
     </row>
     <row r="106">
@@ -5942,18 +5942,18 @@
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J106" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K106" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L106" t="n">
         <v>3</v>
@@ -5962,7 +5962,7 @@
         <v>70</v>
       </c>
       <c r="N106" t="n">
-        <v>530</v>
+        <v>500</v>
       </c>
     </row>
     <row r="107">
@@ -5994,18 +5994,18 @@
       </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J107" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K107" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L107" t="n">
         <v>3</v>
@@ -6014,7 +6014,7 @@
         <v>70</v>
       </c>
       <c r="N107" t="n">
-        <v>480</v>
+        <v>510</v>
       </c>
     </row>
     <row r="108">
@@ -6057,7 +6057,7 @@
         <v>2</v>
       </c>
       <c r="K108" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L108" t="n">
         <v>3</v>
@@ -6150,11 +6150,11 @@
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J110" t="n">
@@ -6213,7 +6213,7 @@
         <v>3</v>
       </c>
       <c r="K111" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L111" t="n">
         <v>4</v>
@@ -6254,18 +6254,18 @@
       </c>
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Ólafur</t>
+          <t>Thelma</t>
         </is>
       </c>
       <c r="J112" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K112" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L112" t="n">
         <v>4</v>
@@ -6306,11 +6306,11 @@
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>Anna</t>
+          <t>Ólafur</t>
         </is>
       </c>
       <c r="J113" t="n">
@@ -6358,18 +6358,18 @@
       </c>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>Thelma</t>
+          <t>Össur</t>
         </is>
       </c>
       <c r="J114" t="n">
         <v>3</v>
       </c>
       <c r="K114" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L114" t="n">
         <v>4</v>
@@ -6378,7 +6378,7 @@
         <v>70</v>
       </c>
       <c r="N114" t="n">
-        <v>520</v>
+        <v>410</v>
       </c>
     </row>
     <row r="115">
@@ -6421,7 +6421,7 @@
         <v>2</v>
       </c>
       <c r="K115" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L115" t="n">
         <v>4</v>
@@ -6430,7 +6430,7 @@
         <v>70</v>
       </c>
       <c r="N115" t="n">
-        <v>470</v>
+        <v>480</v>
       </c>
     </row>
     <row r="116">
@@ -6462,18 +6462,18 @@
       </c>
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J116" t="n">
         <v>2</v>
       </c>
       <c r="K116" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L116" t="n">
         <v>4</v>
@@ -6482,7 +6482,7 @@
         <v>70</v>
       </c>
       <c r="N116" t="n">
-        <v>540</v>
+        <v>470</v>
       </c>
     </row>
     <row r="117">
@@ -6514,11 +6514,11 @@
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J117" t="n">
@@ -6534,7 +6534,7 @@
         <v>70</v>
       </c>
       <c r="N117" t="n">
-        <v>470</v>
+        <v>460</v>
       </c>
     </row>
     <row r="118">
@@ -6566,18 +6566,18 @@
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J118" t="n">
         <v>2</v>
       </c>
       <c r="K118" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L118" t="n">
         <v>4</v>
@@ -6586,7 +6586,7 @@
         <v>70</v>
       </c>
       <c r="N118" t="n">
-        <v>320</v>
+        <v>480</v>
       </c>
     </row>
     <row r="119">
@@ -6618,18 +6618,18 @@
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J119" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K119" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L119" t="n">
         <v>4</v>
@@ -6638,7 +6638,7 @@
         <v>70</v>
       </c>
       <c r="N119" t="n">
-        <v>340</v>
+        <v>320</v>
       </c>
     </row>
     <row r="120">
@@ -6670,18 +6670,18 @@
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J120" t="n">
         <v>1</v>
       </c>
       <c r="K120" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L120" t="n">
         <v>4</v>
@@ -6690,7 +6690,7 @@
         <v>70</v>
       </c>
       <c r="N120" t="n">
-        <v>550</v>
+        <v>340</v>
       </c>
     </row>
     <row r="121">
@@ -6774,18 +6774,18 @@
       </c>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Camilla</t>
         </is>
       </c>
       <c r="J122" t="n">
         <v>1</v>
       </c>
       <c r="K122" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L122" t="n">
         <v>4</v>
@@ -6794,7 +6794,7 @@
         <v>70</v>
       </c>
       <c r="N122" t="n">
-        <v>560</v>
+        <v>500</v>
       </c>
     </row>
     <row r="123">
@@ -6837,7 +6837,7 @@
         <v>1</v>
       </c>
       <c r="K123" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="L123" t="n">
         <v>4</v>
@@ -6846,7 +6846,7 @@
         <v>70</v>
       </c>
       <c r="N123" t="n">
-        <v>570</v>
+        <v>500</v>
       </c>
     </row>
     <row r="124">
@@ -6878,18 +6878,18 @@
       </c>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Bergur</t>
+          <t>Anna</t>
         </is>
       </c>
       <c r="J124" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K124" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="L124" t="n">
         <v>4</v>
@@ -6898,7 +6898,7 @@
         <v>70</v>
       </c>
       <c r="N124" t="n">
-        <v>540</v>
+        <v>500</v>
       </c>
     </row>
     <row r="125">
@@ -6910,12 +6910,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>13:00:00</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -6930,27 +6930,27 @@
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Össur</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J125" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K125" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="L125" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M125" t="n">
         <v>70</v>
       </c>
       <c r="N125" t="n">
-        <v>410</v>
+        <v>550</v>
       </c>
     </row>
     <row r="126">
@@ -6962,12 +6962,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>13:00:00</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -6982,27 +6982,27 @@
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J126" t="n">
         <v>2</v>
       </c>
       <c r="K126" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L126" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M126" t="n">
         <v>70</v>
       </c>
       <c r="N126" t="n">
-        <v>480</v>
+        <v>550</v>
       </c>
     </row>
     <row r="127">
@@ -7014,12 +7014,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>13:00:00</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -7034,27 +7034,27 @@
       </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J127" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K127" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L127" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M127" t="n">
         <v>70</v>
       </c>
       <c r="N127" t="n">
-        <v>470</v>
+        <v>520</v>
       </c>
     </row>
     <row r="128">
@@ -7066,12 +7066,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>13:00:00</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -7086,27 +7086,27 @@
       </c>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J128" t="n">
         <v>2</v>
       </c>
       <c r="K128" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="L128" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M128" t="n">
         <v>70</v>
       </c>
       <c r="N128" t="n">
-        <v>500</v>
+        <v>540</v>
       </c>
     </row>
     <row r="129">
@@ -7118,12 +7118,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>13:00:00</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -7138,27 +7138,27 @@
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J129" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K129" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L129" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M129" t="n">
         <v>70</v>
       </c>
       <c r="N129" t="n">
-        <v>460</v>
+        <v>510</v>
       </c>
     </row>
     <row r="130">
@@ -7170,12 +7170,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>13:00:00</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -7201,16 +7201,16 @@
         <v>2</v>
       </c>
       <c r="K130" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L130" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M130" t="n">
         <v>70</v>
       </c>
       <c r="N130" t="n">
-        <v>460</v>
+        <v>530</v>
       </c>
     </row>
     <row r="131">
@@ -7222,12 +7222,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>13:00:00</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -7256,7 +7256,7 @@
         <v>0</v>
       </c>
       <c r="L131" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M131" t="n">
         <v>70</v>
@@ -7274,12 +7274,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>13:00:00</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -7308,7 +7308,7 @@
         <v>1</v>
       </c>
       <c r="L132" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M132" t="n">
         <v>70</v>
@@ -7326,12 +7326,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>13:00:00</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -7360,7 +7360,7 @@
         <v>2</v>
       </c>
       <c r="L133" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M133" t="n">
         <v>70</v>
@@ -7378,12 +7378,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>13:00:00</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -7398,27 +7398,27 @@
       </c>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Camilla</t>
+          <t>Ólafur</t>
         </is>
       </c>
       <c r="J134" t="n">
         <v>1</v>
       </c>
       <c r="K134" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="L134" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M134" t="n">
         <v>70</v>
       </c>
       <c r="N134" t="n">
-        <v>500</v>
+        <v>520</v>
       </c>
     </row>
     <row r="135">
@@ -7430,12 +7430,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>13:00:00</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -7450,27 +7450,27 @@
       </c>
       <c r="G135" t="inlineStr"/>
       <c r="H135" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Nanna</t>
+          <t>Bergur</t>
         </is>
       </c>
       <c r="J135" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K135" t="n">
         <v>8</v>
       </c>
       <c r="L135" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M135" t="n">
         <v>70</v>
       </c>
       <c r="N135" t="n">
-        <v>500</v>
+        <v>540</v>
       </c>
     </row>
     <row r="136">
@@ -7502,11 +7502,11 @@
       </c>
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="n">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Bergur</t>
         </is>
       </c>
       <c r="J136" t="n">
@@ -7779,15 +7779,15 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+      <c r="P2" t="n">
+        <v>1</v>
+      </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="n">
         <v>1</v>
@@ -7815,13 +7815,13 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" t="n">
-        <v>1</v>
-      </c>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+      <c r="N3" t="n">
+        <v>1</v>
+      </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
@@ -7842,34 +7842,34 @@
         <v>3</v>
       </c>
       <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="n">
-        <v>1</v>
-      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="n">
-        <v>1</v>
-      </c>
+      <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="n">
-        <v>1</v>
-      </c>
+      <c r="U4" t="n">
+        <v>1</v>
+      </c>
+      <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
     </row>
@@ -7887,24 +7887,24 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" t="n">
-        <v>1</v>
-      </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="n">
-        <v>1</v>
-      </c>
+      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
+      <c r="P5" t="n">
+        <v>1</v>
+      </c>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
+      <c r="R5" t="n">
+        <v>1</v>
+      </c>
       <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="n">
-        <v>1</v>
-      </c>
+      <c r="T5" t="n">
+        <v>1</v>
+      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr"/>
@@ -7915,9 +7915,7 @@
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
-      <c r="D6" t="n">
-        <v>1</v>
-      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
@@ -7929,19 +7927,21 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
+      <c r="N6" t="n">
+        <v>1</v>
+      </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="n">
-        <v>1</v>
-      </c>
+      <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="n">
         <v>1</v>
       </c>
-      <c r="V6" t="inlineStr"/>
+      <c r="V6" t="n">
+        <v>1</v>
+      </c>
       <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr"/>
     </row>
@@ -7949,37 +7949,37 @@
       <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
       <c r="C7" t="inlineStr"/>
-      <c r="D7" t="n">
-        <v>1</v>
-      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
       <c r="J7" t="n">
         <v>1</v>
       </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="n">
-        <v>1</v>
-      </c>
+      <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
-      <c r="P7" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="n">
+        <v>1</v>
+      </c>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="n">
-        <v>1</v>
-      </c>
+      <c r="U7" t="n">
+        <v>1</v>
+      </c>
+      <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
     </row>
@@ -7989,19 +7989,23 @@
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
         <v>1</v>
       </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
       <c r="H8" t="n">
         <v>1</v>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="n">
-        <v>1</v>
-      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
@@ -8012,12 +8016,8 @@
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
-      <c r="U8" t="n">
-        <v>1</v>
-      </c>
-      <c r="V8" t="n">
-        <v>1</v>
-      </c>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr"/>
     </row>
@@ -8036,26 +8036,26 @@
       <c r="H9" t="n">
         <v>1</v>
       </c>
-      <c r="I9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="n">
+        <v>1</v>
+      </c>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="n">
-        <v>1</v>
-      </c>
+      <c r="P9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="n">
-        <v>1</v>
-      </c>
+      <c r="U9" t="n">
+        <v>1</v>
+      </c>
+      <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr"/>
     </row>
@@ -8063,15 +8063,15 @@
       <c r="A10" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="n">
-        <v>1</v>
-      </c>
+      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="n">
         <v>1</v>
@@ -8081,9 +8081,7 @@
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
-      <c r="P10" t="n">
-        <v>1</v>
-      </c>
+      <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
@@ -8091,7 +8089,9 @@
       <c r="U10" t="n">
         <v>1</v>
       </c>
-      <c r="V10" t="inlineStr"/>
+      <c r="V10" t="n">
+        <v>1</v>
+      </c>
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr"/>
     </row>
@@ -8099,12 +8099,14 @@
       <c r="A11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="inlineStr"/>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
       <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="n">
-        <v>1</v>
-      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
@@ -8115,11 +8117,11 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="n">
-        <v>1</v>
-      </c>
+      <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
+      <c r="P11" t="n">
+        <v>1</v>
+      </c>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="n">
         <v>1</v>
@@ -8135,13 +8137,17 @@
       <c r="A12" t="n">
         <v>11</v>
       </c>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
       <c r="I12" t="n">
         <v>1</v>
       </c>
@@ -8158,9 +8164,7 @@
       <c r="R12" t="n">
         <v>1</v>
       </c>
-      <c r="S12" t="n">
-        <v>1</v>
-      </c>
+      <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr"/>
@@ -8190,16 +8194,16 @@
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
-      <c r="O13" t="n">
-        <v>1</v>
-      </c>
+      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr"/>
+      <c r="V13" t="n">
+        <v>1</v>
+      </c>
       <c r="W13" t="inlineStr"/>
       <c r="X13" t="inlineStr"/>
     </row>
@@ -8213,13 +8217,17 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>1</v>
+      </c>
       <c r="I14" t="n">
         <v>1</v>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
+      <c r="L14" t="n">
+        <v>1</v>
+      </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
@@ -8227,47 +8235,43 @@
         <v>1</v>
       </c>
       <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="n">
-        <v>1</v>
-      </c>
+      <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr"/>
-      <c r="W14" t="n">
-        <v>1</v>
-      </c>
+      <c r="W14" t="inlineStr"/>
       <c r="X14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
         <v>14</v>
       </c>
-      <c r="B15" t="n">
-        <v>1</v>
-      </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>1</v>
+      </c>
       <c r="I15" t="n">
         <v>1</v>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
+      <c r="M15" t="n">
+        <v>1</v>
+      </c>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="n">
         <v>1</v>
       </c>
       <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="n">
-        <v>1</v>
-      </c>
+      <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
@@ -8279,9 +8283,7 @@
       <c r="A16" t="n">
         <v>15</v>
       </c>
-      <c r="B16" t="n">
-        <v>1</v>
-      </c>
+      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
@@ -8301,13 +8303,15 @@
         <v>1</v>
       </c>
       <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="n">
-        <v>1</v>
-      </c>
-      <c r="S16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="n">
+        <v>1</v>
+      </c>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
+      <c r="V16" t="n">
+        <v>1</v>
+      </c>
       <c r="W16" t="inlineStr"/>
       <c r="X16" t="inlineStr"/>
     </row>
@@ -8315,17 +8319,15 @@
       <c r="A17" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="n">
-        <v>1</v>
-      </c>
+      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" t="n">
-        <v>1</v>
-      </c>
+      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="n">
@@ -8339,13 +8341,13 @@
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
+      <c r="R17" t="n">
+        <v>1</v>
+      </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
-      <c r="V17" t="n">
-        <v>1</v>
-      </c>
+      <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr"/>
       <c r="X17" t="inlineStr"/>
     </row>
@@ -8353,10 +8355,10 @@
       <c r="A18" t="n">
         <v>17</v>
       </c>
-      <c r="B18" t="n">
-        <v>1</v>
-      </c>
-      <c r="C18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
@@ -8367,9 +8369,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" t="n">
-        <v>1</v>
-      </c>
+      <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="n">
         <v>1</v>
@@ -8394,15 +8394,13 @@
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="n">
-        <v>1</v>
-      </c>
+      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" t="n">
-        <v>1</v>
-      </c>
-      <c r="I19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="n">
+        <v>1</v>
+      </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="n">
@@ -8419,7 +8417,9 @@
       <c r="U19" t="n">
         <v>1</v>
       </c>
-      <c r="V19" t="inlineStr"/>
+      <c r="V19" t="n">
+        <v>1</v>
+      </c>
       <c r="W19" t="inlineStr"/>
       <c r="X19" t="inlineStr"/>
     </row>
@@ -8430,31 +8430,31 @@
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" t="n">
-        <v>1</v>
-      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="n">
         <v>1</v>
       </c>
       <c r="L20" t="inlineStr"/>
-      <c r="M20" t="n">
-        <v>1</v>
-      </c>
-      <c r="N20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="n">
+        <v>1</v>
+      </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
+      <c r="R20" t="n">
+        <v>1</v>
+      </c>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr"/>
-      <c r="U20" t="n">
-        <v>1</v>
-      </c>
+      <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr"/>
       <c r="X20" t="inlineStr"/>
@@ -8463,17 +8463,15 @@
       <c r="A21" t="n">
         <v>20</v>
       </c>
-      <c r="B21" t="n">
-        <v>1</v>
-      </c>
+      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" t="n">
-        <v>1</v>
-      </c>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="n">
@@ -8512,19 +8510,19 @@
       <c r="H22" t="n">
         <v>1</v>
       </c>
-      <c r="I22" t="n">
-        <v>1</v>
-      </c>
-      <c r="J22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="n">
+        <v>1</v>
+      </c>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
+      <c r="N22" t="n">
+        <v>1</v>
+      </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr"/>
@@ -8542,9 +8540,7 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="n">
-        <v>1</v>
-      </c>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
@@ -8559,7 +8555,9 @@
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
+      <c r="R23" t="n">
+        <v>1</v>
+      </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
@@ -8575,10 +8573,10 @@
       <c r="A24" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="n">
-        <v>1</v>
-      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
@@ -8595,10 +8593,10 @@
         <v>1</v>
       </c>
       <c r="O24" t="inlineStr"/>
-      <c r="P24" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="n">
+        <v>1</v>
+      </c>
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr"/>
@@ -8616,16 +8614,18 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="n">
-        <v>1</v>
-      </c>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="n">
         <v>1</v>
       </c>
-      <c r="J25" t="inlineStr"/>
+      <c r="J25" t="n">
+        <v>1</v>
+      </c>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
@@ -8649,27 +8649,27 @@
       <c r="A26" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="n">
-        <v>1</v>
-      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" t="n">
-        <v>1</v>
-      </c>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
+      <c r="J26" t="n">
+        <v>1</v>
+      </c>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
+      <c r="N26" t="n">
+        <v>1</v>
+      </c>
       <c r="O26" t="inlineStr"/>
-      <c r="P26" t="n">
-        <v>1</v>
-      </c>
+      <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr"/>
@@ -8691,7 +8691,9 @@
       <c r="E27" t="n">
         <v>1</v>
       </c>
-      <c r="F27" t="inlineStr"/>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
@@ -8712,9 +8714,7 @@
       </c>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr"/>
-      <c r="U27" t="n">
-        <v>1</v>
-      </c>
+      <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr"/>
@@ -8726,12 +8726,12 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="n">
-        <v>1</v>
-      </c>
+      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
+      <c r="H28" t="n">
+        <v>1</v>
+      </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="n">
         <v>1</v>
@@ -8739,19 +8739,19 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" t="n">
-        <v>1</v>
-      </c>
-      <c r="O28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="n">
+        <v>1</v>
+      </c>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr"/>
-      <c r="U28" t="inlineStr"/>
-      <c r="V28" t="n">
-        <v>1</v>
-      </c>
+      <c r="U28" t="n">
+        <v>1</v>
+      </c>
+      <c r="V28" t="inlineStr"/>
       <c r="W28" t="inlineStr"/>
       <c r="X28" t="inlineStr"/>
     </row>
@@ -8759,7 +8759,9 @@
       <c r="A29" t="n">
         <v>28</v>
       </c>
-      <c r="B29" t="inlineStr"/>
+      <c r="B29" t="n">
+        <v>1</v>
+      </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr"/>
@@ -8785,9 +8787,7 @@
       <c r="U29" t="n">
         <v>1</v>
       </c>
-      <c r="V29" t="n">
-        <v>1</v>
-      </c>
+      <c r="V29" t="inlineStr"/>
       <c r="W29" t="inlineStr"/>
       <c r="X29" t="inlineStr"/>
     </row>
@@ -8802,9 +8802,7 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
-      <c r="I30" t="n">
-        <v>1</v>
-      </c>
+      <c r="I30" t="inlineStr"/>
       <c r="J30" t="n">
         <v>1</v>
       </c>
@@ -8823,7 +8821,9 @@
         <v>1</v>
       </c>
       <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr"/>
+      <c r="V30" t="n">
+        <v>1</v>
+      </c>
       <c r="W30" t="inlineStr"/>
       <c r="X30" t="inlineStr"/>
     </row>
@@ -8840,11 +8840,11 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
-      <c r="I31" t="n">
-        <v>1</v>
-      </c>
+      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
+      <c r="K31" t="n">
+        <v>1</v>
+      </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="n">
@@ -8855,10 +8855,10 @@
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr"/>
-      <c r="T31" t="n">
-        <v>1</v>
-      </c>
-      <c r="U31" t="inlineStr"/>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="n">
+        <v>1</v>
+      </c>
       <c r="V31" t="inlineStr"/>
       <c r="W31" t="inlineStr"/>
       <c r="X31" t="inlineStr"/>
@@ -8874,9 +8874,7 @@
         <v>1</v>
       </c>
       <c r="F32" t="inlineStr"/>
-      <c r="G32" t="n">
-        <v>1</v>
-      </c>
+      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="n">
@@ -8892,11 +8890,13 @@
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr"/>
-      <c r="U32" t="n">
-        <v>1</v>
-      </c>
-      <c r="V32" t="inlineStr"/>
-      <c r="W32" t="inlineStr"/>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="n">
+        <v>1</v>
+      </c>
+      <c r="W32" t="n">
+        <v>1</v>
+      </c>
       <c r="X32" t="inlineStr"/>
     </row>
     <row r="33">
@@ -8911,10 +8911,10 @@
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="n">
-        <v>1</v>
-      </c>
-      <c r="I33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="n">
+        <v>1</v>
+      </c>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
breytti open excel til að laga days off
ætti að vera rétt núna
</commit_message>
<xml_diff>
--- a/03_26_schedule_results.xlsx
+++ b/03_26_schedule_results.xlsx
@@ -534,11 +534,11 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -554,7 +554,7 @@
         <v>40</v>
       </c>
       <c r="N2" t="n">
-        <v>390</v>
+        <v>370</v>
       </c>
     </row>
     <row r="3">
@@ -586,15 +586,15 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Nanna</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K3" t="n">
         <v>1</v>
@@ -606,7 +606,7 @@
         <v>40</v>
       </c>
       <c r="N3" t="n">
-        <v>520</v>
+        <v>540</v>
       </c>
     </row>
     <row r="4">
@@ -742,11 +742,11 @@
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J6" t="n">
@@ -846,11 +846,11 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J8" t="n">
@@ -898,15 +898,15 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Anna</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" t="n">
         <v>2</v>
@@ -918,7 +918,7 @@
         <v>80</v>
       </c>
       <c r="N9" t="n">
-        <v>510</v>
+        <v>470</v>
       </c>
     </row>
     <row r="10">
@@ -1002,18 +1002,18 @@
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Ásdís</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
         <v>3</v>
@@ -1022,7 +1022,7 @@
         <v>40</v>
       </c>
       <c r="N11" t="n">
-        <v>390</v>
+        <v>330</v>
       </c>
     </row>
     <row r="12">
@@ -1054,18 +1054,18 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J12" t="n">
         <v>2</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L12" t="n">
         <v>3</v>
@@ -1074,7 +1074,7 @@
         <v>40</v>
       </c>
       <c r="N12" t="n">
-        <v>370</v>
+        <v>540</v>
       </c>
     </row>
     <row r="13">
@@ -1210,18 +1210,18 @@
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J15" t="n">
         <v>2</v>
       </c>
       <c r="K15" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L15" t="n">
         <v>4</v>
@@ -1230,7 +1230,7 @@
         <v>70</v>
       </c>
       <c r="N15" t="n">
-        <v>340</v>
+        <v>470</v>
       </c>
     </row>
     <row r="16">
@@ -1262,18 +1262,18 @@
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J16" t="n">
         <v>2</v>
       </c>
       <c r="K16" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L16" t="n">
         <v>4</v>
@@ -1282,7 +1282,7 @@
         <v>70</v>
       </c>
       <c r="N16" t="n">
-        <v>460</v>
+        <v>340</v>
       </c>
     </row>
     <row r="17">
@@ -1314,18 +1314,18 @@
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K17" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L17" t="n">
         <v>4</v>
@@ -1334,7 +1334,7 @@
         <v>70</v>
       </c>
       <c r="N17" t="n">
-        <v>450</v>
+        <v>340</v>
       </c>
     </row>
     <row r="18">
@@ -1366,18 +1366,18 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L18" t="n">
         <v>4</v>
@@ -1386,7 +1386,7 @@
         <v>70</v>
       </c>
       <c r="N18" t="n">
-        <v>460</v>
+        <v>510</v>
       </c>
     </row>
     <row r="19">
@@ -1418,18 +1418,18 @@
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K19" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L19" t="n">
         <v>4</v>
@@ -1438,7 +1438,7 @@
         <v>70</v>
       </c>
       <c r="N19" t="n">
-        <v>510</v>
+        <v>460</v>
       </c>
     </row>
     <row r="20">
@@ -1470,18 +1470,18 @@
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="L20" t="n">
         <v>4</v>
@@ -1490,7 +1490,7 @@
         <v>70</v>
       </c>
       <c r="N20" t="n">
-        <v>460</v>
+        <v>510</v>
       </c>
     </row>
     <row r="21">
@@ -1522,18 +1522,18 @@
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L21" t="n">
         <v>4</v>
@@ -1542,7 +1542,7 @@
         <v>70</v>
       </c>
       <c r="N21" t="n">
-        <v>290</v>
+        <v>460</v>
       </c>
     </row>
     <row r="22">
@@ -1574,18 +1574,18 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Nanna</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J22" t="n">
         <v>1</v>
       </c>
       <c r="K22" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L22" t="n">
         <v>4</v>
@@ -1594,7 +1594,7 @@
         <v>70</v>
       </c>
       <c r="N22" t="n">
-        <v>500</v>
+        <v>290</v>
       </c>
     </row>
     <row r="23">
@@ -1626,18 +1626,18 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Bergur</t>
+          <t>Nanna</t>
         </is>
       </c>
       <c r="J23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="L23" t="n">
         <v>4</v>
@@ -1646,7 +1646,7 @@
         <v>70</v>
       </c>
       <c r="N23" t="n">
-        <v>330</v>
+        <v>500</v>
       </c>
     </row>
     <row r="24">
@@ -1782,11 +1782,11 @@
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Bergur</t>
         </is>
       </c>
       <c r="J26" t="n">
@@ -1802,7 +1802,7 @@
         <v>80</v>
       </c>
       <c r="N26" t="n">
-        <v>330</v>
+        <v>340</v>
       </c>
     </row>
     <row r="27">
@@ -1834,15 +1834,15 @@
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -1854,7 +1854,7 @@
         <v>80</v>
       </c>
       <c r="N27" t="n">
-        <v>470</v>
+        <v>440</v>
       </c>
     </row>
     <row r="28">
@@ -1886,11 +1886,11 @@
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Bergur</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J28" t="n">
@@ -1906,7 +1906,7 @@
         <v>90</v>
       </c>
       <c r="N28" t="n">
-        <v>470</v>
+        <v>480</v>
       </c>
     </row>
     <row r="29">
@@ -1938,18 +1938,18 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Ásdís</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K29" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L29" t="n">
         <v>3.5</v>
@@ -1958,7 +1958,7 @@
         <v>50</v>
       </c>
       <c r="N29" t="n">
-        <v>510</v>
+        <v>400</v>
       </c>
     </row>
     <row r="30">
@@ -1990,18 +1990,18 @@
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J30" t="n">
         <v>2</v>
       </c>
       <c r="K30" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L30" t="n">
         <v>3.5</v>
@@ -2010,7 +2010,7 @@
         <v>50</v>
       </c>
       <c r="N30" t="n">
-        <v>410</v>
+        <v>490</v>
       </c>
     </row>
     <row r="31">
@@ -2042,18 +2042,18 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K31" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L31" t="n">
         <v>3.5</v>
@@ -2062,7 +2062,7 @@
         <v>50</v>
       </c>
       <c r="N31" t="n">
-        <v>550</v>
+        <v>410</v>
       </c>
     </row>
     <row r="32">
@@ -2094,18 +2094,18 @@
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J32" t="n">
         <v>2</v>
       </c>
       <c r="K32" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L32" t="n">
         <v>3.5</v>
@@ -2114,7 +2114,7 @@
         <v>50</v>
       </c>
       <c r="N32" t="n">
-        <v>420</v>
+        <v>530</v>
       </c>
     </row>
     <row r="33">
@@ -2146,18 +2146,18 @@
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K33" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L33" t="n">
         <v>3.5</v>
@@ -2166,7 +2166,7 @@
         <v>50</v>
       </c>
       <c r="N33" t="n">
-        <v>560</v>
+        <v>530</v>
       </c>
     </row>
     <row r="34">
@@ -2198,18 +2198,18 @@
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K34" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="L34" t="n">
         <v>3.5</v>
@@ -2218,7 +2218,7 @@
         <v>50</v>
       </c>
       <c r="N34" t="n">
-        <v>390</v>
+        <v>560</v>
       </c>
     </row>
     <row r="35">
@@ -2250,18 +2250,18 @@
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J35" t="n">
         <v>1</v>
       </c>
       <c r="K35" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L35" t="n">
         <v>3.5</v>
@@ -2270,7 +2270,7 @@
         <v>50</v>
       </c>
       <c r="N35" t="n">
-        <v>560</v>
+        <v>380</v>
       </c>
     </row>
     <row r="36">
@@ -2302,18 +2302,18 @@
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Camilla</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J36" t="n">
         <v>1</v>
       </c>
       <c r="K36" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L36" t="n">
         <v>3.5</v>
@@ -2322,7 +2322,7 @@
         <v>50</v>
       </c>
       <c r="N36" t="n">
-        <v>550</v>
+        <v>560</v>
       </c>
     </row>
     <row r="37">
@@ -2354,18 +2354,18 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Nanna</t>
+          <t>Camilla</t>
         </is>
       </c>
       <c r="J37" t="n">
         <v>1</v>
       </c>
       <c r="K37" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L37" t="n">
         <v>3.5</v>
@@ -2406,18 +2406,18 @@
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Ólafur</t>
+          <t>Bergur</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L38" t="n">
         <v>3.5</v>
@@ -2426,7 +2426,7 @@
         <v>50</v>
       </c>
       <c r="N38" t="n">
-        <v>350</v>
+        <v>390</v>
       </c>
     </row>
     <row r="39">
@@ -2614,18 +2614,18 @@
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
+        <v>7</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Harpa</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>2</v>
+      </c>
+      <c r="K42" t="n">
         <v>8</v>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>Vala</t>
-        </is>
-      </c>
-      <c r="J42" t="n">
-        <v>2</v>
-      </c>
-      <c r="K42" t="n">
-        <v>10</v>
       </c>
       <c r="L42" t="n">
         <v>4</v>
@@ -2634,7 +2634,7 @@
         <v>50</v>
       </c>
       <c r="N42" t="n">
-        <v>560</v>
+        <v>540</v>
       </c>
     </row>
     <row r="43">
@@ -2978,11 +2978,11 @@
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J49" t="n">
@@ -3041,7 +3041,7 @@
         <v>1</v>
       </c>
       <c r="K50" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L50" t="n">
         <v>4</v>
@@ -3050,7 +3050,7 @@
         <v>50</v>
       </c>
       <c r="N50" t="n">
-        <v>510</v>
+        <v>560</v>
       </c>
     </row>
     <row r="51">
@@ -3134,18 +3134,18 @@
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Helgi</t>
+          <t>Ásdís</t>
         </is>
       </c>
       <c r="J52" t="n">
         <v>3</v>
       </c>
       <c r="K52" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L52" t="n">
         <v>4</v>
@@ -3154,7 +3154,7 @@
         <v>50</v>
       </c>
       <c r="N52" t="n">
-        <v>390</v>
+        <v>570</v>
       </c>
     </row>
     <row r="53">
@@ -3186,18 +3186,18 @@
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Thelma</t>
+          <t>Helgi</t>
         </is>
       </c>
       <c r="J53" t="n">
         <v>3</v>
       </c>
       <c r="K53" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L53" t="n">
         <v>4</v>
@@ -3206,7 +3206,7 @@
         <v>50</v>
       </c>
       <c r="N53" t="n">
-        <v>570</v>
+        <v>390</v>
       </c>
     </row>
     <row r="54">
@@ -3301,7 +3301,7 @@
         <v>2</v>
       </c>
       <c r="K55" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L55" t="n">
         <v>4</v>
@@ -3342,18 +3342,18 @@
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K56" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L56" t="n">
         <v>4</v>
@@ -3362,7 +3362,7 @@
         <v>50</v>
       </c>
       <c r="N56" t="n">
-        <v>570</v>
+        <v>390</v>
       </c>
     </row>
     <row r="57">
@@ -3394,11 +3394,11 @@
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J57" t="n">
@@ -3457,7 +3457,7 @@
         <v>2</v>
       </c>
       <c r="K58" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L58" t="n">
         <v>4</v>
@@ -3509,7 +3509,7 @@
         <v>2</v>
       </c>
       <c r="K59" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L59" t="n">
         <v>4</v>
@@ -3518,7 +3518,7 @@
         <v>50</v>
       </c>
       <c r="N59" t="n">
-        <v>390</v>
+        <v>560</v>
       </c>
     </row>
     <row r="60">
@@ -3561,7 +3561,7 @@
         <v>2</v>
       </c>
       <c r="K60" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L60" t="n">
         <v>4</v>
@@ -3570,7 +3570,7 @@
         <v>50</v>
       </c>
       <c r="N60" t="n">
-        <v>560</v>
+        <v>390</v>
       </c>
     </row>
     <row r="61">
@@ -3654,18 +3654,18 @@
       </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Bergur</t>
+          <t>Ólafur</t>
         </is>
       </c>
       <c r="J62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K62" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="L62" t="n">
         <v>4</v>
@@ -3674,7 +3674,7 @@
         <v>50</v>
       </c>
       <c r="N62" t="n">
-        <v>380</v>
+        <v>570</v>
       </c>
     </row>
     <row r="63">
@@ -3914,18 +3914,18 @@
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K67" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L67" t="n">
         <v>4</v>
@@ -3934,7 +3934,7 @@
         <v>70</v>
       </c>
       <c r="N67" t="n">
-        <v>340</v>
+        <v>330</v>
       </c>
     </row>
     <row r="68">
@@ -3966,18 +3966,18 @@
       </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K68" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L68" t="n">
         <v>4</v>
@@ -3986,7 +3986,7 @@
         <v>70</v>
       </c>
       <c r="N68" t="n">
-        <v>330</v>
+        <v>340</v>
       </c>
     </row>
     <row r="69">
@@ -4018,18 +4018,18 @@
       </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J69" t="n">
         <v>2</v>
       </c>
       <c r="K69" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L69" t="n">
         <v>4.5</v>
@@ -4070,18 +4070,18 @@
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L70" t="n">
         <v>4.5</v>
@@ -4278,11 +4278,11 @@
       </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J74" t="n">
@@ -4298,7 +4298,7 @@
         <v>50</v>
       </c>
       <c r="N74" t="n">
-        <v>410</v>
+        <v>430</v>
       </c>
     </row>
     <row r="75">
@@ -4330,18 +4330,18 @@
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K75" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="L75" t="n">
         <v>3.5</v>
@@ -4350,7 +4350,7 @@
         <v>50</v>
       </c>
       <c r="N75" t="n">
-        <v>510</v>
+        <v>550</v>
       </c>
     </row>
     <row r="76">
@@ -4382,11 +4382,11 @@
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J76" t="n">
@@ -4434,18 +4434,18 @@
       </c>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J77" t="n">
         <v>2</v>
       </c>
       <c r="K77" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="L77" t="n">
         <v>3.5</v>
@@ -4454,7 +4454,7 @@
         <v>50</v>
       </c>
       <c r="N77" t="n">
-        <v>540</v>
+        <v>520</v>
       </c>
     </row>
     <row r="78">
@@ -4486,18 +4486,18 @@
       </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K78" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L78" t="n">
         <v>3.5</v>
@@ -4506,7 +4506,7 @@
         <v>50</v>
       </c>
       <c r="N78" t="n">
-        <v>380</v>
+        <v>520</v>
       </c>
     </row>
     <row r="79">
@@ -4538,18 +4538,18 @@
       </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J79" t="n">
         <v>2</v>
       </c>
       <c r="K79" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="L79" t="n">
         <v>3.5</v>
@@ -4558,7 +4558,7 @@
         <v>50</v>
       </c>
       <c r="N79" t="n">
-        <v>520</v>
+        <v>510</v>
       </c>
     </row>
     <row r="80">
@@ -4590,11 +4590,11 @@
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J80" t="n">
@@ -4642,18 +4642,18 @@
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Ólafur</t>
         </is>
       </c>
       <c r="J81" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K81" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L81" t="n">
         <v>3.5</v>
@@ -4662,7 +4662,7 @@
         <v>50</v>
       </c>
       <c r="N81" t="n">
-        <v>520</v>
+        <v>350</v>
       </c>
     </row>
     <row r="82">
@@ -4694,18 +4694,18 @@
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Anna</t>
         </is>
       </c>
       <c r="J82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K82" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L82" t="n">
         <v>3.5</v>
@@ -4714,7 +4714,7 @@
         <v>50</v>
       </c>
       <c r="N82" t="n">
-        <v>510</v>
+        <v>550</v>
       </c>
     </row>
     <row r="83">
@@ -4798,11 +4798,11 @@
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Ásdís</t>
+          <t>Thelma</t>
         </is>
       </c>
       <c r="J84" t="n">
@@ -4818,7 +4818,7 @@
         <v>50</v>
       </c>
       <c r="N84" t="n">
-        <v>560</v>
+        <v>570</v>
       </c>
     </row>
     <row r="85">
@@ -5162,18 +5162,18 @@
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J91" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K91" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L91" t="n">
         <v>4</v>
@@ -5182,7 +5182,7 @@
         <v>50</v>
       </c>
       <c r="N91" t="n">
-        <v>560</v>
+        <v>520</v>
       </c>
     </row>
     <row r="92">
@@ -5214,18 +5214,18 @@
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>Nanna</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J92" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K92" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L92" t="n">
         <v>4</v>
@@ -5234,7 +5234,7 @@
         <v>50</v>
       </c>
       <c r="N92" t="n">
-        <v>330</v>
+        <v>570</v>
       </c>
     </row>
     <row r="93">
@@ -5266,15 +5266,15 @@
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>Ólafur</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J93" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K93" t="n">
         <v>10</v>
@@ -5318,18 +5318,18 @@
       </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>Anna</t>
+          <t>Nanna</t>
         </is>
       </c>
       <c r="J94" t="n">
         <v>1</v>
       </c>
       <c r="K94" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L94" t="n">
         <v>4</v>
@@ -5338,7 +5338,7 @@
         <v>50</v>
       </c>
       <c r="N94" t="n">
-        <v>560</v>
+        <v>330</v>
       </c>
     </row>
     <row r="95">
@@ -5537,7 +5537,7 @@
         <v>3</v>
       </c>
       <c r="K98" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L98" t="n">
         <v>3</v>
@@ -5546,7 +5546,7 @@
         <v>70</v>
       </c>
       <c r="N98" t="n">
-        <v>460</v>
+        <v>520</v>
       </c>
     </row>
     <row r="99">
@@ -5589,7 +5589,7 @@
         <v>3</v>
       </c>
       <c r="K99" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L99" t="n">
         <v>3</v>
@@ -5641,7 +5641,7 @@
         <v>3</v>
       </c>
       <c r="K100" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L100" t="n">
         <v>3</v>
@@ -5734,18 +5734,18 @@
       </c>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J102" t="n">
         <v>2</v>
       </c>
       <c r="K102" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="L102" t="n">
         <v>3</v>
@@ -5754,7 +5754,7 @@
         <v>70</v>
       </c>
       <c r="N102" t="n">
-        <v>360</v>
+        <v>530</v>
       </c>
     </row>
     <row r="103">
@@ -5786,18 +5786,18 @@
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J103" t="n">
         <v>2</v>
       </c>
       <c r="K103" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="L103" t="n">
         <v>3</v>
@@ -5806,7 +5806,7 @@
         <v>70</v>
       </c>
       <c r="N103" t="n">
-        <v>530</v>
+        <v>500</v>
       </c>
     </row>
     <row r="104">
@@ -5849,7 +5849,7 @@
         <v>2</v>
       </c>
       <c r="K104" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L104" t="n">
         <v>3</v>
@@ -5858,7 +5858,7 @@
         <v>70</v>
       </c>
       <c r="N104" t="n">
-        <v>490</v>
+        <v>390</v>
       </c>
     </row>
     <row r="105">
@@ -5890,15 +5890,15 @@
       </c>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K105" t="n">
         <v>8</v>
@@ -5910,7 +5910,7 @@
         <v>70</v>
       </c>
       <c r="N105" t="n">
-        <v>520</v>
+        <v>530</v>
       </c>
     </row>
     <row r="106">
@@ -5942,18 +5942,18 @@
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J106" t="n">
         <v>2</v>
       </c>
       <c r="K106" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="L106" t="n">
         <v>3</v>
@@ -5962,7 +5962,7 @@
         <v>70</v>
       </c>
       <c r="N106" t="n">
-        <v>530</v>
+        <v>390</v>
       </c>
     </row>
     <row r="107">
@@ -5994,18 +5994,18 @@
       </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J107" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K107" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L107" t="n">
         <v>3</v>
@@ -6014,7 +6014,7 @@
         <v>70</v>
       </c>
       <c r="N107" t="n">
-        <v>390</v>
+        <v>360</v>
       </c>
     </row>
     <row r="108">
@@ -6046,18 +6046,18 @@
       </c>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Bergur</t>
         </is>
       </c>
       <c r="J108" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K108" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L108" t="n">
         <v>3</v>
@@ -6066,7 +6066,7 @@
         <v>70</v>
       </c>
       <c r="N108" t="n">
-        <v>360</v>
+        <v>530</v>
       </c>
     </row>
     <row r="109">
@@ -6150,11 +6150,11 @@
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Thelma</t>
+          <t>Ásdís</t>
         </is>
       </c>
       <c r="J110" t="n">
@@ -6202,15 +6202,15 @@
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="n">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Thelma</t>
         </is>
       </c>
       <c r="J111" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K111" t="n">
         <v>2</v>
@@ -6222,7 +6222,7 @@
         <v>100</v>
       </c>
       <c r="N111" t="n">
-        <v>460</v>
+        <v>450</v>
       </c>
     </row>
     <row r="112">
@@ -6317,7 +6317,7 @@
         <v>2</v>
       </c>
       <c r="K113" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L113" t="n">
         <v>4</v>
@@ -6358,18 +6358,18 @@
       </c>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J114" t="n">
         <v>2</v>
       </c>
       <c r="K114" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L114" t="n">
         <v>4</v>
@@ -6378,7 +6378,7 @@
         <v>70</v>
       </c>
       <c r="N114" t="n">
-        <v>540</v>
+        <v>440</v>
       </c>
     </row>
     <row r="115">
@@ -6410,18 +6410,18 @@
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J115" t="n">
         <v>2</v>
       </c>
       <c r="K115" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L115" t="n">
         <v>4</v>
@@ -6430,7 +6430,7 @@
         <v>70</v>
       </c>
       <c r="N115" t="n">
-        <v>480</v>
+        <v>460</v>
       </c>
     </row>
     <row r="116">
@@ -6462,18 +6462,18 @@
       </c>
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J116" t="n">
         <v>2</v>
       </c>
       <c r="K116" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L116" t="n">
         <v>4</v>
@@ -6482,7 +6482,7 @@
         <v>70</v>
       </c>
       <c r="N116" t="n">
-        <v>460</v>
+        <v>320</v>
       </c>
     </row>
     <row r="117">
@@ -6514,18 +6514,18 @@
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J117" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K117" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L117" t="n">
         <v>4</v>
@@ -6534,7 +6534,7 @@
         <v>70</v>
       </c>
       <c r="N117" t="n">
-        <v>540</v>
+        <v>340</v>
       </c>
     </row>
     <row r="118">
@@ -6566,18 +6566,18 @@
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J118" t="n">
         <v>2</v>
       </c>
       <c r="K118" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="L118" t="n">
         <v>4</v>
@@ -6586,7 +6586,7 @@
         <v>70</v>
       </c>
       <c r="N118" t="n">
-        <v>540</v>
+        <v>340</v>
       </c>
     </row>
     <row r="119">
@@ -6618,18 +6618,18 @@
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J119" t="n">
         <v>1</v>
       </c>
       <c r="K119" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L119" t="n">
         <v>4</v>
@@ -6638,7 +6638,7 @@
         <v>70</v>
       </c>
       <c r="N119" t="n">
-        <v>340</v>
+        <v>510</v>
       </c>
     </row>
     <row r="120">
@@ -6670,18 +6670,18 @@
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Camilla</t>
         </is>
       </c>
       <c r="J120" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K120" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L120" t="n">
         <v>4</v>
@@ -6690,7 +6690,7 @@
         <v>70</v>
       </c>
       <c r="N120" t="n">
-        <v>340</v>
+        <v>500</v>
       </c>
     </row>
     <row r="121">
@@ -6722,18 +6722,18 @@
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Anna</t>
         </is>
       </c>
       <c r="J121" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K121" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L121" t="n">
         <v>4</v>
@@ -6742,7 +6742,7 @@
         <v>70</v>
       </c>
       <c r="N121" t="n">
-        <v>340</v>
+        <v>500</v>
       </c>
     </row>
     <row r="122">
@@ -6774,18 +6774,18 @@
       </c>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>Camilla</t>
+          <t>Bergur</t>
         </is>
       </c>
       <c r="J122" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K122" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L122" t="n">
         <v>4</v>
@@ -6794,7 +6794,7 @@
         <v>70</v>
       </c>
       <c r="N122" t="n">
-        <v>500</v>
+        <v>460</v>
       </c>
     </row>
     <row r="123">
@@ -6837,7 +6837,7 @@
         <v>1</v>
       </c>
       <c r="K123" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L123" t="n">
         <v>4</v>
@@ -6878,18 +6878,18 @@
       </c>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J124" t="n">
         <v>2</v>
       </c>
       <c r="K124" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L124" t="n">
         <v>2</v>
@@ -6898,7 +6898,7 @@
         <v>70</v>
       </c>
       <c r="N124" t="n">
-        <v>550</v>
+        <v>540</v>
       </c>
     </row>
     <row r="125">
@@ -6930,18 +6930,18 @@
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J125" t="n">
         <v>2</v>
       </c>
       <c r="K125" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L125" t="n">
         <v>2</v>
@@ -6982,18 +6982,18 @@
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J126" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K126" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="L126" t="n">
         <v>2</v>
@@ -7002,7 +7002,7 @@
         <v>70</v>
       </c>
       <c r="N126" t="n">
-        <v>550</v>
+        <v>500</v>
       </c>
     </row>
     <row r="127">
@@ -7034,18 +7034,18 @@
       </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K127" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L127" t="n">
         <v>2</v>
@@ -7054,7 +7054,7 @@
         <v>70</v>
       </c>
       <c r="N127" t="n">
-        <v>500</v>
+        <v>540</v>
       </c>
     </row>
     <row r="128">
@@ -7086,18 +7086,18 @@
       </c>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J128" t="n">
         <v>2</v>
       </c>
       <c r="K128" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="L128" t="n">
         <v>2</v>
@@ -7106,7 +7106,7 @@
         <v>70</v>
       </c>
       <c r="N128" t="n">
-        <v>550</v>
+        <v>540</v>
       </c>
     </row>
     <row r="129">
@@ -7138,18 +7138,18 @@
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J129" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K129" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L129" t="n">
         <v>2</v>
@@ -7158,7 +7158,7 @@
         <v>70</v>
       </c>
       <c r="N129" t="n">
-        <v>510</v>
+        <v>550</v>
       </c>
     </row>
     <row r="130">
@@ -7190,18 +7190,18 @@
       </c>
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J130" t="n">
         <v>1</v>
       </c>
       <c r="K130" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L130" t="n">
         <v>2</v>
@@ -7210,7 +7210,7 @@
         <v>70</v>
       </c>
       <c r="N130" t="n">
-        <v>340</v>
+        <v>550</v>
       </c>
     </row>
     <row r="131">
@@ -7242,18 +7242,18 @@
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J131" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L131" t="n">
         <v>2</v>
@@ -7294,18 +7294,18 @@
       </c>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J132" t="n">
         <v>2</v>
       </c>
       <c r="K132" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L132" t="n">
         <v>2</v>
@@ -7346,18 +7346,18 @@
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Ólafur</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J133" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K133" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L133" t="n">
         <v>2</v>
@@ -7366,7 +7366,7 @@
         <v>70</v>
       </c>
       <c r="N133" t="n">
-        <v>520</v>
+        <v>340</v>
       </c>
     </row>
     <row r="134">
@@ -7398,18 +7398,18 @@
       </c>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Bergur</t>
+          <t>Ólafur</t>
         </is>
       </c>
       <c r="J134" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K134" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L134" t="n">
         <v>2</v>
@@ -7418,7 +7418,7 @@
         <v>70</v>
       </c>
       <c r="N134" t="n">
-        <v>540</v>
+        <v>520</v>
       </c>
     </row>
     <row r="135">
@@ -7719,33 +7719,31 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
-      <c r="D2" t="n">
-        <v>1</v>
-      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
         <v>1</v>
       </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="n">
-        <v>1</v>
-      </c>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="n">
         <v>1</v>
       </c>
       <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
+      <c r="T2" t="n">
+        <v>1</v>
+      </c>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
@@ -7837,9 +7835,7 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" t="n">
-        <v>1</v>
-      </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="n">
         <v>1</v>
       </c>
@@ -7847,7 +7843,9 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
+      <c r="P5" t="n">
+        <v>1</v>
+      </c>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="n">
         <v>1</v>
@@ -7901,17 +7899,17 @@
       <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="n">
-        <v>1</v>
-      </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
@@ -7926,10 +7924,10 @@
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
-      <c r="U7" t="n">
-        <v>1</v>
-      </c>
-      <c r="V7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="n">
+        <v>1</v>
+      </c>
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
     </row>
@@ -7941,27 +7939,29 @@
         <v>1</v>
       </c>
       <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="n">
         <v>1</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="n">
-        <v>1</v>
-      </c>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="n">
-        <v>1</v>
-      </c>
+      <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="n">
@@ -7984,22 +7984,20 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="n">
-        <v>1</v>
-      </c>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="n">
         <v>1</v>
       </c>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" t="n">
-        <v>1</v>
-      </c>
+      <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
+      <c r="R9" t="n">
+        <v>1</v>
+      </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="n">
@@ -8051,7 +8049,9 @@
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
@@ -8061,23 +8061,23 @@
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="n">
-        <v>1</v>
-      </c>
+      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
+      <c r="N11" t="n">
+        <v>1</v>
+      </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="n">
         <v>1</v>
       </c>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
+      <c r="R11" t="n">
+        <v>1</v>
+      </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
-      <c r="V11" t="n">
-        <v>1</v>
-      </c>
+      <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr"/>
     </row>
@@ -8091,7 +8091,9 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
       <c r="I12" t="n">
         <v>1</v>
       </c>
@@ -8111,9 +8113,7 @@
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
-      <c r="V12" t="n">
-        <v>1</v>
-      </c>
+      <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
       <c r="X12" t="inlineStr"/>
     </row>
@@ -8127,9 +8127,7 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" t="n">
-        <v>1</v>
-      </c>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
         <v>1</v>
       </c>
@@ -8137,7 +8135,9 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
+      <c r="N13" t="n">
+        <v>1</v>
+      </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
@@ -8163,7 +8163,9 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>1</v>
+      </c>
       <c r="I14" t="n">
         <v>1</v>
       </c>
@@ -8183,9 +8185,7 @@
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
-      <c r="V14" t="n">
-        <v>1</v>
-      </c>
+      <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
       <c r="X14" t="inlineStr"/>
     </row>
@@ -8218,10 +8218,10 @@
         <v>1</v>
       </c>
       <c r="T15" t="inlineStr"/>
-      <c r="U15" t="n">
-        <v>1</v>
-      </c>
-      <c r="V15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="n">
+        <v>1</v>
+      </c>
       <c r="W15" t="inlineStr"/>
       <c r="X15" t="inlineStr"/>
     </row>
@@ -8252,10 +8252,10 @@
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr"/>
-      <c r="U16" t="n">
-        <v>1</v>
-      </c>
-      <c r="V16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="n">
+        <v>1</v>
+      </c>
       <c r="W16" t="n">
         <v>1</v>
       </c>
@@ -8272,28 +8272,28 @@
         <v>1</v>
       </c>
       <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="n">
-        <v>1</v>
-      </c>
+      <c r="J17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="n">
-        <v>1</v>
-      </c>
+      <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="n">
-        <v>1</v>
-      </c>
+      <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
+      <c r="V17" t="n">
+        <v>1</v>
+      </c>
       <c r="W17" t="inlineStr"/>
       <c r="X17" t="inlineStr"/>
     </row>
@@ -8302,35 +8302,33 @@
         <v>17</v>
       </c>
       <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="n">
-        <v>1</v>
-      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
-      <c r="F18" t="n">
-        <v>1</v>
-      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" t="n">
-        <v>1</v>
-      </c>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" t="n">
-        <v>1</v>
-      </c>
+      <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
+      <c r="P18" t="n">
+        <v>1</v>
+      </c>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="n">
         <v>1</v>
       </c>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
+      <c r="U18" t="n">
+        <v>1</v>
+      </c>
       <c r="V18" t="inlineStr"/>
       <c r="W18" t="inlineStr"/>
       <c r="X18" t="inlineStr"/>
@@ -8344,7 +8342,9 @@
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
@@ -8365,9 +8365,7 @@
       <c r="U19" t="n">
         <v>1</v>
       </c>
-      <c r="V19" t="n">
-        <v>1</v>
-      </c>
+      <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr"/>
       <c r="X19" t="inlineStr"/>
     </row>
@@ -8378,34 +8376,32 @@
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="n">
-        <v>1</v>
-      </c>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>1</v>
+      </c>
       <c r="I20" t="inlineStr"/>
-      <c r="J20" t="n">
-        <v>1</v>
-      </c>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="n">
         <v>1</v>
       </c>
-      <c r="L20" t="inlineStr"/>
+      <c r="L20" t="n">
+        <v>1</v>
+      </c>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="n">
-        <v>1</v>
-      </c>
+      <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="n">
-        <v>1</v>
-      </c>
+      <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr"/>
+      <c r="V20" t="n">
+        <v>1</v>
+      </c>
       <c r="W20" t="inlineStr"/>
       <c r="X20" t="inlineStr"/>
     </row>
@@ -8414,19 +8410,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="inlineStr"/>
-      <c r="C21" t="n">
-        <v>1</v>
-      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
-      <c r="J21" t="n">
-        <v>1</v>
-      </c>
-      <c r="K21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="n">
+        <v>1</v>
+      </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="n">
@@ -8435,12 +8431,12 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
+      <c r="R21" t="n">
+        <v>1</v>
+      </c>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr"/>
-      <c r="U21" t="n">
-        <v>1</v>
-      </c>
+      <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
       <c r="X21" t="inlineStr"/>
@@ -8450,28 +8446,28 @@
         <v>21</v>
       </c>
       <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="n">
-        <v>1</v>
-      </c>
+      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" t="n">
-        <v>1</v>
-      </c>
+      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
+      <c r="J22" t="n">
+        <v>1</v>
+      </c>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
+      <c r="N22" t="n">
+        <v>1</v>
+      </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="n">
-        <v>1</v>
-      </c>
+      <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="n">
@@ -8541,7 +8537,9 @@
         <v>1</v>
       </c>
       <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
+      <c r="P24" t="n">
+        <v>1</v>
+      </c>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
@@ -8557,16 +8555,18 @@
       <c r="A25" t="n">
         <v>24</v>
       </c>
-      <c r="B25" t="n">
-        <v>1</v>
-      </c>
+      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
+      <c r="I25" t="n">
+        <v>1</v>
+      </c>
       <c r="J25" t="n">
         <v>1</v>
       </c>
@@ -8579,13 +8579,13 @@
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
+      <c r="R25" t="n">
+        <v>1</v>
+      </c>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
-      <c r="V25" t="n">
-        <v>1</v>
-      </c>
+      <c r="V25" t="inlineStr"/>
       <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr"/>
     </row>
@@ -8593,18 +8593,16 @@
       <c r="A26" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="inlineStr"/>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="n">
-        <v>1</v>
-      </c>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
-      <c r="I26" t="n">
-        <v>1</v>
-      </c>
+      <c r="I26" t="inlineStr"/>
       <c r="J26" t="n">
         <v>1</v>
       </c>
@@ -8615,15 +8613,17 @@
         <v>1</v>
       </c>
       <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
+      <c r="P26" t="n">
+        <v>1</v>
+      </c>
       <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="n">
-        <v>1</v>
-      </c>
+      <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr"/>
+      <c r="V26" t="n">
+        <v>1</v>
+      </c>
       <c r="W26" t="inlineStr"/>
       <c r="X26" t="inlineStr"/>
     </row>
@@ -8637,7 +8637,9 @@
       <c r="E27" t="n">
         <v>1</v>
       </c>
-      <c r="F27" t="inlineStr"/>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="n">
@@ -8649,18 +8651,16 @@
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
-      <c r="P27" t="n">
-        <v>1</v>
-      </c>
+      <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="n">
         <v>1</v>
       </c>
       <c r="S27" t="inlineStr"/>
-      <c r="T27" t="n">
-        <v>1</v>
-      </c>
-      <c r="U27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="n">
+        <v>1</v>
+      </c>
       <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr"/>
@@ -8705,7 +8705,9 @@
       <c r="A29" t="n">
         <v>28</v>
       </c>
-      <c r="B29" t="inlineStr"/>
+      <c r="B29" t="n">
+        <v>1</v>
+      </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="n">
@@ -8713,9 +8715,7 @@
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
-      <c r="H29" t="n">
-        <v>1</v>
-      </c>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="n">
         <v>1</v>
@@ -8747,19 +8747,19 @@
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" t="n">
-        <v>1</v>
-      </c>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
+      <c r="J30" t="n">
+        <v>1</v>
+      </c>
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
+      <c r="N30" t="n">
+        <v>1</v>
+      </c>
       <c r="O30" t="inlineStr"/>
-      <c r="P30" t="n">
-        <v>1</v>
-      </c>
+      <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr"/>
@@ -8780,9 +8780,7 @@
       <c r="B31" t="n">
         <v>1</v>
       </c>
-      <c r="C31" t="n">
-        <v>1</v>
-      </c>
+      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
@@ -8795,16 +8793,18 @@
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
+      <c r="N31" t="n">
+        <v>1</v>
+      </c>
       <c r="O31" t="inlineStr"/>
-      <c r="P31" t="n">
-        <v>1</v>
-      </c>
+      <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr"/>
-      <c r="U31" t="inlineStr"/>
+      <c r="U31" t="n">
+        <v>1</v>
+      </c>
       <c r="V31" t="inlineStr"/>
       <c r="W31" t="inlineStr"/>
       <c r="X31" t="inlineStr"/>
@@ -8816,18 +8816,16 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
-      <c r="E32" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="n">
-        <v>1</v>
-      </c>
-      <c r="H32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="n">
+        <v>1</v>
+      </c>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" t="n">
-        <v>1</v>
-      </c>
+      <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
@@ -8835,13 +8833,15 @@
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr"/>
+      <c r="R32" t="n">
+        <v>1</v>
+      </c>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr"/>
-      <c r="U32" t="inlineStr"/>
-      <c r="V32" t="n">
-        <v>1</v>
-      </c>
+      <c r="U32" t="n">
+        <v>1</v>
+      </c>
+      <c r="V32" t="inlineStr"/>
       <c r="W32" t="inlineStr"/>
       <c r="X32" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
lagaði hvernig excel results prentar
</commit_message>
<xml_diff>
--- a/03_26_schedule_results.xlsx
+++ b/03_26_schedule_results.xlsx
@@ -7588,7 +7588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X33"/>
+  <dimension ref="A1:AF33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7624,90 +7624,130 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>6.5.2024</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>7.5.2024</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>8.5.2024</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>9.5.2024</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>10.5.2024</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>11.5.2024</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>12.5.2024</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>13.5.2024</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>14.5.2024</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>15.5.2024</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>16.5.2024</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>17.5.2024</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>18.5.2024</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>19.5.2024</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>20.5.2024</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>21.5.2024</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>22.5.2024</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>23.5.2024</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>24.5.2024</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>25.5.2024</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>26.5.2024</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>27.5.2024</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>28.5.2024</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>29.5.2024</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>30.5.2024</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>31.5.2024</t>
         </is>
@@ -7727,27 +7767,35 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
-      <c r="T2" t="n">
-        <v>1</v>
-      </c>
-      <c r="U2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="n">
+        <v>1</v>
+      </c>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -7762,30 +7810,38 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="n">
-        <v>1</v>
-      </c>
+      <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
+      <c r="U3" t="n">
+        <v>1</v>
+      </c>
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -7808,18 +7864,26 @@
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R4" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
+      <c r="T4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U4" t="n">
+        <v>1</v>
+      </c>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
-      <c r="X4" t="n">
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7836,28 +7900,36 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="n">
-        <v>1</v>
-      </c>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
-      <c r="P5" t="n">
-        <v>1</v>
-      </c>
+      <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="n">
-        <v>1</v>
-      </c>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="n">
-        <v>1</v>
-      </c>
-      <c r="U5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="n">
+        <v>1</v>
+      </c>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="n">
+        <v>1</v>
+      </c>
       <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -7870,30 +7942,38 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="n">
-        <v>1</v>
-      </c>
+      <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
+      <c r="Q6" t="n">
+        <v>1</v>
+      </c>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
-      <c r="U6" t="n">
-        <v>1</v>
-      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -7907,29 +7987,37 @@
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" t="n">
-        <v>1</v>
-      </c>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
+      <c r="T7" t="n">
+        <v>1</v>
+      </c>
       <c r="U7" t="inlineStr"/>
-      <c r="V7" t="n">
-        <v>1</v>
-      </c>
+      <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -7945,18 +8033,18 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" t="n">
-        <v>1</v>
-      </c>
-      <c r="I8" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="n">
+        <v>1</v>
+      </c>
       <c r="K8" t="n">
         <v>1</v>
       </c>
       <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
+      <c r="M8" t="n">
+        <v>1</v>
+      </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
@@ -7964,12 +8052,20 @@
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
-      <c r="U8" t="n">
-        <v>1</v>
-      </c>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -7985,19 +8081,17 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" t="n">
-        <v>1</v>
-      </c>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="n">
-        <v>1</v>
-      </c>
+      <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="n">
@@ -8006,6 +8100,16 @@
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -8017,31 +8121,39 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="n">
-        <v>1</v>
-      </c>
+      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="n">
-        <v>1</v>
-      </c>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>1</v>
+      </c>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
-      <c r="P10" t="n">
-        <v>1</v>
-      </c>
+      <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
+      <c r="S10" t="n">
+        <v>1</v>
+      </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
-      <c r="V10" t="n">
-        <v>1</v>
-      </c>
+      <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -8056,30 +8168,38 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="n">
-        <v>1</v>
-      </c>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="n">
-        <v>1</v>
-      </c>
+      <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
-      <c r="P11" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="n">
-        <v>1</v>
-      </c>
-      <c r="S11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="n">
+        <v>1</v>
+      </c>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="n">
+        <v>1</v>
+      </c>
       <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
+      <c r="U11" t="n">
+        <v>1</v>
+      </c>
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -8091,31 +8211,39 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="n">
-        <v>1</v>
-      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
+      <c r="N12" t="n">
+        <v>1</v>
+      </c>
       <c r="O12" t="inlineStr"/>
-      <c r="P12" t="n">
-        <v>1</v>
-      </c>
+      <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
+      <c r="S12" t="n">
+        <v>1</v>
+      </c>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
       <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr"/>
+      <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -8128,28 +8256,36 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="n">
-        <v>1</v>
-      </c>
+      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" t="n">
-        <v>1</v>
-      </c>
+      <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
+      <c r="Q13" t="n">
+        <v>1</v>
+      </c>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
-      <c r="V13" t="n">
-        <v>1</v>
-      </c>
+      <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr"/>
-      <c r="X13" t="n">
+      <c r="X13" t="inlineStr"/>
+      <c r="Y13" t="inlineStr"/>
+      <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr"/>
+      <c r="AD13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8163,31 +8299,39 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I14" t="n">
-        <v>1</v>
-      </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" t="n">
+        <v>1</v>
+      </c>
       <c r="L14" t="inlineStr"/>
-      <c r="M14" t="n">
-        <v>1</v>
-      </c>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="n">
-        <v>1</v>
-      </c>
+      <c r="O14" t="n">
+        <v>1</v>
+      </c>
+      <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
+      <c r="S14" t="n">
+        <v>1</v>
+      </c>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
       <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr"/>
+      <c r="Z14" t="inlineStr"/>
+      <c r="AA14" t="inlineStr"/>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr"/>
+      <c r="AD14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -8200,18 +8344,16 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
-      <c r="I15" t="n">
-        <v>1</v>
-      </c>
+      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="K15" t="n">
+        <v>1</v>
+      </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
-      <c r="P15" t="n">
-        <v>1</v>
-      </c>
+      <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="n">
@@ -8219,11 +8361,21 @@
       </c>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
-      <c r="V15" t="n">
-        <v>1</v>
-      </c>
+      <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
+      <c r="X15" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
+      <c r="AD15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr"/>
+      <c r="AF15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -8236,30 +8388,38 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" t="n">
-        <v>1</v>
-      </c>
+      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="K16" t="n">
+        <v>1</v>
+      </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
-      <c r="P16" t="n">
-        <v>1</v>
-      </c>
+      <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
+      <c r="S16" t="n">
+        <v>1</v>
+      </c>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
-      <c r="V16" t="n">
-        <v>1</v>
-      </c>
-      <c r="W16" t="n">
-        <v>1</v>
-      </c>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr"/>
       <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
+      <c r="AA16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
+      <c r="AD16" t="inlineStr"/>
+      <c r="AE16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -8272,16 +8432,16 @@
         <v>1</v>
       </c>
       <c r="F17" t="inlineStr"/>
-      <c r="G17" t="n">
-        <v>1</v>
-      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="n">
-        <v>1</v>
-      </c>
+      <c r="I17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
+      <c r="L17" t="n">
+        <v>1</v>
+      </c>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
@@ -8291,11 +8451,19 @@
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
-      <c r="V17" t="n">
-        <v>1</v>
-      </c>
+      <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr"/>
       <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr"/>
+      <c r="AD17" t="inlineStr"/>
+      <c r="AE17" t="inlineStr"/>
+      <c r="AF17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -8317,14 +8485,12 @@
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" t="n">
-        <v>1</v>
-      </c>
+      <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="n">
-        <v>1</v>
-      </c>
-      <c r="S18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="n">
+        <v>1</v>
+      </c>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="n">
         <v>1</v>
@@ -8332,6 +8498,16 @@
       <c r="V18" t="inlineStr"/>
       <c r="W18" t="inlineStr"/>
       <c r="X18" t="inlineStr"/>
+      <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA18" t="inlineStr"/>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr"/>
+      <c r="AD18" t="inlineStr"/>
+      <c r="AE18" t="inlineStr"/>
+      <c r="AF18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -8347,11 +8523,11 @@
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" t="n">
-        <v>1</v>
-      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
+      <c r="J19" t="n">
+        <v>1</v>
+      </c>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
@@ -8362,12 +8538,20 @@
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr"/>
-      <c r="U19" t="n">
-        <v>1</v>
-      </c>
+      <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr"/>
       <c r="X19" t="inlineStr"/>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA19" t="inlineStr"/>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr"/>
+      <c r="AD19" t="inlineStr"/>
+      <c r="AE19" t="inlineStr"/>
+      <c r="AF19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -8379,19 +8563,19 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" t="n">
-        <v>1</v>
-      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="n">
-        <v>1</v>
-      </c>
-      <c r="L20" t="n">
-        <v>1</v>
-      </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
+      <c r="J20" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N20" t="n">
+        <v>1</v>
+      </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
@@ -8399,11 +8583,19 @@
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
-      <c r="V20" t="n">
-        <v>1</v>
-      </c>
+      <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr"/>
       <c r="X20" t="inlineStr"/>
+      <c r="Y20" t="inlineStr"/>
+      <c r="Z20" t="inlineStr"/>
+      <c r="AA20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr"/>
+      <c r="AD20" t="inlineStr"/>
+      <c r="AE20" t="inlineStr"/>
+      <c r="AF20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -8420,26 +8612,34 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
-      <c r="K21" t="n">
-        <v>1</v>
-      </c>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="n">
-        <v>1</v>
-      </c>
+      <c r="M21" t="n">
+        <v>1</v>
+      </c>
+      <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q21" t="n">
+        <v>1</v>
+      </c>
+      <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
+      <c r="U21" t="n">
+        <v>1</v>
+      </c>
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
       <c r="X21" t="inlineStr"/>
+      <c r="Y21" t="inlineStr"/>
+      <c r="Z21" t="inlineStr"/>
+      <c r="AA21" t="inlineStr"/>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr"/>
+      <c r="AD21" t="inlineStr"/>
+      <c r="AE21" t="inlineStr"/>
+      <c r="AF21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -8455,27 +8655,35 @@
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" t="n">
-        <v>1</v>
-      </c>
+      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
+      <c r="L22" t="n">
+        <v>1</v>
+      </c>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" t="n">
-        <v>1</v>
-      </c>
+      <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
+      <c r="Q22" t="n">
+        <v>1</v>
+      </c>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr"/>
-      <c r="U22" t="n">
-        <v>1</v>
-      </c>
+      <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr"/>
       <c r="X22" t="inlineStr"/>
+      <c r="Y22" t="inlineStr"/>
+      <c r="Z22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA22" t="inlineStr"/>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr"/>
+      <c r="AD22" t="inlineStr"/>
+      <c r="AE22" t="inlineStr"/>
+      <c r="AF22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -8489,29 +8697,37 @@
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" t="n">
-        <v>1</v>
-      </c>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
+      <c r="J23" t="n">
+        <v>1</v>
+      </c>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
-      <c r="O23" t="n">
-        <v>1</v>
-      </c>
+      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
+      <c r="R23" t="n">
+        <v>1</v>
+      </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
-      <c r="V23" t="n">
-        <v>1</v>
-      </c>
+      <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr"/>
       <c r="X23" t="inlineStr"/>
+      <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr"/>
+      <c r="AA23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr"/>
+      <c r="AD23" t="inlineStr"/>
+      <c r="AE23" t="inlineStr"/>
+      <c r="AF23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -8527,29 +8743,37 @@
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" t="n">
-        <v>1</v>
-      </c>
+      <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
+      <c r="L24" t="n">
+        <v>1</v>
+      </c>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" t="n">
-        <v>1</v>
-      </c>
+      <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
-      <c r="P24" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="n">
+        <v>1</v>
+      </c>
       <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
+      <c r="S24" t="n">
+        <v>1</v>
+      </c>
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
-      <c r="V24" t="n">
-        <v>1</v>
-      </c>
+      <c r="V24" t="inlineStr"/>
       <c r="W24" t="inlineStr"/>
       <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr"/>
+      <c r="AD24" t="inlineStr"/>
+      <c r="AE24" t="inlineStr"/>
+      <c r="AF24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -8564,30 +8788,38 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
-      <c r="I25" t="n">
-        <v>1</v>
-      </c>
-      <c r="J25" t="n">
-        <v>1</v>
-      </c>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="n">
+        <v>1</v>
+      </c>
+      <c r="L25" t="n">
+        <v>1</v>
+      </c>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="n">
-        <v>1</v>
-      </c>
+      <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q25" t="n">
+        <v>1</v>
+      </c>
+      <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
+      <c r="U25" t="n">
+        <v>1</v>
+      </c>
       <c r="V25" t="inlineStr"/>
       <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr"/>
+      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr"/>
+      <c r="AD25" t="inlineStr"/>
+      <c r="AE25" t="inlineStr"/>
+      <c r="AF25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -8603,29 +8835,37 @@
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="n">
-        <v>1</v>
-      </c>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
+      <c r="L26" t="n">
+        <v>1</v>
+      </c>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" t="n">
-        <v>1</v>
-      </c>
+      <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
-      <c r="P26" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="n">
+        <v>1</v>
+      </c>
       <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr"/>
+      <c r="S26" t="n">
+        <v>1</v>
+      </c>
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
-      <c r="V26" t="n">
-        <v>1</v>
-      </c>
+      <c r="V26" t="inlineStr"/>
       <c r="W26" t="inlineStr"/>
       <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB26" t="inlineStr"/>
+      <c r="AC26" t="inlineStr"/>
+      <c r="AD26" t="inlineStr"/>
+      <c r="AE26" t="inlineStr"/>
+      <c r="AF26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -8642,20 +8882,18 @@
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
-      <c r="I27" t="n">
-        <v>1</v>
-      </c>
+      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+      <c r="K27" t="n">
+        <v>1</v>
+      </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="n">
-        <v>1</v>
-      </c>
+      <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr"/>
       <c r="U27" t="n">
@@ -8664,6 +8902,16 @@
       <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA27" t="inlineStr"/>
+      <c r="AB27" t="inlineStr"/>
+      <c r="AC27" t="inlineStr"/>
+      <c r="AD27" t="inlineStr"/>
+      <c r="AE27" t="inlineStr"/>
+      <c r="AF27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -8677,15 +8925,15 @@
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
-      <c r="H28" t="n">
-        <v>1</v>
-      </c>
+      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="n">
         <v>1</v>
       </c>
       <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
+      <c r="L28" t="n">
+        <v>1</v>
+      </c>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr"/>
@@ -8694,12 +8942,20 @@
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr"/>
-      <c r="U28" t="n">
-        <v>1</v>
-      </c>
+      <c r="U28" t="inlineStr"/>
       <c r="V28" t="inlineStr"/>
       <c r="W28" t="inlineStr"/>
       <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA28" t="inlineStr"/>
+      <c r="AB28" t="inlineStr"/>
+      <c r="AC28" t="inlineStr"/>
+      <c r="AD28" t="inlineStr"/>
+      <c r="AE28" t="inlineStr"/>
+      <c r="AF28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -8717,25 +8973,33 @@
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" t="n">
-        <v>1</v>
-      </c>
+      <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
+      <c r="L29" t="n">
+        <v>1</v>
+      </c>
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
-      <c r="P29" t="n">
-        <v>1</v>
-      </c>
+      <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr"/>
-      <c r="S29" t="inlineStr"/>
+      <c r="S29" t="n">
+        <v>1</v>
+      </c>
       <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="inlineStr"/>
       <c r="W29" t="inlineStr"/>
       <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
+      <c r="AA29" t="inlineStr"/>
+      <c r="AB29" t="inlineStr"/>
+      <c r="AC29" t="inlineStr"/>
+      <c r="AD29" t="inlineStr"/>
+      <c r="AE29" t="inlineStr"/>
+      <c r="AF29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -8749,29 +9013,37 @@
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" t="n">
-        <v>1</v>
-      </c>
+      <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
+      <c r="L30" t="n">
+        <v>1</v>
+      </c>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" t="n">
-        <v>1</v>
-      </c>
+      <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
+      <c r="Q30" t="n">
+        <v>1</v>
+      </c>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr"/>
-      <c r="T30" t="n">
-        <v>1</v>
-      </c>
+      <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr"/>
-      <c r="V30" t="n">
-        <v>1</v>
-      </c>
+      <c r="V30" t="inlineStr"/>
       <c r="W30" t="inlineStr"/>
       <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z30" t="inlineStr"/>
+      <c r="AA30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB30" t="inlineStr"/>
+      <c r="AC30" t="inlineStr"/>
+      <c r="AD30" t="inlineStr"/>
+      <c r="AE30" t="inlineStr"/>
+      <c r="AF30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -8788,26 +9060,34 @@
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
-      <c r="K31" t="n">
-        <v>1</v>
-      </c>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="n">
-        <v>1</v>
-      </c>
+      <c r="M31" t="n">
+        <v>1</v>
+      </c>
+      <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
+      <c r="Q31" t="n">
+        <v>1</v>
+      </c>
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr"/>
-      <c r="U31" t="n">
-        <v>1</v>
-      </c>
+      <c r="U31" t="inlineStr"/>
       <c r="V31" t="inlineStr"/>
       <c r="W31" t="inlineStr"/>
       <c r="X31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr"/>
+      <c r="Z31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA31" t="inlineStr"/>
+      <c r="AB31" t="inlineStr"/>
+      <c r="AC31" t="inlineStr"/>
+      <c r="AD31" t="inlineStr"/>
+      <c r="AE31" t="inlineStr"/>
+      <c r="AF31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -8821,11 +9101,11 @@
         <v>1</v>
       </c>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" t="n">
-        <v>1</v>
-      </c>
+      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
+      <c r="J32" t="n">
+        <v>1</v>
+      </c>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
@@ -8833,9 +9113,7 @@
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="n">
-        <v>1</v>
-      </c>
+      <c r="R32" t="inlineStr"/>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr"/>
       <c r="U32" t="n">
@@ -8844,6 +9122,16 @@
       <c r="V32" t="inlineStr"/>
       <c r="W32" t="inlineStr"/>
       <c r="X32" t="inlineStr"/>
+      <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA32" t="inlineStr"/>
+      <c r="AB32" t="inlineStr"/>
+      <c r="AC32" t="inlineStr"/>
+      <c r="AD32" t="inlineStr"/>
+      <c r="AE32" t="inlineStr"/>
+      <c r="AF32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -8857,29 +9145,37 @@
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="n">
-        <v>1</v>
-      </c>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
+      <c r="J33" t="n">
+        <v>1</v>
+      </c>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr"/>
-      <c r="T33" t="inlineStr"/>
-      <c r="U33" t="n">
-        <v>1</v>
-      </c>
+      <c r="T33" t="n">
+        <v>1</v>
+      </c>
+      <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr"/>
       <c r="W33" t="inlineStr"/>
       <c r="X33" t="inlineStr"/>
+      <c r="Y33" t="inlineStr"/>
+      <c r="Z33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA33" t="inlineStr"/>
+      <c r="AB33" t="inlineStr"/>
+      <c r="AC33" t="inlineStr"/>
+      <c r="AD33" t="inlineStr"/>
+      <c r="AE33" t="inlineStr"/>
+      <c r="AF33" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bætti við persónulegum stigum f. category
til að dreifa aðeins betur categories á hvern starfsmann. breytti líka væginu á persónulegum stigum fyrir fjölda vakta í hverri viku, nú dreifast vaktir enn betur yfir tímabilið
</commit_message>
<xml_diff>
--- a/03_26_schedule_results.xlsx
+++ b/03_26_schedule_results.xlsx
@@ -534,11 +534,11 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -554,7 +554,7 @@
         <v>40</v>
       </c>
       <c r="N2" t="n">
-        <v>400</v>
+        <v>370</v>
       </c>
     </row>
     <row r="3">
@@ -586,15 +586,15 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" t="n">
         <v>1</v>
@@ -606,7 +606,7 @@
         <v>40</v>
       </c>
       <c r="N3" t="n">
-        <v>540</v>
+        <v>430</v>
       </c>
     </row>
     <row r="4">
@@ -638,15 +638,15 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -658,7 +658,7 @@
         <v>100</v>
       </c>
       <c r="N4" t="n">
-        <v>480</v>
+        <v>440</v>
       </c>
     </row>
     <row r="5">
@@ -690,18 +690,18 @@
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Össur</t>
+          <t>Thelma</t>
         </is>
       </c>
       <c r="J5" t="n">
         <v>3</v>
       </c>
       <c r="K5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L5" t="n">
         <v>3</v>
@@ -710,7 +710,7 @@
         <v>80</v>
       </c>
       <c r="N5" t="n">
-        <v>430</v>
+        <v>410</v>
       </c>
     </row>
     <row r="6">
@@ -742,18 +742,18 @@
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Thelma</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L6" t="n">
         <v>3</v>
@@ -762,7 +762,7 @@
         <v>80</v>
       </c>
       <c r="N6" t="n">
-        <v>410</v>
+        <v>470</v>
       </c>
     </row>
     <row r="7">
@@ -846,11 +846,11 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J8" t="n">
@@ -898,11 +898,11 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J9" t="n">
@@ -1002,15 +1002,15 @@
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Helgi</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K11" t="n">
         <v>1</v>
@@ -1022,7 +1022,7 @@
         <v>40</v>
       </c>
       <c r="N11" t="n">
-        <v>550</v>
+        <v>440</v>
       </c>
     </row>
     <row r="12">
@@ -1054,11 +1054,11 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Bergur</t>
         </is>
       </c>
       <c r="J12" t="n">
@@ -1158,18 +1158,18 @@
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Össur</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L14" t="n">
         <v>4</v>
@@ -1178,7 +1178,7 @@
         <v>70</v>
       </c>
       <c r="N14" t="n">
-        <v>340</v>
+        <v>420</v>
       </c>
     </row>
     <row r="15">
@@ -1210,18 +1210,18 @@
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
+        <v>7</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Harpa</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K15" t="n">
         <v>9</v>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Freyja</t>
-        </is>
-      </c>
-      <c r="J15" t="n">
-        <v>2</v>
-      </c>
-      <c r="K15" t="n">
-        <v>6</v>
       </c>
       <c r="L15" t="n">
         <v>4</v>
@@ -1230,7 +1230,7 @@
         <v>70</v>
       </c>
       <c r="N15" t="n">
-        <v>460</v>
+        <v>510</v>
       </c>
     </row>
     <row r="16">
@@ -1262,18 +1262,18 @@
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L16" t="n">
         <v>4</v>
@@ -1282,7 +1282,7 @@
         <v>70</v>
       </c>
       <c r="N16" t="n">
-        <v>510</v>
+        <v>340</v>
       </c>
     </row>
     <row r="17">
@@ -1325,7 +1325,7 @@
         <v>2</v>
       </c>
       <c r="K17" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L17" t="n">
         <v>4</v>
@@ -1366,18 +1366,18 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J18" t="n">
         <v>2</v>
       </c>
       <c r="K18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L18" t="n">
         <v>4</v>
@@ -1386,7 +1386,7 @@
         <v>70</v>
       </c>
       <c r="N18" t="n">
-        <v>470</v>
+        <v>500</v>
       </c>
     </row>
     <row r="19">
@@ -1418,18 +1418,18 @@
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L19" t="n">
         <v>4</v>
@@ -1438,7 +1438,7 @@
         <v>70</v>
       </c>
       <c r="N19" t="n">
-        <v>330</v>
+        <v>470</v>
       </c>
     </row>
     <row r="20">
@@ -1470,18 +1470,18 @@
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
         <v>4</v>
@@ -1490,7 +1490,7 @@
         <v>70</v>
       </c>
       <c r="N20" t="n">
-        <v>340</v>
+        <v>330</v>
       </c>
     </row>
     <row r="21">
@@ -1522,18 +1522,18 @@
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J21" t="n">
         <v>2</v>
       </c>
       <c r="K21" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L21" t="n">
         <v>4</v>
@@ -1542,7 +1542,7 @@
         <v>70</v>
       </c>
       <c r="N21" t="n">
-        <v>460</v>
+        <v>340</v>
       </c>
     </row>
     <row r="22">
@@ -1574,11 +1574,11 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J22" t="n">
@@ -1594,7 +1594,7 @@
         <v>70</v>
       </c>
       <c r="N22" t="n">
-        <v>510</v>
+        <v>520</v>
       </c>
     </row>
     <row r="23">
@@ -1626,18 +1626,18 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Ólafur</t>
+          <t>Camilla</t>
         </is>
       </c>
       <c r="J23" t="n">
         <v>1</v>
       </c>
       <c r="K23" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L23" t="n">
         <v>4</v>
@@ -1646,7 +1646,7 @@
         <v>70</v>
       </c>
       <c r="N23" t="n">
-        <v>430</v>
+        <v>500</v>
       </c>
     </row>
     <row r="24">
@@ -1678,11 +1678,11 @@
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Camilla</t>
+          <t>Nanna</t>
         </is>
       </c>
       <c r="J24" t="n">
@@ -1698,7 +1698,7 @@
         <v>100</v>
       </c>
       <c r="N24" t="n">
-        <v>430</v>
+        <v>420</v>
       </c>
     </row>
     <row r="25">
@@ -1834,15 +1834,15 @@
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Bergur</t>
+          <t>Ólafur</t>
         </is>
       </c>
       <c r="J27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -1854,7 +1854,7 @@
         <v>80</v>
       </c>
       <c r="N27" t="n">
-        <v>500</v>
+        <v>440</v>
       </c>
     </row>
     <row r="28">
@@ -1886,11 +1886,11 @@
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J28" t="n">
@@ -1906,7 +1906,7 @@
         <v>90</v>
       </c>
       <c r="N28" t="n">
-        <v>490</v>
+        <v>480</v>
       </c>
     </row>
     <row r="29">
@@ -1938,18 +1938,18 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Össur</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K29" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L29" t="n">
         <v>3.5</v>
@@ -1958,7 +1958,7 @@
         <v>50</v>
       </c>
       <c r="N29" t="n">
-        <v>550</v>
+        <v>420</v>
       </c>
     </row>
     <row r="30">
@@ -1990,18 +1990,18 @@
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J30" t="n">
         <v>2</v>
       </c>
       <c r="K30" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L30" t="n">
         <v>3.5</v>
@@ -2010,7 +2010,7 @@
         <v>50</v>
       </c>
       <c r="N30" t="n">
-        <v>540</v>
+        <v>510</v>
       </c>
     </row>
     <row r="31">
@@ -2042,18 +2042,18 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K31" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L31" t="n">
         <v>3.5</v>
@@ -2062,7 +2062,7 @@
         <v>50</v>
       </c>
       <c r="N31" t="n">
-        <v>410</v>
+        <v>490</v>
       </c>
     </row>
     <row r="32">
@@ -2094,18 +2094,18 @@
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J32" t="n">
         <v>2</v>
       </c>
       <c r="K32" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L32" t="n">
         <v>3.5</v>
@@ -2114,7 +2114,7 @@
         <v>50</v>
       </c>
       <c r="N32" t="n">
-        <v>530</v>
+        <v>410</v>
       </c>
     </row>
     <row r="33">
@@ -2146,18 +2146,18 @@
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J33" t="n">
         <v>2</v>
       </c>
       <c r="K33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L33" t="n">
         <v>3.5</v>
@@ -2166,7 +2166,7 @@
         <v>50</v>
       </c>
       <c r="N33" t="n">
-        <v>390</v>
+        <v>430</v>
       </c>
     </row>
     <row r="34">
@@ -2198,18 +2198,18 @@
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K34" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L34" t="n">
         <v>3.5</v>
@@ -2218,7 +2218,7 @@
         <v>50</v>
       </c>
       <c r="N34" t="n">
-        <v>390</v>
+        <v>380</v>
       </c>
     </row>
     <row r="35">
@@ -2250,11 +2250,11 @@
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J35" t="n">
@@ -2270,7 +2270,7 @@
         <v>50</v>
       </c>
       <c r="N35" t="n">
-        <v>520</v>
+        <v>440</v>
       </c>
     </row>
     <row r="36">
@@ -2302,18 +2302,18 @@
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Camilla</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K36" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="L36" t="n">
         <v>3.5</v>
@@ -2322,7 +2322,7 @@
         <v>50</v>
       </c>
       <c r="N36" t="n">
-        <v>550</v>
+        <v>480</v>
       </c>
     </row>
     <row r="37">
@@ -2354,18 +2354,18 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Nanna</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K37" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L37" t="n">
         <v>3.5</v>
@@ -2374,7 +2374,7 @@
         <v>50</v>
       </c>
       <c r="N37" t="n">
-        <v>370</v>
+        <v>540</v>
       </c>
     </row>
     <row r="38">
@@ -2406,18 +2406,18 @@
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Bergur</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J38" t="n">
         <v>2</v>
       </c>
       <c r="K38" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L38" t="n">
         <v>3.5</v>
@@ -2426,7 +2426,7 @@
         <v>50</v>
       </c>
       <c r="N38" t="n">
-        <v>550</v>
+        <v>540</v>
       </c>
     </row>
     <row r="39">
@@ -2469,7 +2469,7 @@
         <v>1</v>
       </c>
       <c r="K39" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L39" t="n">
         <v>3.5</v>
@@ -2614,18 +2614,18 @@
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K42" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L42" t="n">
         <v>4</v>
@@ -2634,7 +2634,7 @@
         <v>50</v>
       </c>
       <c r="N42" t="n">
-        <v>560</v>
+        <v>330</v>
       </c>
     </row>
     <row r="43">
@@ -2666,18 +2666,18 @@
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J43" t="n">
         <v>2</v>
       </c>
       <c r="K43" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L43" t="n">
         <v>4</v>
@@ -2718,18 +2718,18 @@
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K44" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="L44" t="n">
         <v>4</v>
@@ -2738,7 +2738,7 @@
         <v>50</v>
       </c>
       <c r="N44" t="n">
-        <v>330</v>
+        <v>510</v>
       </c>
     </row>
     <row r="45">
@@ -2781,7 +2781,7 @@
         <v>1</v>
       </c>
       <c r="K45" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="L45" t="n">
         <v>4</v>
@@ -2790,7 +2790,7 @@
         <v>50</v>
       </c>
       <c r="N45" t="n">
-        <v>560</v>
+        <v>490</v>
       </c>
     </row>
     <row r="46">
@@ -2937,7 +2937,7 @@
         <v>1</v>
       </c>
       <c r="K48" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L48" t="n">
         <v>4</v>
@@ -2946,7 +2946,7 @@
         <v>50</v>
       </c>
       <c r="N48" t="n">
-        <v>550</v>
+        <v>490</v>
       </c>
     </row>
     <row r="49">
@@ -2989,7 +2989,7 @@
         <v>1</v>
       </c>
       <c r="K49" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L49" t="n">
         <v>4</v>
@@ -2998,7 +2998,7 @@
         <v>50</v>
       </c>
       <c r="N49" t="n">
-        <v>560</v>
+        <v>510</v>
       </c>
     </row>
     <row r="50">
@@ -3082,11 +3082,11 @@
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Camilla</t>
         </is>
       </c>
       <c r="J51" t="n">
@@ -3154,7 +3154,7 @@
         <v>50</v>
       </c>
       <c r="N52" t="n">
-        <v>390</v>
+        <v>490</v>
       </c>
     </row>
     <row r="53">
@@ -3186,18 +3186,18 @@
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Thelma</t>
+          <t>Össur</t>
         </is>
       </c>
       <c r="J53" t="n">
         <v>3</v>
       </c>
       <c r="K53" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="L53" t="n">
         <v>4</v>
@@ -3206,7 +3206,7 @@
         <v>50</v>
       </c>
       <c r="N53" t="n">
-        <v>580</v>
+        <v>540</v>
       </c>
     </row>
     <row r="54">
@@ -3238,11 +3238,11 @@
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J54" t="n">
@@ -3258,7 +3258,7 @@
         <v>50</v>
       </c>
       <c r="N54" t="n">
-        <v>380</v>
+        <v>370</v>
       </c>
     </row>
     <row r="55">
@@ -3290,18 +3290,18 @@
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J55" t="n">
         <v>2</v>
       </c>
       <c r="K55" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L55" t="n">
         <v>4</v>
@@ -3310,7 +3310,7 @@
         <v>50</v>
       </c>
       <c r="N55" t="n">
-        <v>390</v>
+        <v>560</v>
       </c>
     </row>
     <row r="56">
@@ -3342,18 +3342,18 @@
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J56" t="n">
         <v>2</v>
       </c>
       <c r="K56" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L56" t="n">
         <v>4</v>
@@ -3394,18 +3394,18 @@
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J57" t="n">
         <v>2</v>
       </c>
       <c r="K57" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L57" t="n">
         <v>4</v>
@@ -3414,7 +3414,7 @@
         <v>50</v>
       </c>
       <c r="N57" t="n">
-        <v>580</v>
+        <v>390</v>
       </c>
     </row>
     <row r="58">
@@ -3498,18 +3498,18 @@
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J59" t="n">
         <v>2</v>
       </c>
       <c r="K59" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="L59" t="n">
         <v>4</v>
@@ -3518,7 +3518,7 @@
         <v>50</v>
       </c>
       <c r="N59" t="n">
-        <v>390</v>
+        <v>560</v>
       </c>
     </row>
     <row r="60">
@@ -3550,18 +3550,18 @@
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J60" t="n">
         <v>2</v>
       </c>
       <c r="K60" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L60" t="n">
         <v>4</v>
@@ -3570,7 +3570,7 @@
         <v>50</v>
       </c>
       <c r="N60" t="n">
-        <v>570</v>
+        <v>390</v>
       </c>
     </row>
     <row r="61">
@@ -3706,11 +3706,11 @@
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J63" t="n">
@@ -3726,7 +3726,7 @@
         <v>80</v>
       </c>
       <c r="N63" t="n">
-        <v>440</v>
+        <v>450</v>
       </c>
     </row>
     <row r="64">
@@ -4018,15 +4018,15 @@
       </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K69" t="n">
         <v>0</v>
@@ -4070,11 +4070,11 @@
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J70" t="n">
@@ -4090,7 +4090,7 @@
         <v>100</v>
       </c>
       <c r="N70" t="n">
-        <v>480</v>
+        <v>490</v>
       </c>
     </row>
     <row r="71">
@@ -4122,11 +4122,11 @@
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Pétur</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J71" t="n">
@@ -4142,7 +4142,7 @@
         <v>100</v>
       </c>
       <c r="N71" t="n">
-        <v>480</v>
+        <v>490</v>
       </c>
     </row>
     <row r="72">
@@ -4185,7 +4185,7 @@
         <v>3</v>
       </c>
       <c r="K72" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="L72" t="n">
         <v>3.5</v>
@@ -4194,7 +4194,7 @@
         <v>50</v>
       </c>
       <c r="N72" t="n">
-        <v>540</v>
+        <v>470</v>
       </c>
     </row>
     <row r="73">
@@ -4237,7 +4237,7 @@
         <v>3</v>
       </c>
       <c r="K73" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="L73" t="n">
         <v>3.5</v>
@@ -4246,7 +4246,7 @@
         <v>50</v>
       </c>
       <c r="N73" t="n">
-        <v>510</v>
+        <v>540</v>
       </c>
     </row>
     <row r="74">
@@ -4289,7 +4289,7 @@
         <v>3</v>
       </c>
       <c r="K74" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L74" t="n">
         <v>3.5</v>
@@ -4330,11 +4330,11 @@
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J75" t="n">
@@ -4350,7 +4350,7 @@
         <v>50</v>
       </c>
       <c r="N75" t="n">
-        <v>510</v>
+        <v>530</v>
       </c>
     </row>
     <row r="76">
@@ -4382,18 +4382,18 @@
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J76" t="n">
         <v>2</v>
       </c>
       <c r="K76" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L76" t="n">
         <v>3.5</v>
@@ -4402,7 +4402,7 @@
         <v>50</v>
       </c>
       <c r="N76" t="n">
-        <v>530</v>
+        <v>380</v>
       </c>
     </row>
     <row r="77">
@@ -4434,11 +4434,11 @@
       </c>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J77" t="n">
@@ -4454,7 +4454,7 @@
         <v>50</v>
       </c>
       <c r="N77" t="n">
-        <v>400</v>
+        <v>380</v>
       </c>
     </row>
     <row r="78">
@@ -4486,18 +4486,18 @@
       </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K78" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L78" t="n">
         <v>3.5</v>
@@ -4506,7 +4506,7 @@
         <v>50</v>
       </c>
       <c r="N78" t="n">
-        <v>390</v>
+        <v>540</v>
       </c>
     </row>
     <row r="79">
@@ -4538,18 +4538,18 @@
       </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J79" t="n">
         <v>2</v>
       </c>
       <c r="K79" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L79" t="n">
         <v>3.5</v>
@@ -4558,7 +4558,7 @@
         <v>50</v>
       </c>
       <c r="N79" t="n">
-        <v>520</v>
+        <v>380</v>
       </c>
     </row>
     <row r="80">
@@ -4590,18 +4590,18 @@
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K80" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L80" t="n">
         <v>3.5</v>
@@ -4610,7 +4610,7 @@
         <v>50</v>
       </c>
       <c r="N80" t="n">
-        <v>520</v>
+        <v>370</v>
       </c>
     </row>
     <row r="81">
@@ -4642,18 +4642,18 @@
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Nanna</t>
         </is>
       </c>
       <c r="J81" t="n">
         <v>1</v>
       </c>
       <c r="K81" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L81" t="n">
         <v>3.5</v>
@@ -4662,7 +4662,7 @@
         <v>50</v>
       </c>
       <c r="N81" t="n">
-        <v>370</v>
+        <v>540</v>
       </c>
     </row>
     <row r="82">
@@ -4694,18 +4694,18 @@
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Bergur</t>
+          <t>Ólafur</t>
         </is>
       </c>
       <c r="J82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K82" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L82" t="n">
         <v>3.5</v>
@@ -4714,7 +4714,7 @@
         <v>50</v>
       </c>
       <c r="N82" t="n">
-        <v>420</v>
+        <v>540</v>
       </c>
     </row>
     <row r="83">
@@ -4798,18 +4798,18 @@
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Pétur</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J84" t="n">
         <v>2</v>
       </c>
       <c r="K84" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L84" t="n">
         <v>4</v>
@@ -4818,7 +4818,7 @@
         <v>50</v>
       </c>
       <c r="N84" t="n">
-        <v>380</v>
+        <v>390</v>
       </c>
     </row>
     <row r="85">
@@ -4850,18 +4850,18 @@
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
+        <v>11</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Oliver</t>
+        </is>
+      </c>
+      <c r="J85" t="n">
+        <v>2</v>
+      </c>
+      <c r="K85" t="n">
         <v>9</v>
-      </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>Freyja</t>
-        </is>
-      </c>
-      <c r="J85" t="n">
-        <v>2</v>
-      </c>
-      <c r="K85" t="n">
-        <v>6</v>
       </c>
       <c r="L85" t="n">
         <v>4</v>
@@ -4870,7 +4870,7 @@
         <v>50</v>
       </c>
       <c r="N85" t="n">
-        <v>390</v>
+        <v>560</v>
       </c>
     </row>
     <row r="86">
@@ -4902,18 +4902,18 @@
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J86" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K86" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L86" t="n">
         <v>4</v>
@@ -4922,7 +4922,7 @@
         <v>50</v>
       </c>
       <c r="N86" t="n">
-        <v>560</v>
+        <v>540</v>
       </c>
     </row>
     <row r="87">
@@ -4954,18 +4954,18 @@
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J87" t="n">
         <v>2</v>
       </c>
       <c r="K87" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L87" t="n">
         <v>4</v>
@@ -4974,7 +4974,7 @@
         <v>50</v>
       </c>
       <c r="N87" t="n">
-        <v>380</v>
+        <v>400</v>
       </c>
     </row>
     <row r="88">
@@ -5006,18 +5006,18 @@
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J88" t="n">
         <v>2</v>
       </c>
       <c r="K88" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L88" t="n">
         <v>4</v>
@@ -5026,7 +5026,7 @@
         <v>50</v>
       </c>
       <c r="N88" t="n">
-        <v>380</v>
+        <v>390</v>
       </c>
     </row>
     <row r="89">
@@ -5058,18 +5058,18 @@
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J89" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K89" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L89" t="n">
         <v>4</v>
@@ -5078,7 +5078,7 @@
         <v>50</v>
       </c>
       <c r="N89" t="n">
-        <v>560</v>
+        <v>390</v>
       </c>
     </row>
     <row r="90">
@@ -5110,18 +5110,18 @@
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J90" t="n">
         <v>2</v>
       </c>
       <c r="K90" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L90" t="n">
         <v>4</v>
@@ -5130,7 +5130,7 @@
         <v>50</v>
       </c>
       <c r="N90" t="n">
-        <v>540</v>
+        <v>390</v>
       </c>
     </row>
     <row r="91">
@@ -5162,15 +5162,15 @@
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J91" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K91" t="n">
         <v>10</v>
@@ -5214,18 +5214,18 @@
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Camilla</t>
         </is>
       </c>
       <c r="J92" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K92" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L92" t="n">
         <v>4</v>
@@ -5234,7 +5234,7 @@
         <v>50</v>
       </c>
       <c r="N92" t="n">
-        <v>380</v>
+        <v>330</v>
       </c>
     </row>
     <row r="93">
@@ -5266,18 +5266,18 @@
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>Camilla</t>
+          <t>Anna</t>
         </is>
       </c>
       <c r="J93" t="n">
         <v>1</v>
       </c>
       <c r="K93" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L93" t="n">
         <v>4</v>
@@ -5286,7 +5286,7 @@
         <v>50</v>
       </c>
       <c r="N93" t="n">
-        <v>330</v>
+        <v>560</v>
       </c>
     </row>
     <row r="94">
@@ -5329,7 +5329,7 @@
         <v>2</v>
       </c>
       <c r="K94" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L94" t="n">
         <v>4</v>
@@ -5338,7 +5338,7 @@
         <v>50</v>
       </c>
       <c r="N94" t="n">
-        <v>370</v>
+        <v>410</v>
       </c>
     </row>
     <row r="95">
@@ -5370,15 +5370,15 @@
       </c>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="n">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>Anna</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J95" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K95" t="n">
         <v>0</v>
@@ -5390,7 +5390,7 @@
         <v>80</v>
       </c>
       <c r="N95" t="n">
-        <v>440</v>
+        <v>460</v>
       </c>
     </row>
     <row r="96">
@@ -5526,18 +5526,18 @@
       </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>Ásdís</t>
+          <t>Össur</t>
         </is>
       </c>
       <c r="J98" t="n">
         <v>3</v>
       </c>
       <c r="K98" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L98" t="n">
         <v>3</v>
@@ -5578,18 +5578,18 @@
       </c>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>Helgi</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J99" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K99" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="L99" t="n">
         <v>3</v>
@@ -5598,7 +5598,7 @@
         <v>70</v>
       </c>
       <c r="N99" t="n">
-        <v>460</v>
+        <v>540</v>
       </c>
     </row>
     <row r="100">
@@ -5630,18 +5630,18 @@
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J100" t="n">
         <v>2</v>
       </c>
       <c r="K100" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="L100" t="n">
         <v>3</v>
@@ -5650,7 +5650,7 @@
         <v>70</v>
       </c>
       <c r="N100" t="n">
-        <v>530</v>
+        <v>490</v>
       </c>
     </row>
     <row r="101">
@@ -5682,11 +5682,11 @@
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J101" t="n">
@@ -5702,7 +5702,7 @@
         <v>70</v>
       </c>
       <c r="N101" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
     </row>
     <row r="102">
@@ -5734,18 +5734,18 @@
       </c>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J102" t="n">
         <v>2</v>
       </c>
       <c r="K102" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L102" t="n">
         <v>3</v>
@@ -5754,7 +5754,7 @@
         <v>70</v>
       </c>
       <c r="N102" t="n">
-        <v>460</v>
+        <v>380</v>
       </c>
     </row>
     <row r="103">
@@ -5786,18 +5786,18 @@
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J103" t="n">
         <v>2</v>
       </c>
       <c r="K103" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L103" t="n">
         <v>3</v>
@@ -5806,7 +5806,7 @@
         <v>70</v>
       </c>
       <c r="N103" t="n">
-        <v>380</v>
+        <v>360</v>
       </c>
     </row>
     <row r="104">
@@ -5838,18 +5838,18 @@
       </c>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J104" t="n">
         <v>2</v>
       </c>
       <c r="K104" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L104" t="n">
         <v>3</v>
@@ -5858,7 +5858,7 @@
         <v>70</v>
       </c>
       <c r="N104" t="n">
-        <v>360</v>
+        <v>510</v>
       </c>
     </row>
     <row r="105">
@@ -5890,18 +5890,18 @@
       </c>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K105" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L105" t="n">
         <v>3</v>
@@ -5910,7 +5910,7 @@
         <v>70</v>
       </c>
       <c r="N105" t="n">
-        <v>500</v>
+        <v>540</v>
       </c>
     </row>
     <row r="106">
@@ -5942,18 +5942,18 @@
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Ólafur</t>
         </is>
       </c>
       <c r="J106" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K106" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L106" t="n">
         <v>3</v>
@@ -5962,7 +5962,7 @@
         <v>70</v>
       </c>
       <c r="N106" t="n">
-        <v>530</v>
+        <v>360</v>
       </c>
     </row>
     <row r="107">
@@ -5994,18 +5994,18 @@
       </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>Ólafur</t>
+          <t>Bergur</t>
         </is>
       </c>
       <c r="J107" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K107" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L107" t="n">
         <v>3</v>
@@ -6014,7 +6014,7 @@
         <v>70</v>
       </c>
       <c r="N107" t="n">
-        <v>360</v>
+        <v>480</v>
       </c>
     </row>
     <row r="108">
@@ -6057,7 +6057,7 @@
         <v>1</v>
       </c>
       <c r="K108" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L108" t="n">
         <v>3</v>
@@ -6098,11 +6098,11 @@
       </c>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J109" t="n">
@@ -6118,7 +6118,7 @@
         <v>90</v>
       </c>
       <c r="N109" t="n">
-        <v>480</v>
+        <v>470</v>
       </c>
     </row>
     <row r="110">
@@ -6150,11 +6150,11 @@
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J110" t="n">
@@ -6170,7 +6170,7 @@
         <v>100</v>
       </c>
       <c r="N110" t="n">
-        <v>490</v>
+        <v>470</v>
       </c>
     </row>
     <row r="111">
@@ -6202,11 +6202,11 @@
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J111" t="n">
@@ -6222,7 +6222,7 @@
         <v>100</v>
       </c>
       <c r="N111" t="n">
-        <v>470</v>
+        <v>460</v>
       </c>
     </row>
     <row r="112">
@@ -6254,11 +6254,11 @@
       </c>
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Nanna</t>
+          <t>Anna</t>
         </is>
       </c>
       <c r="J112" t="n">
@@ -6274,7 +6274,7 @@
         <v>100</v>
       </c>
       <c r="N112" t="n">
-        <v>470</v>
+        <v>460</v>
       </c>
     </row>
     <row r="113">
@@ -6306,18 +6306,18 @@
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>Össur</t>
+          <t>Ásdís</t>
         </is>
       </c>
       <c r="J113" t="n">
         <v>3</v>
       </c>
       <c r="K113" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L113" t="n">
         <v>4</v>
@@ -6326,7 +6326,7 @@
         <v>70</v>
       </c>
       <c r="N113" t="n">
-        <v>500</v>
+        <v>540</v>
       </c>
     </row>
     <row r="114">
@@ -6369,7 +6369,7 @@
         <v>3</v>
       </c>
       <c r="K114" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L114" t="n">
         <v>4</v>
@@ -6430,7 +6430,7 @@
         <v>70</v>
       </c>
       <c r="N115" t="n">
-        <v>450</v>
+        <v>400</v>
       </c>
     </row>
     <row r="116">
@@ -6473,7 +6473,7 @@
         <v>2</v>
       </c>
       <c r="K116" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="L116" t="n">
         <v>4</v>
@@ -6482,7 +6482,7 @@
         <v>70</v>
       </c>
       <c r="N116" t="n">
-        <v>460</v>
+        <v>550</v>
       </c>
     </row>
     <row r="117">
@@ -6514,18 +6514,18 @@
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J117" t="n">
         <v>2</v>
       </c>
       <c r="K117" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L117" t="n">
         <v>4</v>
@@ -6534,7 +6534,7 @@
         <v>70</v>
       </c>
       <c r="N117" t="n">
-        <v>340</v>
+        <v>540</v>
       </c>
     </row>
     <row r="118">
@@ -6566,18 +6566,18 @@
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J118" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K118" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L118" t="n">
         <v>4</v>
@@ -6586,7 +6586,7 @@
         <v>70</v>
       </c>
       <c r="N118" t="n">
-        <v>510</v>
+        <v>540</v>
       </c>
     </row>
     <row r="119">
@@ -6618,18 +6618,18 @@
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J119" t="n">
         <v>2</v>
       </c>
       <c r="K119" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="L119" t="n">
         <v>4</v>
@@ -6638,7 +6638,7 @@
         <v>70</v>
       </c>
       <c r="N119" t="n">
-        <v>340</v>
+        <v>540</v>
       </c>
     </row>
     <row r="120">
@@ -6670,18 +6670,18 @@
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K120" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L120" t="n">
         <v>4</v>
@@ -6722,18 +6722,18 @@
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Camilla</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J121" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K121" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L121" t="n">
         <v>4</v>
@@ -6742,7 +6742,7 @@
         <v>70</v>
       </c>
       <c r="N121" t="n">
-        <v>500</v>
+        <v>340</v>
       </c>
     </row>
     <row r="122">
@@ -6774,18 +6774,18 @@
       </c>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>Ólafur</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J122" t="n">
         <v>1</v>
       </c>
       <c r="K122" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L122" t="n">
         <v>4</v>
@@ -6794,7 +6794,7 @@
         <v>70</v>
       </c>
       <c r="N122" t="n">
-        <v>500</v>
+        <v>340</v>
       </c>
     </row>
     <row r="123">
@@ -6826,18 +6826,18 @@
       </c>
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>Anna</t>
+          <t>Nanna</t>
         </is>
       </c>
       <c r="J123" t="n">
         <v>1</v>
       </c>
       <c r="K123" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L123" t="n">
         <v>4</v>
@@ -6846,7 +6846,7 @@
         <v>70</v>
       </c>
       <c r="N123" t="n">
-        <v>510</v>
+        <v>490</v>
       </c>
     </row>
     <row r="124">
@@ -6878,18 +6878,18 @@
       </c>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Pétur</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J124" t="n">
         <v>2</v>
       </c>
       <c r="K124" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L124" t="n">
         <v>2</v>
@@ -6898,7 +6898,7 @@
         <v>70</v>
       </c>
       <c r="N124" t="n">
-        <v>550</v>
+        <v>560</v>
       </c>
     </row>
     <row r="125">
@@ -6930,18 +6930,18 @@
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J125" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K125" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L125" t="n">
         <v>2</v>
@@ -6950,7 +6950,7 @@
         <v>70</v>
       </c>
       <c r="N125" t="n">
-        <v>520</v>
+        <v>340</v>
       </c>
     </row>
     <row r="126">
@@ -6982,18 +6982,18 @@
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J126" t="n">
         <v>2</v>
       </c>
       <c r="K126" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L126" t="n">
         <v>2</v>
@@ -7002,7 +7002,7 @@
         <v>70</v>
       </c>
       <c r="N126" t="n">
-        <v>550</v>
+        <v>570</v>
       </c>
     </row>
     <row r="127">
@@ -7034,18 +7034,18 @@
       </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K127" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L127" t="n">
         <v>2</v>
@@ -7054,7 +7054,7 @@
         <v>70</v>
       </c>
       <c r="N127" t="n">
-        <v>340</v>
+        <v>540</v>
       </c>
     </row>
     <row r="128">
@@ -7086,15 +7086,15 @@
       </c>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J128" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K128" t="n">
         <v>10</v>
@@ -7106,7 +7106,7 @@
         <v>70</v>
       </c>
       <c r="N128" t="n">
-        <v>550</v>
+        <v>580</v>
       </c>
     </row>
     <row r="129">
@@ -7138,15 +7138,15 @@
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J129" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K129" t="n">
         <v>4</v>
@@ -7158,7 +7158,7 @@
         <v>70</v>
       </c>
       <c r="N129" t="n">
-        <v>540</v>
+        <v>550</v>
       </c>
     </row>
     <row r="130">
@@ -7190,18 +7190,18 @@
       </c>
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J130" t="n">
         <v>2</v>
       </c>
       <c r="K130" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L130" t="n">
         <v>2</v>
@@ -7346,18 +7346,18 @@
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Camilla</t>
         </is>
       </c>
       <c r="J133" t="n">
         <v>1</v>
       </c>
       <c r="K133" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="L133" t="n">
         <v>2</v>
@@ -7366,7 +7366,7 @@
         <v>70</v>
       </c>
       <c r="N133" t="n">
-        <v>540</v>
+        <v>570</v>
       </c>
     </row>
     <row r="134">
@@ -7398,18 +7398,18 @@
       </c>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Nanna</t>
+          <t>Bergur</t>
         </is>
       </c>
       <c r="J134" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K134" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L134" t="n">
         <v>2</v>
@@ -7418,7 +7418,7 @@
         <v>70</v>
       </c>
       <c r="N134" t="n">
-        <v>540</v>
+        <v>550</v>
       </c>
     </row>
     <row r="135">
@@ -7502,18 +7502,18 @@
       </c>
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Helgi</t>
         </is>
       </c>
       <c r="J136" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K136" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L136" t="n">
         <v>4</v>
@@ -7554,18 +7554,18 @@
       </c>
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J137" t="n">
         <v>1</v>
       </c>
       <c r="K137" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L137" t="n">
         <v>4</v>
@@ -7782,14 +7782,14 @@
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
-      <c r="U2" t="n">
-        <v>1</v>
-      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
+      <c r="Z2" t="n">
+        <v>1</v>
+      </c>
       <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
@@ -7803,9 +7803,7 @@
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
-      <c r="D3" t="n">
-        <v>1</v>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
         <v>1</v>
       </c>
@@ -7828,9 +7826,7 @@
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="n">
-        <v>1</v>
-      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr"/>
@@ -7841,27 +7837,29 @@
       <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="inlineStr"/>
       <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
+      <c r="AF3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="n">
-        <v>1</v>
-      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" t="n">
-        <v>1</v>
-      </c>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
@@ -7872,14 +7870,14 @@
       <c r="T4" t="n">
         <v>1</v>
       </c>
-      <c r="U4" t="inlineStr"/>
+      <c r="U4" t="n">
+        <v>1</v>
+      </c>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="n">
-        <v>1</v>
-      </c>
+      <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="inlineStr"/>
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
@@ -7903,9 +7901,7 @@
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="n">
-        <v>1</v>
-      </c>
+      <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
         <v>1</v>
       </c>
@@ -7937,7 +7933,9 @@
       <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
@@ -7952,25 +7950,23 @@
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
-      <c r="O6" t="n">
-        <v>1</v>
-      </c>
+      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
-      <c r="S6" t="n">
-        <v>1</v>
-      </c>
+      <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
+      <c r="U6" t="n">
+        <v>1</v>
+      </c>
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
+      <c r="Y6" t="n">
+        <v>1</v>
+      </c>
       <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="n">
-        <v>1</v>
-      </c>
+      <c r="AA6" t="inlineStr"/>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="inlineStr"/>
@@ -7981,25 +7977,21 @@
       <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="n">
-        <v>1</v>
-      </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
-      <c r="D7" t="n">
-        <v>1</v>
-      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="n">
-        <v>1</v>
-      </c>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="n">
         <v>1</v>
       </c>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
@@ -8010,13 +8002,17 @@
       <c r="T7" t="n">
         <v>1</v>
       </c>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" t="n">
+        <v>1</v>
+      </c>
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr"/>
+      <c r="AA7" t="n">
+        <v>1</v>
+      </c>
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr"/>
@@ -8029,8 +8025,12 @@
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
@@ -8058,9 +8058,7 @@
       <c r="Z8" t="n">
         <v>1</v>
       </c>
-      <c r="AA8" t="n">
-        <v>1</v>
-      </c>
+      <c r="AA8" t="inlineStr"/>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr"/>
@@ -8080,7 +8078,9 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="n">
+        <v>1</v>
+      </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
@@ -8094,9 +8094,7 @@
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
-      <c r="U9" t="n">
-        <v>1</v>
-      </c>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr"/>
@@ -8115,12 +8113,12 @@
       <c r="A10" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
-      <c r="E10" t="n">
-        <v>1</v>
-      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
@@ -8140,14 +8138,14 @@
         <v>1</v>
       </c>
       <c r="T10" t="inlineStr"/>
-      <c r="U10" t="n">
-        <v>1</v>
-      </c>
+      <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr"/>
-      <c r="Z10" t="inlineStr"/>
+      <c r="Z10" t="n">
+        <v>1</v>
+      </c>
       <c r="AA10" t="inlineStr"/>
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
@@ -8160,7 +8158,9 @@
         <v>10</v>
       </c>
       <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
@@ -8178,13 +8178,9 @@
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
-      <c r="S11" t="n">
-        <v>1</v>
-      </c>
+      <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="n">
         <v>1</v>
@@ -8205,9 +8201,7 @@
       <c r="A12" t="n">
         <v>11</v>
       </c>
-      <c r="B12" t="n">
-        <v>1</v>
-      </c>
+      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
@@ -8215,7 +8209,9 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
       <c r="K12" t="n">
         <v>1</v>
       </c>
@@ -8226,8 +8222,12 @@
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
-      <c r="T12" t="inlineStr"/>
+      <c r="S12" t="n">
+        <v>1</v>
+      </c>
+      <c r="T12" t="n">
+        <v>1</v>
+      </c>
       <c r="U12" t="n">
         <v>1</v>
       </c>
@@ -8236,9 +8236,7 @@
       <c r="X12" t="inlineStr"/>
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="inlineStr"/>
-      <c r="AA12" t="n">
-        <v>1</v>
-      </c>
+      <c r="AA12" t="inlineStr"/>
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr"/>
       <c r="AD12" t="inlineStr"/>
@@ -8252,17 +8250,15 @@
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
-      <c r="E13" t="n">
-        <v>1</v>
-      </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="n">
-        <v>1</v>
-      </c>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
@@ -8270,7 +8266,9 @@
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr"/>
+      <c r="S13" t="n">
+        <v>1</v>
+      </c>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr"/>
@@ -8307,9 +8305,7 @@
         <v>1</v>
       </c>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" t="n">
-        <v>1</v>
-      </c>
+      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
@@ -8342,27 +8338,29 @@
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
+      <c r="J15" t="n">
+        <v>1</v>
+      </c>
       <c r="K15" t="n">
         <v>1</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" t="n">
-        <v>1</v>
-      </c>
+      <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
+      <c r="Q15" t="n">
+        <v>1</v>
+      </c>
       <c r="R15" t="inlineStr"/>
-      <c r="S15" t="n">
-        <v>1</v>
-      </c>
+      <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr"/>
@@ -8391,31 +8389,31 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" t="n">
-        <v>1</v>
-      </c>
+      <c r="J16" t="inlineStr"/>
       <c r="K16" t="n">
         <v>1</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="n">
-        <v>1</v>
-      </c>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
+      <c r="Q16" t="n">
+        <v>1</v>
+      </c>
       <c r="R16" t="inlineStr"/>
-      <c r="S16" t="n">
-        <v>1</v>
-      </c>
+      <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
+      <c r="X16" t="n">
+        <v>1</v>
+      </c>
       <c r="Y16" t="inlineStr"/>
-      <c r="Z16" t="inlineStr"/>
+      <c r="Z16" t="n">
+        <v>1</v>
+      </c>
       <c r="AA16" t="inlineStr"/>
       <c r="AB16" t="inlineStr"/>
       <c r="AC16" t="inlineStr"/>
@@ -8446,21 +8444,21 @@
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
+      <c r="S17" t="n">
+        <v>1</v>
+      </c>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr"/>
       <c r="X17" t="inlineStr"/>
       <c r="Y17" t="inlineStr"/>
-      <c r="Z17" t="inlineStr"/>
-      <c r="AA17" t="n">
-        <v>1</v>
-      </c>
+      <c r="Z17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA17" t="inlineStr"/>
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="inlineStr"/>
@@ -8472,7 +8470,9 @@
         <v>17</v>
       </c>
       <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
@@ -8486,18 +8486,16 @@
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
+      <c r="S18" t="n">
+        <v>1</v>
+      </c>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr"/>
       <c r="W18" t="inlineStr"/>
-      <c r="X18" t="n">
-        <v>1</v>
-      </c>
+      <c r="X18" t="inlineStr"/>
       <c r="Y18" t="inlineStr"/>
       <c r="Z18" t="n">
         <v>1</v>
@@ -8526,29 +8524,29 @@
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="K19" t="n">
+        <v>1</v>
+      </c>
       <c r="L19" t="inlineStr"/>
-      <c r="M19" t="n">
-        <v>1</v>
-      </c>
+      <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
-      <c r="S19" t="n">
-        <v>1</v>
-      </c>
+      <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr"/>
       <c r="X19" t="inlineStr"/>
-      <c r="Y19" t="inlineStr"/>
-      <c r="Z19" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA19" t="inlineStr"/>
+      <c r="Y19" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z19" t="inlineStr"/>
+      <c r="AA19" t="n">
+        <v>1</v>
+      </c>
       <c r="AB19" t="inlineStr"/>
       <c r="AC19" t="inlineStr"/>
       <c r="AD19" t="inlineStr"/>
@@ -8559,9 +8557,7 @@
       <c r="A20" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="n">
-        <v>1</v>
-      </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
@@ -8571,28 +8567,30 @@
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
+      <c r="J20" t="n">
+        <v>1</v>
+      </c>
       <c r="K20" t="inlineStr"/>
-      <c r="L20" t="n">
-        <v>1</v>
-      </c>
+      <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
+      <c r="N20" t="n">
+        <v>1</v>
+      </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr"/>
-      <c r="U20" t="n">
-        <v>1</v>
-      </c>
+      <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr"/>
       <c r="X20" t="inlineStr"/>
       <c r="Y20" t="inlineStr"/>
       <c r="Z20" t="inlineStr"/>
-      <c r="AA20" t="inlineStr"/>
+      <c r="AA20" t="n">
+        <v>1</v>
+      </c>
       <c r="AB20" t="inlineStr"/>
       <c r="AC20" t="inlineStr"/>
       <c r="AD20" t="inlineStr"/>
@@ -8617,7 +8615,9 @@
         <v>1</v>
       </c>
       <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
+      <c r="L21" t="n">
+        <v>1</v>
+      </c>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
@@ -8628,13 +8628,13 @@
         <v>1</v>
       </c>
       <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
+      <c r="U21" t="n">
+        <v>1</v>
+      </c>
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
       <c r="X21" t="inlineStr"/>
-      <c r="Y21" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y21" t="inlineStr"/>
       <c r="Z21" t="inlineStr"/>
       <c r="AA21" t="inlineStr"/>
       <c r="AB21" t="inlineStr"/>
@@ -8647,12 +8647,12 @@
       <c r="A22" t="n">
         <v>21</v>
       </c>
-      <c r="B22" t="inlineStr"/>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="n">
-        <v>1</v>
-      </c>
+      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
@@ -8668,11 +8668,11 @@
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
+      <c r="S22" t="n">
+        <v>1</v>
+      </c>
       <c r="T22" t="inlineStr"/>
-      <c r="U22" t="n">
-        <v>1</v>
-      </c>
+      <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr"/>
       <c r="X22" t="inlineStr"/>
@@ -8680,7 +8680,9 @@
       <c r="Z22" t="n">
         <v>1</v>
       </c>
-      <c r="AA22" t="inlineStr"/>
+      <c r="AA22" t="n">
+        <v>1</v>
+      </c>
       <c r="AB22" t="inlineStr"/>
       <c r="AC22" t="inlineStr"/>
       <c r="AD22" t="inlineStr"/>
@@ -8691,12 +8693,12 @@
       <c r="A23" t="n">
         <v>22</v>
       </c>
-      <c r="B23" t="inlineStr"/>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="n">
-        <v>1</v>
-      </c>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
@@ -8710,7 +8712,9 @@
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
+      <c r="Q23" t="n">
+        <v>1</v>
+      </c>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr"/>
@@ -8727,40 +8731,36 @@
       <c r="AC23" t="inlineStr"/>
       <c r="AD23" t="inlineStr"/>
       <c r="AE23" t="inlineStr"/>
-      <c r="AF23" t="n">
-        <v>1</v>
-      </c>
+      <c r="AF23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
         <v>23</v>
       </c>
       <c r="B24" t="inlineStr"/>
-      <c r="C24" t="n">
-        <v>1</v>
-      </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
+      <c r="J24" t="n">
+        <v>1</v>
+      </c>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="n">
         <v>1</v>
       </c>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
+      <c r="N24" t="n">
+        <v>1</v>
+      </c>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
-      <c r="S24" t="n">
-        <v>1</v>
-      </c>
+      <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr"/>
@@ -8789,26 +8789,24 @@
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" t="n">
-        <v>1</v>
-      </c>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="n">
         <v>1</v>
       </c>
-      <c r="L25" t="n">
-        <v>1</v>
-      </c>
+      <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
+      <c r="Q25" t="n">
+        <v>1</v>
+      </c>
       <c r="R25" t="inlineStr"/>
-      <c r="S25" t="n">
-        <v>1</v>
-      </c>
+      <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
+      <c r="U25" t="n">
+        <v>1</v>
+      </c>
       <c r="V25" t="inlineStr"/>
       <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr"/>
@@ -8828,27 +8826,27 @@
         <v>25</v>
       </c>
       <c r="B26" t="inlineStr"/>
-      <c r="C26" t="n">
-        <v>1</v>
-      </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
+      <c r="J26" t="n">
+        <v>1</v>
+      </c>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="n">
         <v>1</v>
       </c>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
+      <c r="O26" t="n">
+        <v>1</v>
+      </c>
       <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr"/>
@@ -8874,7 +8872,9 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
@@ -8884,7 +8884,9 @@
         <v>1</v>
       </c>
       <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
+      <c r="M27" t="n">
+        <v>1</v>
+      </c>
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
@@ -8892,19 +8894,17 @@
         <v>1</v>
       </c>
       <c r="R27" t="inlineStr"/>
-      <c r="S27" t="inlineStr"/>
+      <c r="S27" t="n">
+        <v>1</v>
+      </c>
       <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr"/>
-      <c r="Y27" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y27" t="inlineStr"/>
       <c r="Z27" t="inlineStr"/>
-      <c r="AA27" t="n">
-        <v>1</v>
-      </c>
+      <c r="AA27" t="inlineStr"/>
       <c r="AB27" t="inlineStr"/>
       <c r="AC27" t="inlineStr"/>
       <c r="AD27" t="inlineStr"/>
@@ -8925,11 +8925,11 @@
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" t="n">
-        <v>1</v>
-      </c>
+      <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
+      <c r="L28" t="n">
+        <v>1</v>
+      </c>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr"/>
@@ -8945,10 +8945,10 @@
       <c r="W28" t="inlineStr"/>
       <c r="X28" t="inlineStr"/>
       <c r="Y28" t="inlineStr"/>
-      <c r="Z28" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="n">
+        <v>1</v>
+      </c>
       <c r="AB28" t="inlineStr"/>
       <c r="AC28" t="inlineStr"/>
       <c r="AD28" t="inlineStr"/>
@@ -8962,14 +8962,14 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" t="n">
-        <v>1</v>
-      </c>
+      <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="n">
         <v>1</v>
@@ -8978,7 +8978,9 @@
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
+      <c r="Q29" t="n">
+        <v>1</v>
+      </c>
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr"/>
@@ -8986,13 +8988,11 @@
       <c r="V29" t="inlineStr"/>
       <c r="W29" t="inlineStr"/>
       <c r="X29" t="inlineStr"/>
-      <c r="Y29" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z29" t="inlineStr"/>
-      <c r="AA29" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA29" t="inlineStr"/>
       <c r="AB29" t="inlineStr"/>
       <c r="AC29" t="inlineStr"/>
       <c r="AD29" t="inlineStr"/>
@@ -9006,10 +9006,10 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
-      <c r="E30" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
@@ -9022,7 +9022,9 @@
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
+      <c r="Q30" t="n">
+        <v>1</v>
+      </c>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr"/>
@@ -9033,9 +9035,7 @@
       <c r="W30" t="inlineStr"/>
       <c r="X30" t="inlineStr"/>
       <c r="Y30" t="inlineStr"/>
-      <c r="Z30" t="n">
-        <v>1</v>
-      </c>
+      <c r="Z30" t="inlineStr"/>
       <c r="AA30" t="inlineStr"/>
       <c r="AB30" t="inlineStr"/>
       <c r="AC30" t="inlineStr"/>
@@ -9068,18 +9068,18 @@
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
-      <c r="T31" t="n">
-        <v>1</v>
-      </c>
+      <c r="S31" t="n">
+        <v>1</v>
+      </c>
+      <c r="T31" t="inlineStr"/>
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="inlineStr"/>
       <c r="W31" t="inlineStr"/>
       <c r="X31" t="inlineStr"/>
-      <c r="Y31" t="inlineStr"/>
-      <c r="Z31" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y31" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z31" t="inlineStr"/>
       <c r="AA31" t="inlineStr"/>
       <c r="AB31" t="inlineStr"/>
       <c r="AC31" t="inlineStr"/>
@@ -9093,17 +9093,15 @@
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
       <c r="E32" t="inlineStr"/>
-      <c r="F32" t="n">
-        <v>1</v>
-      </c>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" t="n">
-        <v>1</v>
-      </c>
+      <c r="J32" t="inlineStr"/>
       <c r="K32" t="n">
         <v>1</v>
       </c>
@@ -9112,21 +9110,23 @@
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="n">
         <v>1</v>
       </c>
       <c r="T32" t="inlineStr"/>
-      <c r="U32" t="inlineStr"/>
+      <c r="U32" t="n">
+        <v>1</v>
+      </c>
       <c r="V32" t="inlineStr"/>
       <c r="W32" t="inlineStr"/>
       <c r="X32" t="inlineStr"/>
       <c r="Y32" t="inlineStr"/>
       <c r="Z32" t="inlineStr"/>
-      <c r="AA32" t="inlineStr"/>
+      <c r="AA32" t="n">
+        <v>1</v>
+      </c>
       <c r="AB32" t="inlineStr"/>
       <c r="AC32" t="inlineStr"/>
       <c r="AD32" t="inlineStr"/>

</xml_diff>

<commit_message>
breytti engu, var að keyra út frá nýju input
</commit_message>
<xml_diff>
--- a/03_26_schedule_results.xlsx
+++ b/03_26_schedule_results.xlsx
@@ -690,18 +690,18 @@
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Thelma</t>
+          <t>Helgi</t>
         </is>
       </c>
       <c r="J5" t="n">
         <v>3</v>
       </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L5" t="n">
         <v>3</v>
@@ -710,7 +710,7 @@
         <v>80</v>
       </c>
       <c r="N5" t="n">
-        <v>410</v>
+        <v>470</v>
       </c>
     </row>
     <row r="6">
@@ -742,18 +742,18 @@
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Thelma</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L6" t="n">
         <v>3</v>
@@ -762,7 +762,7 @@
         <v>80</v>
       </c>
       <c r="N6" t="n">
-        <v>470</v>
+        <v>410</v>
       </c>
     </row>
     <row r="7">
@@ -846,11 +846,11 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J8" t="n">
@@ -1470,18 +1470,18 @@
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J20" t="n">
         <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L20" t="n">
         <v>4</v>
@@ -1490,7 +1490,7 @@
         <v>70</v>
       </c>
       <c r="N20" t="n">
-        <v>330</v>
+        <v>530</v>
       </c>
     </row>
     <row r="21">
@@ -1522,18 +1522,18 @@
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
         <v>4</v>
@@ -1542,7 +1542,7 @@
         <v>70</v>
       </c>
       <c r="N21" t="n">
-        <v>340</v>
+        <v>330</v>
       </c>
     </row>
     <row r="22">
@@ -1574,18 +1574,18 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K22" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="L22" t="n">
         <v>4</v>
@@ -1594,7 +1594,7 @@
         <v>70</v>
       </c>
       <c r="N22" t="n">
-        <v>520</v>
+        <v>340</v>
       </c>
     </row>
     <row r="23">
@@ -1886,11 +1886,11 @@
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J28" t="n">
@@ -1990,18 +1990,18 @@
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J30" t="n">
         <v>2</v>
       </c>
       <c r="K30" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L30" t="n">
         <v>3.5</v>
@@ -2010,7 +2010,7 @@
         <v>50</v>
       </c>
       <c r="N30" t="n">
-        <v>510</v>
+        <v>490</v>
       </c>
     </row>
     <row r="31">
@@ -2042,18 +2042,18 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K31" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L31" t="n">
         <v>3.5</v>
@@ -2062,7 +2062,7 @@
         <v>50</v>
       </c>
       <c r="N31" t="n">
-        <v>490</v>
+        <v>510</v>
       </c>
     </row>
     <row r="32">
@@ -2094,18 +2094,18 @@
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K32" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L32" t="n">
         <v>3.5</v>
@@ -2114,7 +2114,7 @@
         <v>50</v>
       </c>
       <c r="N32" t="n">
-        <v>410</v>
+        <v>490</v>
       </c>
     </row>
     <row r="33">
@@ -2146,18 +2146,18 @@
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J33" t="n">
         <v>2</v>
       </c>
       <c r="K33" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L33" t="n">
         <v>3.5</v>
@@ -2166,7 +2166,7 @@
         <v>50</v>
       </c>
       <c r="N33" t="n">
-        <v>430</v>
+        <v>410</v>
       </c>
     </row>
     <row r="34">
@@ -2198,18 +2198,18 @@
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L34" t="n">
         <v>3.5</v>
@@ -2218,7 +2218,7 @@
         <v>50</v>
       </c>
       <c r="N34" t="n">
-        <v>380</v>
+        <v>430</v>
       </c>
     </row>
     <row r="35">
@@ -2250,18 +2250,18 @@
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K35" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L35" t="n">
         <v>3.5</v>
@@ -2270,7 +2270,7 @@
         <v>50</v>
       </c>
       <c r="N35" t="n">
-        <v>440</v>
+        <v>380</v>
       </c>
     </row>
     <row r="36">
@@ -2313,7 +2313,7 @@
         <v>2</v>
       </c>
       <c r="K36" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L36" t="n">
         <v>3.5</v>
@@ -2458,11 +2458,11 @@
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Gunnar</t>
+          <t>Nanna</t>
         </is>
       </c>
       <c r="J39" t="n">
@@ -2478,7 +2478,7 @@
         <v>50</v>
       </c>
       <c r="N39" t="n">
-        <v>550</v>
+        <v>540</v>
       </c>
     </row>
     <row r="40">
@@ -2510,18 +2510,18 @@
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Pétur</t>
+          <t>Össur</t>
         </is>
       </c>
       <c r="J40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K40" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L40" t="n">
         <v>4</v>
@@ -2530,7 +2530,7 @@
         <v>50</v>
       </c>
       <c r="N40" t="n">
-        <v>330</v>
+        <v>540</v>
       </c>
     </row>
     <row r="41">
@@ -2562,18 +2562,18 @@
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J41" t="n">
         <v>2</v>
       </c>
       <c r="K41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L41" t="n">
         <v>4</v>
@@ -2582,7 +2582,7 @@
         <v>50</v>
       </c>
       <c r="N41" t="n">
-        <v>310</v>
+        <v>330</v>
       </c>
     </row>
     <row r="42">
@@ -2614,18 +2614,18 @@
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J42" t="n">
         <v>2</v>
       </c>
       <c r="K42" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L42" t="n">
         <v>4</v>
@@ -2634,7 +2634,7 @@
         <v>50</v>
       </c>
       <c r="N42" t="n">
-        <v>330</v>
+        <v>310</v>
       </c>
     </row>
     <row r="43">
@@ -2666,18 +2666,18 @@
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J43" t="n">
         <v>2</v>
       </c>
       <c r="K43" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L43" t="n">
         <v>4</v>
@@ -2718,18 +2718,18 @@
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K44" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="L44" t="n">
         <v>4</v>
@@ -2738,7 +2738,7 @@
         <v>50</v>
       </c>
       <c r="N44" t="n">
-        <v>510</v>
+        <v>330</v>
       </c>
     </row>
     <row r="45">
@@ -2989,7 +2989,7 @@
         <v>1</v>
       </c>
       <c r="K49" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L49" t="n">
         <v>4</v>
@@ -3154,7 +3154,7 @@
         <v>50</v>
       </c>
       <c r="N52" t="n">
-        <v>490</v>
+        <v>390</v>
       </c>
     </row>
     <row r="53">
@@ -3186,18 +3186,18 @@
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Össur</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K53" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L53" t="n">
         <v>4</v>
@@ -3206,7 +3206,7 @@
         <v>50</v>
       </c>
       <c r="N53" t="n">
-        <v>540</v>
+        <v>370</v>
       </c>
     </row>
     <row r="54">
@@ -3238,18 +3238,18 @@
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J54" t="n">
         <v>2</v>
       </c>
       <c r="K54" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="L54" t="n">
         <v>4</v>
@@ -3258,7 +3258,7 @@
         <v>50</v>
       </c>
       <c r="N54" t="n">
-        <v>370</v>
+        <v>560</v>
       </c>
     </row>
     <row r="55">
@@ -3290,18 +3290,18 @@
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J55" t="n">
         <v>2</v>
       </c>
       <c r="K55" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L55" t="n">
         <v>4</v>
@@ -3310,7 +3310,7 @@
         <v>50</v>
       </c>
       <c r="N55" t="n">
-        <v>560</v>
+        <v>390</v>
       </c>
     </row>
     <row r="56">
@@ -3342,18 +3342,18 @@
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J56" t="n">
         <v>2</v>
       </c>
       <c r="K56" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L56" t="n">
         <v>4</v>
@@ -3362,7 +3362,7 @@
         <v>50</v>
       </c>
       <c r="N56" t="n">
-        <v>390</v>
+        <v>580</v>
       </c>
     </row>
     <row r="57">
@@ -3394,18 +3394,18 @@
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J57" t="n">
         <v>2</v>
       </c>
       <c r="K57" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L57" t="n">
         <v>4</v>
@@ -3414,7 +3414,7 @@
         <v>50</v>
       </c>
       <c r="N57" t="n">
-        <v>390</v>
+        <v>350</v>
       </c>
     </row>
     <row r="58">
@@ -3446,18 +3446,18 @@
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K58" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="L58" t="n">
         <v>4</v>
@@ -3466,7 +3466,7 @@
         <v>50</v>
       </c>
       <c r="N58" t="n">
-        <v>350</v>
+        <v>580</v>
       </c>
     </row>
     <row r="59">
@@ -3509,7 +3509,7 @@
         <v>2</v>
       </c>
       <c r="K59" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L59" t="n">
         <v>4</v>
@@ -3518,7 +3518,7 @@
         <v>50</v>
       </c>
       <c r="N59" t="n">
-        <v>560</v>
+        <v>390</v>
       </c>
     </row>
     <row r="60">
@@ -3706,15 +3706,15 @@
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K63" t="n">
         <v>0</v>
@@ -3726,7 +3726,7 @@
         <v>80</v>
       </c>
       <c r="N63" t="n">
-        <v>450</v>
+        <v>470</v>
       </c>
     </row>
     <row r="64">
@@ -4226,18 +4226,18 @@
       </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Helgi</t>
+          <t>Thelma</t>
         </is>
       </c>
       <c r="J73" t="n">
         <v>3</v>
       </c>
       <c r="K73" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L73" t="n">
         <v>3.5</v>
@@ -4246,7 +4246,7 @@
         <v>50</v>
       </c>
       <c r="N73" t="n">
-        <v>540</v>
+        <v>530</v>
       </c>
     </row>
     <row r="74">
@@ -4278,18 +4278,18 @@
       </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Thelma</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K74" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L74" t="n">
         <v>3.5</v>
@@ -4298,7 +4298,7 @@
         <v>50</v>
       </c>
       <c r="N74" t="n">
-        <v>530</v>
+        <v>520</v>
       </c>
     </row>
     <row r="75">
@@ -4341,7 +4341,7 @@
         <v>2</v>
       </c>
       <c r="K75" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L75" t="n">
         <v>3.5</v>
@@ -4486,18 +4486,18 @@
       </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K78" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L78" t="n">
         <v>3.5</v>
@@ -4506,7 +4506,7 @@
         <v>50</v>
       </c>
       <c r="N78" t="n">
-        <v>540</v>
+        <v>530</v>
       </c>
     </row>
     <row r="79">
@@ -4538,18 +4538,18 @@
       </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K79" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="L79" t="n">
         <v>3.5</v>
@@ -4558,7 +4558,7 @@
         <v>50</v>
       </c>
       <c r="N79" t="n">
-        <v>380</v>
+        <v>540</v>
       </c>
     </row>
     <row r="80">
@@ -4590,18 +4590,18 @@
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J80" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K80" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L80" t="n">
         <v>3.5</v>
@@ -4610,7 +4610,7 @@
         <v>50</v>
       </c>
       <c r="N80" t="n">
-        <v>370</v>
+        <v>380</v>
       </c>
     </row>
     <row r="81">
@@ -4642,18 +4642,18 @@
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Nanna</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J81" t="n">
         <v>1</v>
       </c>
       <c r="K81" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L81" t="n">
         <v>3.5</v>
@@ -4662,7 +4662,7 @@
         <v>50</v>
       </c>
       <c r="N81" t="n">
-        <v>540</v>
+        <v>370</v>
       </c>
     </row>
     <row r="82">
@@ -4705,7 +4705,7 @@
         <v>1</v>
       </c>
       <c r="K82" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L82" t="n">
         <v>3.5</v>
@@ -4798,18 +4798,18 @@
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J84" t="n">
         <v>2</v>
       </c>
       <c r="K84" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L84" t="n">
         <v>4</v>
@@ -4818,7 +4818,7 @@
         <v>50</v>
       </c>
       <c r="N84" t="n">
-        <v>390</v>
+        <v>420</v>
       </c>
     </row>
     <row r="85">
@@ -4850,18 +4850,18 @@
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J85" t="n">
         <v>2</v>
       </c>
       <c r="K85" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L85" t="n">
         <v>4</v>
@@ -4870,7 +4870,7 @@
         <v>50</v>
       </c>
       <c r="N85" t="n">
-        <v>560</v>
+        <v>390</v>
       </c>
     </row>
     <row r="86">
@@ -4902,18 +4902,18 @@
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J86" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K86" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L86" t="n">
         <v>4</v>
@@ -4954,18 +4954,18 @@
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J87" t="n">
         <v>2</v>
       </c>
       <c r="K87" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L87" t="n">
         <v>4</v>
@@ -4974,7 +4974,7 @@
         <v>50</v>
       </c>
       <c r="N87" t="n">
-        <v>400</v>
+        <v>560</v>
       </c>
     </row>
     <row r="88">
@@ -5006,18 +5006,18 @@
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J88" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K88" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L88" t="n">
         <v>4</v>
@@ -5026,7 +5026,7 @@
         <v>50</v>
       </c>
       <c r="N88" t="n">
-        <v>390</v>
+        <v>540</v>
       </c>
     </row>
     <row r="89">
@@ -5058,18 +5058,18 @@
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J89" t="n">
         <v>2</v>
       </c>
       <c r="K89" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L89" t="n">
         <v>4</v>
@@ -5078,7 +5078,7 @@
         <v>50</v>
       </c>
       <c r="N89" t="n">
-        <v>390</v>
+        <v>400</v>
       </c>
     </row>
     <row r="90">
@@ -5110,18 +5110,18 @@
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J90" t="n">
         <v>2</v>
       </c>
       <c r="K90" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L90" t="n">
         <v>4</v>
@@ -5162,18 +5162,18 @@
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J91" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K91" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="L91" t="n">
         <v>4</v>
@@ -5182,7 +5182,7 @@
         <v>50</v>
       </c>
       <c r="N91" t="n">
-        <v>570</v>
+        <v>390</v>
       </c>
     </row>
     <row r="92">
@@ -5277,7 +5277,7 @@
         <v>1</v>
       </c>
       <c r="K93" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L93" t="n">
         <v>4</v>
@@ -5329,7 +5329,7 @@
         <v>2</v>
       </c>
       <c r="K94" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L94" t="n">
         <v>4</v>
@@ -5526,18 +5526,18 @@
       </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>Össur</t>
+          <t>Helgi</t>
         </is>
       </c>
       <c r="J98" t="n">
         <v>3</v>
       </c>
       <c r="K98" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="L98" t="n">
         <v>3</v>
@@ -5546,7 +5546,7 @@
         <v>70</v>
       </c>
       <c r="N98" t="n">
-        <v>490</v>
+        <v>540</v>
       </c>
     </row>
     <row r="99">
@@ -5578,18 +5578,18 @@
       </c>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>Pétur</t>
+          <t>Össur</t>
         </is>
       </c>
       <c r="J99" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K99" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="L99" t="n">
         <v>3</v>
@@ -5598,7 +5598,7 @@
         <v>70</v>
       </c>
       <c r="N99" t="n">
-        <v>540</v>
+        <v>490</v>
       </c>
     </row>
     <row r="100">
@@ -5630,18 +5630,18 @@
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="n">
+        <v>5</v>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Pétur</t>
+        </is>
+      </c>
+      <c r="J100" t="n">
+        <v>2</v>
+      </c>
+      <c r="K100" t="n">
         <v>6</v>
-      </c>
-      <c r="I100" t="inlineStr">
-        <is>
-          <t>Unnur</t>
-        </is>
-      </c>
-      <c r="J100" t="n">
-        <v>2</v>
-      </c>
-      <c r="K100" t="n">
-        <v>5</v>
       </c>
       <c r="L100" t="n">
         <v>3</v>
@@ -5682,18 +5682,18 @@
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J101" t="n">
         <v>2</v>
       </c>
       <c r="K101" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L101" t="n">
         <v>3</v>
@@ -5702,7 +5702,7 @@
         <v>70</v>
       </c>
       <c r="N101" t="n">
-        <v>540</v>
+        <v>490</v>
       </c>
     </row>
     <row r="102">
@@ -5838,18 +5838,18 @@
       </c>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J104" t="n">
         <v>2</v>
       </c>
       <c r="K104" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L104" t="n">
         <v>3</v>
@@ -5858,7 +5858,7 @@
         <v>70</v>
       </c>
       <c r="N104" t="n">
-        <v>510</v>
+        <v>540</v>
       </c>
     </row>
     <row r="105">
@@ -6057,7 +6057,7 @@
         <v>1</v>
       </c>
       <c r="K108" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L108" t="n">
         <v>3</v>
@@ -6150,18 +6150,18 @@
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Pétur</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J110" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K110" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L110" t="n">
         <v>4</v>
@@ -6170,7 +6170,7 @@
         <v>100</v>
       </c>
       <c r="N110" t="n">
-        <v>470</v>
+        <v>460</v>
       </c>
     </row>
     <row r="111">
@@ -6202,18 +6202,18 @@
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J111" t="n">
         <v>1</v>
       </c>
       <c r="K111" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L111" t="n">
         <v>4</v>
@@ -6222,7 +6222,7 @@
         <v>100</v>
       </c>
       <c r="N111" t="n">
-        <v>460</v>
+        <v>470</v>
       </c>
     </row>
     <row r="112">
@@ -6462,18 +6462,18 @@
       </c>
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J116" t="n">
         <v>2</v>
       </c>
       <c r="K116" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="L116" t="n">
         <v>4</v>
@@ -6482,7 +6482,7 @@
         <v>70</v>
       </c>
       <c r="N116" t="n">
-        <v>550</v>
+        <v>540</v>
       </c>
     </row>
     <row r="117">
@@ -6514,18 +6514,18 @@
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J117" t="n">
         <v>2</v>
       </c>
       <c r="K117" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L117" t="n">
         <v>4</v>
@@ -6566,18 +6566,18 @@
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J118" t="n">
         <v>2</v>
       </c>
       <c r="K118" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="L118" t="n">
         <v>4</v>
@@ -6618,18 +6618,18 @@
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J119" t="n">
         <v>2</v>
       </c>
       <c r="K119" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L119" t="n">
         <v>4</v>
@@ -6638,7 +6638,7 @@
         <v>70</v>
       </c>
       <c r="N119" t="n">
-        <v>540</v>
+        <v>340</v>
       </c>
     </row>
     <row r="120">
@@ -6670,18 +6670,18 @@
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J120" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K120" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="L120" t="n">
         <v>4</v>
@@ -6690,7 +6690,7 @@
         <v>70</v>
       </c>
       <c r="N120" t="n">
-        <v>340</v>
+        <v>550</v>
       </c>
     </row>
     <row r="121">
@@ -6878,11 +6878,11 @@
       </c>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J124" t="n">
@@ -6930,18 +6930,18 @@
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J125" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K125" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L125" t="n">
         <v>2</v>
@@ -6950,7 +6950,7 @@
         <v>70</v>
       </c>
       <c r="N125" t="n">
-        <v>340</v>
+        <v>560</v>
       </c>
     </row>
     <row r="126">
@@ -6982,18 +6982,18 @@
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J126" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K126" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L126" t="n">
         <v>2</v>
@@ -7002,7 +7002,7 @@
         <v>70</v>
       </c>
       <c r="N126" t="n">
-        <v>570</v>
+        <v>340</v>
       </c>
     </row>
     <row r="127">
@@ -7034,18 +7034,18 @@
       </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J127" t="n">
         <v>2</v>
       </c>
       <c r="K127" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L127" t="n">
         <v>2</v>
@@ -7054,7 +7054,7 @@
         <v>70</v>
       </c>
       <c r="N127" t="n">
-        <v>540</v>
+        <v>570</v>
       </c>
     </row>
     <row r="128">
@@ -7086,18 +7086,18 @@
       </c>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J128" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K128" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L128" t="n">
         <v>2</v>
@@ -7106,7 +7106,7 @@
         <v>70</v>
       </c>
       <c r="N128" t="n">
-        <v>580</v>
+        <v>550</v>
       </c>
     </row>
     <row r="129">
@@ -7138,18 +7138,18 @@
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J129" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K129" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L129" t="n">
         <v>2</v>
@@ -7158,7 +7158,7 @@
         <v>70</v>
       </c>
       <c r="N129" t="n">
-        <v>550</v>
+        <v>340</v>
       </c>
     </row>
     <row r="130">
@@ -7190,18 +7190,18 @@
       </c>
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J130" t="n">
         <v>2</v>
       </c>
       <c r="K130" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L130" t="n">
         <v>2</v>
@@ -7210,7 +7210,7 @@
         <v>70</v>
       </c>
       <c r="N130" t="n">
-        <v>550</v>
+        <v>340</v>
       </c>
     </row>
     <row r="131">
@@ -7242,18 +7242,18 @@
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J131" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K131" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L131" t="n">
         <v>2</v>
@@ -7262,7 +7262,7 @@
         <v>70</v>
       </c>
       <c r="N131" t="n">
-        <v>340</v>
+        <v>540</v>
       </c>
     </row>
     <row r="132">
@@ -7294,18 +7294,18 @@
       </c>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Camilla</t>
         </is>
       </c>
       <c r="J132" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K132" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="L132" t="n">
         <v>2</v>
@@ -7314,7 +7314,7 @@
         <v>70</v>
       </c>
       <c r="N132" t="n">
-        <v>340</v>
+        <v>570</v>
       </c>
     </row>
     <row r="133">
@@ -7346,18 +7346,18 @@
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Camilla</t>
+          <t>Bergur</t>
         </is>
       </c>
       <c r="J133" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K133" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L133" t="n">
         <v>2</v>
@@ -7366,7 +7366,7 @@
         <v>70</v>
       </c>
       <c r="N133" t="n">
-        <v>570</v>
+        <v>550</v>
       </c>
     </row>
     <row r="134">
@@ -7398,18 +7398,18 @@
       </c>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Bergur</t>
+          <t>Gunnar</t>
         </is>
       </c>
       <c r="J134" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K134" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="L134" t="n">
         <v>2</v>
@@ -7418,7 +7418,7 @@
         <v>70</v>
       </c>
       <c r="N134" t="n">
-        <v>550</v>
+        <v>570</v>
       </c>
     </row>
     <row r="135">
@@ -7502,15 +7502,15 @@
       </c>
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Helgi</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J136" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K136" t="n">
         <v>1</v>
@@ -7801,7 +7801,9 @@
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
@@ -7820,13 +7822,13 @@
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
+      <c r="U3" t="n">
+        <v>1</v>
+      </c>
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr"/>
@@ -7837,9 +7839,7 @@
       <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="inlineStr"/>
       <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="n">
-        <v>1</v>
-      </c>
+      <c r="AF3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -7856,10 +7856,10 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="n">
-        <v>1</v>
-      </c>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
@@ -7954,7 +7954,9 @@
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
+      <c r="S6" t="n">
+        <v>1</v>
+      </c>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="n">
         <v>1</v>
@@ -7962,11 +7964,11 @@
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
+      <c r="AA6" t="n">
+        <v>1</v>
+      </c>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="inlineStr"/>
@@ -8078,19 +8080,21 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="n">
-        <v>1</v>
-      </c>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
         <v>1</v>
       </c>
-      <c r="M9" t="inlineStr"/>
+      <c r="M9" t="n">
+        <v>1</v>
+      </c>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
+      <c r="Q9" t="n">
+        <v>1</v>
+      </c>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
@@ -8099,9 +8103,7 @@
       <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr"/>
-      <c r="Z9" t="n">
-        <v>1</v>
-      </c>
+      <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="inlineStr"/>
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
@@ -8113,10 +8115,10 @@
       <c r="A10" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
@@ -8158,9 +8160,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="inlineStr"/>
-      <c r="C11" t="n">
-        <v>1</v>
-      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
@@ -8169,22 +8169,22 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="n">
-        <v>1</v>
-      </c>
+      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
+      <c r="S11" t="n">
+        <v>1</v>
+      </c>
       <c r="T11" t="inlineStr"/>
-      <c r="U11" t="n">
-        <v>1</v>
-      </c>
+      <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr"/>
@@ -8195,7 +8195,9 @@
       <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="inlineStr"/>
       <c r="AE11" t="inlineStr"/>
-      <c r="AF11" t="inlineStr"/>
+      <c r="AF11" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -8305,7 +8307,9 @@
         <v>1</v>
       </c>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
+      <c r="L14" t="n">
+        <v>1</v>
+      </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
@@ -8492,7 +8496,9 @@
         <v>1</v>
       </c>
       <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
+      <c r="U18" t="n">
+        <v>1</v>
+      </c>
       <c r="V18" t="inlineStr"/>
       <c r="W18" t="inlineStr"/>
       <c r="X18" t="inlineStr"/>
@@ -8500,9 +8506,7 @@
       <c r="Z18" t="n">
         <v>1</v>
       </c>
-      <c r="AA18" t="n">
-        <v>1</v>
-      </c>
+      <c r="AA18" t="inlineStr"/>
       <c r="AB18" t="inlineStr"/>
       <c r="AC18" t="inlineStr"/>
       <c r="AD18" t="inlineStr"/>
@@ -8518,16 +8522,18 @@
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
-      <c r="K19" t="n">
-        <v>1</v>
-      </c>
-      <c r="L19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="n">
+        <v>1</v>
+      </c>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
@@ -8544,9 +8550,7 @@
         <v>1</v>
       </c>
       <c r="Z19" t="inlineStr"/>
-      <c r="AA19" t="n">
-        <v>1</v>
-      </c>
+      <c r="AA19" t="inlineStr"/>
       <c r="AB19" t="inlineStr"/>
       <c r="AC19" t="inlineStr"/>
       <c r="AD19" t="inlineStr"/>
@@ -8587,10 +8591,10 @@
       <c r="W20" t="inlineStr"/>
       <c r="X20" t="inlineStr"/>
       <c r="Y20" t="inlineStr"/>
-      <c r="Z20" t="inlineStr"/>
-      <c r="AA20" t="n">
-        <v>1</v>
-      </c>
+      <c r="Z20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA20" t="inlineStr"/>
       <c r="AB20" t="inlineStr"/>
       <c r="AC20" t="inlineStr"/>
       <c r="AD20" t="inlineStr"/>
@@ -8610,10 +8614,10 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="n">
-        <v>1</v>
-      </c>
+      <c r="I21" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="n">
         <v>1</v>
@@ -8622,15 +8626,13 @@
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
+      <c r="Q21" t="n">
+        <v>1</v>
+      </c>
       <c r="R21" t="inlineStr"/>
-      <c r="S21" t="n">
-        <v>1</v>
-      </c>
+      <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr"/>
-      <c r="U21" t="n">
-        <v>1</v>
-      </c>
+      <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
       <c r="X21" t="inlineStr"/>
@@ -8872,9 +8874,7 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="n">
-        <v>1</v>
-      </c>
+      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
@@ -8884,9 +8884,7 @@
         <v>1</v>
       </c>
       <c r="L27" t="inlineStr"/>
-      <c r="M27" t="n">
-        <v>1</v>
-      </c>
+      <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
@@ -8894,17 +8892,19 @@
         <v>1</v>
       </c>
       <c r="R27" t="inlineStr"/>
-      <c r="S27" t="n">
-        <v>1</v>
-      </c>
+      <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr"/>
-      <c r="Y27" t="inlineStr"/>
+      <c r="Y27" t="n">
+        <v>1</v>
+      </c>
       <c r="Z27" t="inlineStr"/>
-      <c r="AA27" t="inlineStr"/>
+      <c r="AA27" t="n">
+        <v>1</v>
+      </c>
       <c r="AB27" t="inlineStr"/>
       <c r="AC27" t="inlineStr"/>
       <c r="AD27" t="inlineStr"/>
@@ -8969,7 +8969,9 @@
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
+      <c r="J29" t="n">
+        <v>1</v>
+      </c>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="n">
         <v>1</v>
@@ -8978,9 +8980,7 @@
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr"/>
@@ -9145,9 +9145,7 @@
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" t="n">
-        <v>1</v>
-      </c>
+      <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
@@ -9170,7 +9168,9 @@
       <c r="X33" t="inlineStr"/>
       <c r="Y33" t="inlineStr"/>
       <c r="Z33" t="inlineStr"/>
-      <c r="AA33" t="inlineStr"/>
+      <c r="AA33" t="n">
+        <v>1</v>
+      </c>
       <c r="AB33" t="inlineStr"/>
       <c r="AC33" t="inlineStr"/>
       <c r="AD33" t="inlineStr"/>

</xml_diff>

<commit_message>
breytti úthlutun vakta út frá fríum
nú er forgangsröðunin á starfsmönnum öðruvísi, þeir sem eru skráðir í mikið frí ættu að fá færri vaktir í hlutfalli við fríið þeirra
</commit_message>
<xml_diff>
--- a/03_26_schedule_results.xlsx
+++ b/03_26_schedule_results.xlsx
@@ -586,15 +586,15 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K3" t="n">
         <v>1</v>
@@ -606,7 +606,7 @@
         <v>40</v>
       </c>
       <c r="N3" t="n">
-        <v>430</v>
+        <v>480</v>
       </c>
     </row>
     <row r="4">
@@ -898,11 +898,11 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J9" t="n">
@@ -1210,18 +1210,18 @@
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J15" t="n">
         <v>2</v>
       </c>
       <c r="K15" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L15" t="n">
         <v>4</v>
@@ -1230,7 +1230,7 @@
         <v>70</v>
       </c>
       <c r="N15" t="n">
-        <v>510</v>
+        <v>340</v>
       </c>
     </row>
     <row r="16">
@@ -1262,18 +1262,18 @@
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J16" t="n">
         <v>2</v>
       </c>
       <c r="K16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L16" t="n">
         <v>4</v>
@@ -1282,7 +1282,7 @@
         <v>70</v>
       </c>
       <c r="N16" t="n">
-        <v>340</v>
+        <v>480</v>
       </c>
     </row>
     <row r="17">
@@ -1314,18 +1314,18 @@
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J17" t="n">
         <v>2</v>
       </c>
       <c r="K17" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="L17" t="n">
         <v>4</v>
@@ -1334,7 +1334,7 @@
         <v>70</v>
       </c>
       <c r="N17" t="n">
-        <v>480</v>
+        <v>500</v>
       </c>
     </row>
     <row r="18">
@@ -1366,18 +1366,18 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J18" t="n">
         <v>2</v>
       </c>
       <c r="K18" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="L18" t="n">
         <v>4</v>
@@ -1386,7 +1386,7 @@
         <v>70</v>
       </c>
       <c r="N18" t="n">
-        <v>500</v>
+        <v>470</v>
       </c>
     </row>
     <row r="19">
@@ -1418,18 +1418,18 @@
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K19" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="L19" t="n">
         <v>4</v>
@@ -1438,7 +1438,7 @@
         <v>70</v>
       </c>
       <c r="N19" t="n">
-        <v>470</v>
+        <v>530</v>
       </c>
     </row>
     <row r="20">
@@ -1470,18 +1470,18 @@
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J20" t="n">
         <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
         <v>4</v>
@@ -1490,7 +1490,7 @@
         <v>70</v>
       </c>
       <c r="N20" t="n">
-        <v>530</v>
+        <v>330</v>
       </c>
     </row>
     <row r="21">
@@ -1522,18 +1522,18 @@
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L21" t="n">
         <v>4</v>
@@ -1542,7 +1542,7 @@
         <v>70</v>
       </c>
       <c r="N21" t="n">
-        <v>330</v>
+        <v>340</v>
       </c>
     </row>
     <row r="22">
@@ -1574,18 +1574,18 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Camilla</t>
         </is>
       </c>
       <c r="J22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K22" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L22" t="n">
         <v>4</v>
@@ -1594,7 +1594,7 @@
         <v>70</v>
       </c>
       <c r="N22" t="n">
-        <v>340</v>
+        <v>500</v>
       </c>
     </row>
     <row r="23">
@@ -1626,18 +1626,18 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Camilla</t>
+          <t>Anna</t>
         </is>
       </c>
       <c r="J23" t="n">
         <v>1</v>
       </c>
       <c r="K23" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L23" t="n">
         <v>4</v>
@@ -1646,7 +1646,7 @@
         <v>70</v>
       </c>
       <c r="N23" t="n">
-        <v>500</v>
+        <v>530</v>
       </c>
     </row>
     <row r="24">
@@ -2001,7 +2001,7 @@
         <v>2</v>
       </c>
       <c r="K30" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L30" t="n">
         <v>3.5</v>
@@ -2053,7 +2053,7 @@
         <v>2</v>
       </c>
       <c r="K31" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L31" t="n">
         <v>3.5</v>
@@ -2094,18 +2094,18 @@
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K32" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L32" t="n">
         <v>3.5</v>
@@ -2114,7 +2114,7 @@
         <v>50</v>
       </c>
       <c r="N32" t="n">
-        <v>490</v>
+        <v>410</v>
       </c>
     </row>
     <row r="33">
@@ -2146,18 +2146,18 @@
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J33" t="n">
         <v>2</v>
       </c>
       <c r="K33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L33" t="n">
         <v>3.5</v>
@@ -2166,7 +2166,7 @@
         <v>50</v>
       </c>
       <c r="N33" t="n">
-        <v>410</v>
+        <v>430</v>
       </c>
     </row>
     <row r="34">
@@ -2198,18 +2198,18 @@
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L34" t="n">
         <v>3.5</v>
@@ -2218,7 +2218,7 @@
         <v>50</v>
       </c>
       <c r="N34" t="n">
-        <v>430</v>
+        <v>380</v>
       </c>
     </row>
     <row r="35">
@@ -2250,18 +2250,18 @@
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K35" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L35" t="n">
         <v>3.5</v>
@@ -2270,7 +2270,7 @@
         <v>50</v>
       </c>
       <c r="N35" t="n">
-        <v>380</v>
+        <v>520</v>
       </c>
     </row>
     <row r="36">
@@ -2302,18 +2302,18 @@
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J36" t="n">
         <v>2</v>
       </c>
       <c r="K36" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L36" t="n">
         <v>3.5</v>
@@ -2322,7 +2322,7 @@
         <v>50</v>
       </c>
       <c r="N36" t="n">
-        <v>480</v>
+        <v>540</v>
       </c>
     </row>
     <row r="37">
@@ -2354,11 +2354,11 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J37" t="n">
@@ -2406,15 +2406,15 @@
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Nanna</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K38" t="n">
         <v>9</v>
@@ -2458,11 +2458,11 @@
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Nanna</t>
+          <t>Gunnar</t>
         </is>
       </c>
       <c r="J39" t="n">
@@ -2478,7 +2478,7 @@
         <v>50</v>
       </c>
       <c r="N39" t="n">
-        <v>540</v>
+        <v>550</v>
       </c>
     </row>
     <row r="40">
@@ -2666,18 +2666,18 @@
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K43" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="L43" t="n">
         <v>4</v>
@@ -2686,7 +2686,7 @@
         <v>50</v>
       </c>
       <c r="N43" t="n">
-        <v>330</v>
+        <v>530</v>
       </c>
     </row>
     <row r="44">
@@ -2718,18 +2718,18 @@
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J44" t="n">
         <v>2</v>
       </c>
       <c r="K44" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L44" t="n">
         <v>4</v>
@@ -2770,18 +2770,18 @@
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K45" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L45" t="n">
         <v>4</v>
@@ -2790,7 +2790,7 @@
         <v>50</v>
       </c>
       <c r="N45" t="n">
-        <v>490</v>
+        <v>330</v>
       </c>
     </row>
     <row r="46">
@@ -2822,18 +2822,18 @@
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K46" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L46" t="n">
         <v>4</v>
@@ -2842,7 +2842,7 @@
         <v>50</v>
       </c>
       <c r="N46" t="n">
-        <v>330</v>
+        <v>490</v>
       </c>
     </row>
     <row r="47">
@@ -2874,18 +2874,18 @@
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K47" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L47" t="n">
         <v>4</v>
@@ -2894,7 +2894,7 @@
         <v>50</v>
       </c>
       <c r="N47" t="n">
-        <v>320</v>
+        <v>330</v>
       </c>
     </row>
     <row r="48">
@@ -2926,18 +2926,18 @@
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Ólafur</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J48" t="n">
         <v>1</v>
       </c>
       <c r="K48" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L48" t="n">
         <v>4</v>
@@ -2946,7 +2946,7 @@
         <v>50</v>
       </c>
       <c r="N48" t="n">
-        <v>490</v>
+        <v>320</v>
       </c>
     </row>
     <row r="49">
@@ -2978,18 +2978,18 @@
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Anna</t>
+          <t>Ólafur</t>
         </is>
       </c>
       <c r="J49" t="n">
         <v>1</v>
       </c>
       <c r="K49" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L49" t="n">
         <v>4</v>
@@ -2998,7 +2998,7 @@
         <v>50</v>
       </c>
       <c r="N49" t="n">
-        <v>510</v>
+        <v>490</v>
       </c>
     </row>
     <row r="50">
@@ -3249,7 +3249,7 @@
         <v>2</v>
       </c>
       <c r="K54" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L54" t="n">
         <v>4</v>
@@ -3342,18 +3342,18 @@
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J56" t="n">
         <v>2</v>
       </c>
       <c r="K56" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L56" t="n">
         <v>4</v>
@@ -3362,7 +3362,7 @@
         <v>50</v>
       </c>
       <c r="N56" t="n">
-        <v>580</v>
+        <v>350</v>
       </c>
     </row>
     <row r="57">
@@ -3394,18 +3394,18 @@
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K57" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="L57" t="n">
         <v>4</v>
@@ -3414,7 +3414,7 @@
         <v>50</v>
       </c>
       <c r="N57" t="n">
-        <v>350</v>
+        <v>580</v>
       </c>
     </row>
     <row r="58">
@@ -3446,18 +3446,18 @@
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K58" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L58" t="n">
         <v>4</v>
@@ -3466,7 +3466,7 @@
         <v>50</v>
       </c>
       <c r="N58" t="n">
-        <v>580</v>
+        <v>390</v>
       </c>
     </row>
     <row r="59">
@@ -3498,18 +3498,18 @@
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J59" t="n">
         <v>2</v>
       </c>
       <c r="K59" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L59" t="n">
         <v>4</v>
@@ -3550,18 +3550,18 @@
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J60" t="n">
         <v>2</v>
       </c>
       <c r="K60" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L60" t="n">
         <v>4</v>
@@ -3602,18 +3602,18 @@
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Nanna</t>
         </is>
       </c>
       <c r="J61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K61" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L61" t="n">
         <v>4</v>
@@ -3622,7 +3622,7 @@
         <v>50</v>
       </c>
       <c r="N61" t="n">
-        <v>390</v>
+        <v>320</v>
       </c>
     </row>
     <row r="62">
@@ -3654,18 +3654,18 @@
       </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Nanna</t>
+          <t>Anna</t>
         </is>
       </c>
       <c r="J62" t="n">
         <v>1</v>
       </c>
       <c r="K62" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L62" t="n">
         <v>4</v>
@@ -3674,7 +3674,7 @@
         <v>50</v>
       </c>
       <c r="N62" t="n">
-        <v>320</v>
+        <v>580</v>
       </c>
     </row>
     <row r="63">
@@ -4237,7 +4237,7 @@
         <v>3</v>
       </c>
       <c r="K73" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L73" t="n">
         <v>3.5</v>
@@ -4289,7 +4289,7 @@
         <v>2</v>
       </c>
       <c r="K74" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L74" t="n">
         <v>3.5</v>
@@ -4341,7 +4341,7 @@
         <v>2</v>
       </c>
       <c r="K75" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L75" t="n">
         <v>3.5</v>
@@ -4486,18 +4486,18 @@
       </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J78" t="n">
         <v>2</v>
       </c>
       <c r="K78" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="L78" t="n">
         <v>3.5</v>
@@ -4506,7 +4506,7 @@
         <v>50</v>
       </c>
       <c r="N78" t="n">
-        <v>530</v>
+        <v>440</v>
       </c>
     </row>
     <row r="79">
@@ -4538,15 +4538,15 @@
       </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K79" t="n">
         <v>9</v>
@@ -4558,7 +4558,7 @@
         <v>50</v>
       </c>
       <c r="N79" t="n">
-        <v>540</v>
+        <v>530</v>
       </c>
     </row>
     <row r="80">
@@ -4590,18 +4590,18 @@
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K80" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L80" t="n">
         <v>3.5</v>
@@ -4610,7 +4610,7 @@
         <v>50</v>
       </c>
       <c r="N80" t="n">
-        <v>380</v>
+        <v>540</v>
       </c>
     </row>
     <row r="81">
@@ -4642,18 +4642,18 @@
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K81" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L81" t="n">
         <v>3.5</v>
@@ -4662,7 +4662,7 @@
         <v>50</v>
       </c>
       <c r="N81" t="n">
-        <v>370</v>
+        <v>380</v>
       </c>
     </row>
     <row r="82">
@@ -4694,18 +4694,18 @@
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Ólafur</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J82" t="n">
         <v>1</v>
       </c>
       <c r="K82" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L82" t="n">
         <v>3.5</v>
@@ -4714,7 +4714,7 @@
         <v>50</v>
       </c>
       <c r="N82" t="n">
-        <v>540</v>
+        <v>370</v>
       </c>
     </row>
     <row r="83">
@@ -4954,18 +4954,18 @@
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K87" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L87" t="n">
         <v>4</v>
@@ -4974,7 +4974,7 @@
         <v>50</v>
       </c>
       <c r="N87" t="n">
-        <v>560</v>
+        <v>580</v>
       </c>
     </row>
     <row r="88">
@@ -5006,18 +5006,18 @@
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J88" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K88" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L88" t="n">
         <v>4</v>
@@ -5026,7 +5026,7 @@
         <v>50</v>
       </c>
       <c r="N88" t="n">
-        <v>540</v>
+        <v>580</v>
       </c>
     </row>
     <row r="89">
@@ -5069,7 +5069,7 @@
         <v>2</v>
       </c>
       <c r="K89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L89" t="n">
         <v>4</v>
@@ -5121,7 +5121,7 @@
         <v>2</v>
       </c>
       <c r="K90" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L90" t="n">
         <v>4</v>
@@ -5173,7 +5173,7 @@
         <v>2</v>
       </c>
       <c r="K91" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L91" t="n">
         <v>4</v>
@@ -5266,18 +5266,18 @@
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>Anna</t>
+          <t>Ólafur</t>
         </is>
       </c>
       <c r="J93" t="n">
         <v>1</v>
       </c>
       <c r="K93" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L93" t="n">
         <v>4</v>
@@ -5286,7 +5286,7 @@
         <v>50</v>
       </c>
       <c r="N93" t="n">
-        <v>560</v>
+        <v>540</v>
       </c>
     </row>
     <row r="94">
@@ -5526,18 +5526,18 @@
       </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>Helgi</t>
+          <t>Ásdís</t>
         </is>
       </c>
       <c r="J98" t="n">
         <v>3</v>
       </c>
       <c r="K98" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L98" t="n">
         <v>3</v>
@@ -5578,18 +5578,18 @@
       </c>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>Össur</t>
+          <t>Helgi</t>
         </is>
       </c>
       <c r="J99" t="n">
         <v>3</v>
       </c>
       <c r="K99" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="L99" t="n">
         <v>3</v>
@@ -5598,7 +5598,7 @@
         <v>70</v>
       </c>
       <c r="N99" t="n">
-        <v>490</v>
+        <v>540</v>
       </c>
     </row>
     <row r="100">
@@ -5630,18 +5630,18 @@
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>Pétur</t>
+          <t>Össur</t>
         </is>
       </c>
       <c r="J100" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K100" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L100" t="n">
         <v>3</v>
@@ -5682,18 +5682,18 @@
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J101" t="n">
         <v>2</v>
       </c>
       <c r="K101" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L101" t="n">
         <v>3</v>
@@ -5734,18 +5734,18 @@
       </c>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J102" t="n">
         <v>2</v>
       </c>
       <c r="K102" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L102" t="n">
         <v>3</v>
@@ -5754,7 +5754,7 @@
         <v>70</v>
       </c>
       <c r="N102" t="n">
-        <v>380</v>
+        <v>490</v>
       </c>
     </row>
     <row r="103">
@@ -5786,18 +5786,18 @@
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J103" t="n">
         <v>2</v>
       </c>
       <c r="K103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L103" t="n">
         <v>3</v>
@@ -5806,7 +5806,7 @@
         <v>70</v>
       </c>
       <c r="N103" t="n">
-        <v>360</v>
+        <v>380</v>
       </c>
     </row>
     <row r="104">
@@ -5838,18 +5838,18 @@
       </c>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J104" t="n">
         <v>2</v>
       </c>
       <c r="K104" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L104" t="n">
         <v>3</v>
@@ -5858,7 +5858,7 @@
         <v>70</v>
       </c>
       <c r="N104" t="n">
-        <v>540</v>
+        <v>360</v>
       </c>
     </row>
     <row r="105">
@@ -6005,7 +6005,7 @@
         <v>2</v>
       </c>
       <c r="K107" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L107" t="n">
         <v>3</v>
@@ -6057,7 +6057,7 @@
         <v>1</v>
       </c>
       <c r="K108" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L108" t="n">
         <v>3</v>
@@ -6306,18 +6306,18 @@
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>Ásdís</t>
+          <t>Thelma</t>
         </is>
       </c>
       <c r="J113" t="n">
         <v>3</v>
       </c>
       <c r="K113" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L113" t="n">
         <v>4</v>
@@ -6326,7 +6326,7 @@
         <v>70</v>
       </c>
       <c r="N113" t="n">
-        <v>540</v>
+        <v>480</v>
       </c>
     </row>
     <row r="114">
@@ -6358,18 +6358,18 @@
       </c>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>Thelma</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J114" t="n">
+        <v>2</v>
+      </c>
+      <c r="K114" t="n">
         <v>3</v>
-      </c>
-      <c r="K114" t="n">
-        <v>4</v>
       </c>
       <c r="L114" t="n">
         <v>4</v>
@@ -6378,7 +6378,7 @@
         <v>70</v>
       </c>
       <c r="N114" t="n">
-        <v>480</v>
+        <v>400</v>
       </c>
     </row>
     <row r="115">
@@ -6410,18 +6410,18 @@
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="n">
+        <v>9</v>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Freyja</t>
+        </is>
+      </c>
+      <c r="J115" t="n">
+        <v>2</v>
+      </c>
+      <c r="K115" t="n">
         <v>7</v>
-      </c>
-      <c r="I115" t="inlineStr">
-        <is>
-          <t>Harpa</t>
-        </is>
-      </c>
-      <c r="J115" t="n">
-        <v>2</v>
-      </c>
-      <c r="K115" t="n">
-        <v>3</v>
       </c>
       <c r="L115" t="n">
         <v>4</v>
@@ -6430,7 +6430,7 @@
         <v>70</v>
       </c>
       <c r="N115" t="n">
-        <v>400</v>
+        <v>540</v>
       </c>
     </row>
     <row r="116">
@@ -6462,18 +6462,18 @@
       </c>
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J116" t="n">
         <v>2</v>
       </c>
       <c r="K116" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L116" t="n">
         <v>4</v>
@@ -6514,18 +6514,18 @@
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J117" t="n">
         <v>2</v>
       </c>
       <c r="K117" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L117" t="n">
         <v>4</v>
@@ -6566,18 +6566,18 @@
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J118" t="n">
         <v>2</v>
       </c>
       <c r="K118" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L118" t="n">
         <v>4</v>
@@ -6586,7 +6586,7 @@
         <v>70</v>
       </c>
       <c r="N118" t="n">
-        <v>540</v>
+        <v>340</v>
       </c>
     </row>
     <row r="119">
@@ -6618,18 +6618,18 @@
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J119" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K119" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="L119" t="n">
         <v>4</v>
@@ -6638,7 +6638,7 @@
         <v>70</v>
       </c>
       <c r="N119" t="n">
-        <v>340</v>
+        <v>550</v>
       </c>
     </row>
     <row r="120">
@@ -6670,18 +6670,18 @@
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K120" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="L120" t="n">
         <v>4</v>
@@ -6690,7 +6690,7 @@
         <v>70</v>
       </c>
       <c r="N120" t="n">
-        <v>550</v>
+        <v>340</v>
       </c>
     </row>
     <row r="121">
@@ -6722,18 +6722,18 @@
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J121" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K121" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L121" t="n">
         <v>4</v>
@@ -6774,18 +6774,18 @@
       </c>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Camilla</t>
         </is>
       </c>
       <c r="J122" t="n">
         <v>1</v>
       </c>
       <c r="K122" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L122" t="n">
         <v>4</v>
@@ -6794,7 +6794,7 @@
         <v>70</v>
       </c>
       <c r="N122" t="n">
-        <v>340</v>
+        <v>570</v>
       </c>
     </row>
     <row r="123">
@@ -6982,18 +6982,18 @@
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J126" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K126" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L126" t="n">
         <v>2</v>
@@ -7002,7 +7002,7 @@
         <v>70</v>
       </c>
       <c r="N126" t="n">
-        <v>340</v>
+        <v>510</v>
       </c>
     </row>
     <row r="127">
@@ -7034,11 +7034,11 @@
       </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J127" t="n">
@@ -7054,7 +7054,7 @@
         <v>70</v>
       </c>
       <c r="N127" t="n">
-        <v>570</v>
+        <v>590</v>
       </c>
     </row>
     <row r="128">
@@ -7086,18 +7086,18 @@
       </c>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J128" t="n">
         <v>2</v>
       </c>
       <c r="K128" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="L128" t="n">
         <v>2</v>
@@ -7106,7 +7106,7 @@
         <v>70</v>
       </c>
       <c r="N128" t="n">
-        <v>550</v>
+        <v>580</v>
       </c>
     </row>
     <row r="129">
@@ -7138,18 +7138,18 @@
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="n">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J129" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K129" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L129" t="n">
         <v>2</v>
@@ -7190,18 +7190,18 @@
       </c>
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J130" t="n">
         <v>2</v>
       </c>
       <c r="K130" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="L130" t="n">
         <v>2</v>
@@ -7210,7 +7210,7 @@
         <v>70</v>
       </c>
       <c r="N130" t="n">
-        <v>340</v>
+        <v>570</v>
       </c>
     </row>
     <row r="131">
@@ -7242,18 +7242,18 @@
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J131" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K131" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L131" t="n">
         <v>2</v>
@@ -7262,7 +7262,7 @@
         <v>70</v>
       </c>
       <c r="N131" t="n">
-        <v>540</v>
+        <v>340</v>
       </c>
     </row>
     <row r="132">
@@ -7294,18 +7294,18 @@
       </c>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Camilla</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J132" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K132" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L132" t="n">
         <v>2</v>
@@ -7314,7 +7314,7 @@
         <v>70</v>
       </c>
       <c r="N132" t="n">
-        <v>570</v>
+        <v>340</v>
       </c>
     </row>
     <row r="133">
@@ -7346,15 +7346,15 @@
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Bergur</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J133" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K133" t="n">
         <v>4</v>
@@ -7366,7 +7366,7 @@
         <v>70</v>
       </c>
       <c r="N133" t="n">
-        <v>550</v>
+        <v>540</v>
       </c>
     </row>
     <row r="134">
@@ -7398,18 +7398,18 @@
       </c>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Gunnar</t>
+          <t>Bergur</t>
         </is>
       </c>
       <c r="J134" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K134" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="L134" t="n">
         <v>2</v>
@@ -7418,7 +7418,7 @@
         <v>70</v>
       </c>
       <c r="N134" t="n">
-        <v>570</v>
+        <v>550</v>
       </c>
     </row>
     <row r="135">
@@ -7782,14 +7782,14 @@
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" t="n">
+        <v>1</v>
+      </c>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="n">
-        <v>1</v>
-      </c>
+      <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
@@ -8030,9 +8030,7 @@
       <c r="D8" t="n">
         <v>1</v>
       </c>
-      <c r="E8" t="n">
-        <v>1</v>
-      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
@@ -8060,7 +8058,9 @@
       <c r="Z8" t="n">
         <v>1</v>
       </c>
-      <c r="AA8" t="inlineStr"/>
+      <c r="AA8" t="n">
+        <v>1</v>
+      </c>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr"/>
@@ -8104,7 +8104,9 @@
       <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
-      <c r="AA9" t="inlineStr"/>
+      <c r="AA9" t="n">
+        <v>1</v>
+      </c>
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="inlineStr"/>
@@ -8224,9 +8226,7 @@
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
-      <c r="S12" t="n">
-        <v>1</v>
-      </c>
+      <c r="S12" t="inlineStr"/>
       <c r="T12" t="n">
         <v>1</v>
       </c>
@@ -8238,7 +8238,9 @@
       <c r="X12" t="inlineStr"/>
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="inlineStr"/>
-      <c r="AA12" t="inlineStr"/>
+      <c r="AA12" t="n">
+        <v>1</v>
+      </c>
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr"/>
       <c r="AD12" t="inlineStr"/>
@@ -8249,7 +8251,9 @@
       <c r="A13" t="n">
         <v>12</v>
       </c>
-      <c r="B13" t="inlineStr"/>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
@@ -8257,10 +8261,10 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
-      <c r="J13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
@@ -8307,9 +8311,7 @@
         <v>1</v>
       </c>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" t="n">
-        <v>1</v>
-      </c>
+      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
@@ -8318,7 +8320,9 @@
         <v>1</v>
       </c>
       <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
+      <c r="S14" t="n">
+        <v>1</v>
+      </c>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="n">
         <v>1</v>
@@ -8474,9 +8478,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="inlineStr"/>
-      <c r="C18" t="n">
-        <v>1</v>
-      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
@@ -8490,15 +8492,15 @@
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
+      <c r="Q18" t="n">
+        <v>1</v>
+      </c>
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="n">
         <v>1</v>
       </c>
       <c r="T18" t="inlineStr"/>
-      <c r="U18" t="n">
-        <v>1</v>
-      </c>
+      <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr"/>
       <c r="W18" t="inlineStr"/>
       <c r="X18" t="inlineStr"/>
@@ -8649,10 +8651,10 @@
       <c r="A22" t="n">
         <v>21</v>
       </c>
-      <c r="B22" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" t="inlineStr"/>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -8682,9 +8684,7 @@
       <c r="Z22" t="n">
         <v>1</v>
       </c>
-      <c r="AA22" t="n">
-        <v>1</v>
-      </c>
+      <c r="AA22" t="inlineStr"/>
       <c r="AB22" t="inlineStr"/>
       <c r="AC22" t="inlineStr"/>
       <c r="AD22" t="inlineStr"/>
@@ -8945,10 +8945,10 @@
       <c r="W28" t="inlineStr"/>
       <c r="X28" t="inlineStr"/>
       <c r="Y28" t="inlineStr"/>
-      <c r="Z28" t="inlineStr"/>
-      <c r="AA28" t="n">
-        <v>1</v>
-      </c>
+      <c r="Z28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA28" t="inlineStr"/>
       <c r="AB28" t="inlineStr"/>
       <c r="AC28" t="inlineStr"/>
       <c r="AD28" t="inlineStr"/>
@@ -9022,11 +9022,11 @@
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
-      <c r="S30" t="inlineStr"/>
+      <c r="S30" t="n">
+        <v>1</v>
+      </c>
       <c r="T30" t="inlineStr"/>
       <c r="U30" t="n">
         <v>1</v>
@@ -9052,25 +9052,25 @@
         <v>1</v>
       </c>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="n">
+        <v>1</v>
+      </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
-      <c r="K31" t="n">
-        <v>1</v>
-      </c>
-      <c r="L31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="n">
+        <v>1</v>
+      </c>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
-      <c r="S31" t="n">
-        <v>1</v>
-      </c>
+      <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr"/>
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="inlineStr"/>
@@ -9145,7 +9145,9 @@
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
+      <c r="J33" t="n">
+        <v>1</v>
+      </c>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
@@ -9168,9 +9170,7 @@
       <c r="X33" t="inlineStr"/>
       <c r="Y33" t="inlineStr"/>
       <c r="Z33" t="inlineStr"/>
-      <c r="AA33" t="n">
-        <v>1</v>
-      </c>
+      <c r="AA33" t="inlineStr"/>
       <c r="AB33" t="inlineStr"/>
       <c r="AC33" t="inlineStr"/>
       <c r="AD33" t="inlineStr"/>

</xml_diff>

<commit_message>
lagaði hvernig open_excel er lesið
</commit_message>
<xml_diff>
--- a/03_26_schedule_results.xlsx
+++ b/03_26_schedule_results.xlsx
@@ -534,18 +534,18 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Thelma</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L2" t="n">
         <v>3</v>
@@ -554,7 +554,7 @@
         <v>40</v>
       </c>
       <c r="N2" t="n">
-        <v>90</v>
+        <v>230</v>
       </c>
     </row>
     <row r="3">
@@ -586,18 +586,18 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
         <v>3</v>
@@ -606,7 +606,7 @@
         <v>40</v>
       </c>
       <c r="N3" t="n">
-        <v>260</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4">
@@ -638,15 +638,15 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -658,7 +658,7 @@
         <v>100</v>
       </c>
       <c r="N4" t="n">
-        <v>240</v>
+        <v>260</v>
       </c>
     </row>
     <row r="5">
@@ -742,11 +742,11 @@
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J6" t="n">
@@ -846,18 +846,18 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J8" t="n">
         <v>2</v>
       </c>
       <c r="K8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L8" t="n">
         <v>3</v>
@@ -866,7 +866,7 @@
         <v>80</v>
       </c>
       <c r="N8" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
     </row>
     <row r="9">
@@ -898,18 +898,18 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J9" t="n">
         <v>1</v>
       </c>
       <c r="K9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L9" t="n">
         <v>3</v>
@@ -1002,18 +1002,18 @@
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J11" t="n">
         <v>2</v>
       </c>
       <c r="K11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
         <v>3</v>
@@ -1022,7 +1022,7 @@
         <v>40</v>
       </c>
       <c r="N11" t="n">
-        <v>180</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12">
@@ -1054,18 +1054,18 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Nanna</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L12" t="n">
         <v>3</v>
@@ -1074,7 +1074,7 @@
         <v>40</v>
       </c>
       <c r="N12" t="n">
-        <v>90</v>
+        <v>190</v>
       </c>
     </row>
     <row r="13">
@@ -1117,7 +1117,7 @@
         <v>3</v>
       </c>
       <c r="K13" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L13" t="n">
         <v>4</v>
@@ -1126,7 +1126,7 @@
         <v>70</v>
       </c>
       <c r="N13" t="n">
-        <v>70</v>
+        <v>170</v>
       </c>
     </row>
     <row r="14">
@@ -1178,7 +1178,7 @@
         <v>70</v>
       </c>
       <c r="N14" t="n">
-        <v>70</v>
+        <v>160</v>
       </c>
     </row>
     <row r="15">
@@ -1210,18 +1210,18 @@
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Thelma</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L15" t="n">
         <v>4</v>
@@ -1262,18 +1262,18 @@
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J16" t="n">
         <v>2</v>
       </c>
       <c r="K16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L16" t="n">
         <v>4</v>
@@ -1314,18 +1314,18 @@
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
         <v>4</v>
@@ -1366,18 +1366,18 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L18" t="n">
         <v>4</v>
@@ -1386,7 +1386,7 @@
         <v>70</v>
       </c>
       <c r="N18" t="n">
-        <v>70</v>
+        <v>170</v>
       </c>
     </row>
     <row r="19">
@@ -1418,18 +1418,18 @@
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J19" t="n">
         <v>2</v>
       </c>
       <c r="K19" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L19" t="n">
         <v>4</v>
@@ -1438,7 +1438,7 @@
         <v>70</v>
       </c>
       <c r="N19" t="n">
-        <v>160</v>
+        <v>170</v>
       </c>
     </row>
     <row r="20">
@@ -1470,18 +1470,18 @@
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J20" t="n">
         <v>2</v>
       </c>
       <c r="K20" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L20" t="n">
         <v>4</v>
@@ -1522,18 +1522,18 @@
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J21" t="n">
         <v>2</v>
       </c>
       <c r="K21" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L21" t="n">
         <v>4</v>
@@ -1574,18 +1574,18 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Anna</t>
+          <t>Bergur</t>
         </is>
       </c>
       <c r="J22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K22" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="L22" t="n">
         <v>4</v>
@@ -1637,7 +1637,7 @@
         <v>1</v>
       </c>
       <c r="K23" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L23" t="n">
         <v>4</v>
@@ -1750,7 +1750,7 @@
         <v>80</v>
       </c>
       <c r="N25" t="n">
-        <v>80</v>
+        <v>130</v>
       </c>
     </row>
     <row r="26">
@@ -1782,11 +1782,11 @@
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Pétur</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J26" t="n">
@@ -1834,11 +1834,11 @@
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J27" t="n">
@@ -1886,11 +1886,11 @@
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J28" t="n">
@@ -1938,18 +1938,18 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Pétur</t>
+          <t>Össur</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K29" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="L29" t="n">
         <v>3.5</v>
@@ -1958,7 +1958,7 @@
         <v>50</v>
       </c>
       <c r="N29" t="n">
-        <v>130</v>
+        <v>280</v>
       </c>
     </row>
     <row r="30">
@@ -1990,18 +1990,18 @@
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J30" t="n">
         <v>2</v>
       </c>
       <c r="K30" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L30" t="n">
         <v>3.5</v>
@@ -2010,7 +2010,7 @@
         <v>50</v>
       </c>
       <c r="N30" t="n">
-        <v>290</v>
+        <v>190</v>
       </c>
     </row>
     <row r="31">
@@ -2042,18 +2042,18 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J31" t="n">
         <v>2</v>
       </c>
       <c r="K31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L31" t="n">
         <v>3.5</v>
@@ -2062,7 +2062,7 @@
         <v>50</v>
       </c>
       <c r="N31" t="n">
-        <v>170</v>
+        <v>130</v>
       </c>
     </row>
     <row r="32">
@@ -2094,11 +2094,11 @@
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J32" t="n">
@@ -2114,7 +2114,7 @@
         <v>50</v>
       </c>
       <c r="N32" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
     </row>
     <row r="33">
@@ -2146,18 +2146,18 @@
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J33" t="n">
         <v>2</v>
       </c>
       <c r="K33" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="L33" t="n">
         <v>3.5</v>
@@ -2166,7 +2166,7 @@
         <v>50</v>
       </c>
       <c r="N33" t="n">
-        <v>300</v>
+        <v>250</v>
       </c>
     </row>
     <row r="34">
@@ -2198,18 +2198,18 @@
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L34" t="n">
         <v>3.5</v>
@@ -2218,7 +2218,7 @@
         <v>50</v>
       </c>
       <c r="N34" t="n">
-        <v>190</v>
+        <v>290</v>
       </c>
     </row>
     <row r="35">
@@ -2250,18 +2250,18 @@
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K35" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L35" t="n">
         <v>3.5</v>
@@ -2270,7 +2270,7 @@
         <v>50</v>
       </c>
       <c r="N35" t="n">
-        <v>290</v>
+        <v>200</v>
       </c>
     </row>
     <row r="36">
@@ -2302,18 +2302,18 @@
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K36" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L36" t="n">
         <v>3.5</v>
@@ -2322,7 +2322,7 @@
         <v>50</v>
       </c>
       <c r="N36" t="n">
-        <v>290</v>
+        <v>270</v>
       </c>
     </row>
     <row r="37">
@@ -2354,18 +2354,18 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K37" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L37" t="n">
         <v>3.5</v>
@@ -2374,7 +2374,7 @@
         <v>50</v>
       </c>
       <c r="N37" t="n">
-        <v>300</v>
+        <v>190</v>
       </c>
     </row>
     <row r="38">
@@ -2406,18 +2406,18 @@
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J38" t="n">
         <v>2</v>
       </c>
       <c r="K38" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="L38" t="n">
         <v>3.5</v>
@@ -2426,7 +2426,7 @@
         <v>50</v>
       </c>
       <c r="N38" t="n">
-        <v>150</v>
+        <v>290</v>
       </c>
     </row>
     <row r="39">
@@ -2458,18 +2458,18 @@
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Nanna</t>
+          <t>Anna</t>
         </is>
       </c>
       <c r="J39" t="n">
         <v>1</v>
       </c>
       <c r="K39" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L39" t="n">
         <v>3.5</v>
@@ -2530,7 +2530,7 @@
         <v>50</v>
       </c>
       <c r="N40" t="n">
-        <v>130</v>
+        <v>50</v>
       </c>
     </row>
     <row r="41">
@@ -2562,15 +2562,15 @@
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Helgi</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K41" t="n">
         <v>8</v>
@@ -2582,7 +2582,7 @@
         <v>50</v>
       </c>
       <c r="N41" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
     </row>
     <row r="42">
@@ -2614,15 +2614,15 @@
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Össur</t>
         </is>
       </c>
       <c r="J42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K42" t="n">
         <v>9</v>
@@ -2634,7 +2634,7 @@
         <v>50</v>
       </c>
       <c r="N42" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
     </row>
     <row r="43">
@@ -2666,18 +2666,18 @@
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Thelma</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K43" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="L43" t="n">
         <v>4</v>
@@ -2718,18 +2718,18 @@
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J44" t="n">
         <v>2</v>
       </c>
       <c r="K44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L44" t="n">
         <v>4</v>
@@ -2770,18 +2770,18 @@
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J45" t="n">
         <v>2</v>
       </c>
       <c r="K45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L45" t="n">
         <v>4</v>
@@ -2822,18 +2822,18 @@
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J46" t="n">
         <v>2</v>
       </c>
       <c r="K46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L46" t="n">
         <v>4</v>
@@ -2874,18 +2874,18 @@
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K47" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="L47" t="n">
         <v>4</v>
@@ -2894,7 +2894,7 @@
         <v>50</v>
       </c>
       <c r="N47" t="n">
-        <v>220</v>
+        <v>50</v>
       </c>
     </row>
     <row r="48">
@@ -3145,7 +3145,7 @@
         <v>3</v>
       </c>
       <c r="K52" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L52" t="n">
         <v>4</v>
@@ -3154,7 +3154,7 @@
         <v>50</v>
       </c>
       <c r="N52" t="n">
-        <v>220</v>
+        <v>100</v>
       </c>
     </row>
     <row r="53">
@@ -3186,18 +3186,18 @@
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
+        <v>6</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Unnur</t>
+        </is>
+      </c>
+      <c r="J53" t="n">
+        <v>2</v>
+      </c>
+      <c r="K53" t="n">
         <v>3</v>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>Össur</t>
-        </is>
-      </c>
-      <c r="J53" t="n">
-        <v>3</v>
-      </c>
-      <c r="K53" t="n">
-        <v>9</v>
       </c>
       <c r="L53" t="n">
         <v>4</v>
@@ -3206,7 +3206,7 @@
         <v>50</v>
       </c>
       <c r="N53" t="n">
-        <v>220</v>
+        <v>90</v>
       </c>
     </row>
     <row r="54">
@@ -3238,11 +3238,11 @@
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J54" t="n">
@@ -3290,18 +3290,18 @@
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K55" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="L55" t="n">
         <v>4</v>
@@ -3310,7 +3310,7 @@
         <v>50</v>
       </c>
       <c r="N55" t="n">
-        <v>120</v>
+        <v>220</v>
       </c>
     </row>
     <row r="56">
@@ -3353,7 +3353,7 @@
         <v>2</v>
       </c>
       <c r="K56" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L56" t="n">
         <v>4</v>
@@ -3405,7 +3405,7 @@
         <v>2</v>
       </c>
       <c r="K57" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L57" t="n">
         <v>4</v>
@@ -3414,7 +3414,7 @@
         <v>50</v>
       </c>
       <c r="N57" t="n">
-        <v>120</v>
+        <v>200</v>
       </c>
     </row>
     <row r="58">
@@ -3446,18 +3446,18 @@
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J58" t="n">
         <v>2</v>
       </c>
       <c r="K58" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L58" t="n">
         <v>4</v>
@@ -3466,7 +3466,7 @@
         <v>50</v>
       </c>
       <c r="N58" t="n">
-        <v>50</v>
+        <v>120</v>
       </c>
     </row>
     <row r="59">
@@ -3498,18 +3498,18 @@
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K59" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L59" t="n">
         <v>4</v>
@@ -3518,7 +3518,7 @@
         <v>50</v>
       </c>
       <c r="N59" t="n">
-        <v>250</v>
+        <v>50</v>
       </c>
     </row>
     <row r="60">
@@ -3665,7 +3665,7 @@
         <v>1</v>
       </c>
       <c r="K62" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L62" t="n">
         <v>4</v>
@@ -3706,11 +3706,11 @@
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J63" t="n">
@@ -3778,7 +3778,7 @@
         <v>70</v>
       </c>
       <c r="N64" t="n">
-        <v>140</v>
+        <v>120</v>
       </c>
     </row>
     <row r="65">
@@ -3810,11 +3810,11 @@
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J65" t="n">
@@ -3914,11 +3914,11 @@
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J67" t="n">
@@ -3966,11 +3966,11 @@
       </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J68" t="n">
@@ -4018,15 +4018,15 @@
       </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Helgi</t>
         </is>
       </c>
       <c r="J69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K69" t="n">
         <v>1</v>
@@ -4070,11 +4070,11 @@
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J70" t="n">
@@ -4090,7 +4090,7 @@
         <v>100</v>
       </c>
       <c r="N70" t="n">
-        <v>260</v>
+        <v>270</v>
       </c>
     </row>
     <row r="71">
@@ -4122,11 +4122,11 @@
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J71" t="n">
@@ -4142,7 +4142,7 @@
         <v>100</v>
       </c>
       <c r="N71" t="n">
-        <v>270</v>
+        <v>260</v>
       </c>
     </row>
     <row r="72">
@@ -4185,7 +4185,7 @@
         <v>3</v>
       </c>
       <c r="K72" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L72" t="n">
         <v>3.5</v>
@@ -4226,18 +4226,18 @@
       </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Helgi</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K73" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="L73" t="n">
         <v>3.5</v>
@@ -4246,7 +4246,7 @@
         <v>50</v>
       </c>
       <c r="N73" t="n">
-        <v>270</v>
+        <v>170</v>
       </c>
     </row>
     <row r="74">
@@ -4278,18 +4278,18 @@
       </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Össur</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J74" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K74" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L74" t="n">
         <v>3.5</v>
@@ -4330,18 +4330,18 @@
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Thelma</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J75" t="n">
+        <v>2</v>
+      </c>
+      <c r="K75" t="n">
         <v>3</v>
-      </c>
-      <c r="K75" t="n">
-        <v>7</v>
       </c>
       <c r="L75" t="n">
         <v>3.5</v>
@@ -4350,7 +4350,7 @@
         <v>50</v>
       </c>
       <c r="N75" t="n">
-        <v>260</v>
+        <v>170</v>
       </c>
     </row>
     <row r="76">
@@ -4382,18 +4382,18 @@
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J76" t="n">
         <v>2</v>
       </c>
       <c r="K76" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L76" t="n">
         <v>3.5</v>
@@ -4402,7 +4402,7 @@
         <v>50</v>
       </c>
       <c r="N76" t="n">
-        <v>170</v>
+        <v>250</v>
       </c>
     </row>
     <row r="77">
@@ -4434,18 +4434,18 @@
       </c>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J77" t="n">
         <v>2</v>
       </c>
       <c r="K77" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L77" t="n">
         <v>3.5</v>
@@ -4486,11 +4486,11 @@
       </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J78" t="n">
@@ -4538,18 +4538,18 @@
       </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K79" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="L79" t="n">
         <v>3.5</v>
@@ -4558,7 +4558,7 @@
         <v>50</v>
       </c>
       <c r="N79" t="n">
-        <v>170</v>
+        <v>290</v>
       </c>
     </row>
     <row r="80">
@@ -4590,18 +4590,18 @@
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Camilla</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J80" t="n">
         <v>1</v>
       </c>
       <c r="K80" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L80" t="n">
         <v>3.5</v>
@@ -4642,18 +4642,18 @@
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Ólafur</t>
+          <t>Camilla</t>
         </is>
       </c>
       <c r="J81" t="n">
         <v>1</v>
       </c>
       <c r="K81" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L81" t="n">
         <v>3.5</v>
@@ -4662,7 +4662,7 @@
         <v>50</v>
       </c>
       <c r="N81" t="n">
-        <v>150</v>
+        <v>250</v>
       </c>
     </row>
     <row r="82">
@@ -4694,18 +4694,18 @@
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Bergur</t>
+          <t>Ólafur</t>
         </is>
       </c>
       <c r="J82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K82" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L82" t="n">
         <v>3.5</v>
@@ -4714,7 +4714,7 @@
         <v>50</v>
       </c>
       <c r="N82" t="n">
-        <v>270</v>
+        <v>150</v>
       </c>
     </row>
     <row r="83">
@@ -4798,11 +4798,11 @@
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Pétur</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J84" t="n">
@@ -4850,18 +4850,18 @@
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J85" t="n">
         <v>2</v>
       </c>
       <c r="K85" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L85" t="n">
         <v>4</v>
@@ -4870,7 +4870,7 @@
         <v>50</v>
       </c>
       <c r="N85" t="n">
-        <v>230</v>
+        <v>220</v>
       </c>
     </row>
     <row r="86">
@@ -4902,18 +4902,18 @@
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J86" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K86" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L86" t="n">
         <v>4</v>
@@ -4922,7 +4922,7 @@
         <v>50</v>
       </c>
       <c r="N86" t="n">
-        <v>200</v>
+        <v>220</v>
       </c>
     </row>
     <row r="87">
@@ -4954,11 +4954,11 @@
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J87" t="n">
@@ -4974,7 +4974,7 @@
         <v>50</v>
       </c>
       <c r="N87" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="88">
@@ -5006,11 +5006,11 @@
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J88" t="n">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J89" t="n">
@@ -5110,11 +5110,11 @@
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J90" t="n">
@@ -5162,11 +5162,11 @@
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J91" t="n">
@@ -5214,18 +5214,18 @@
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Nanna</t>
         </is>
       </c>
       <c r="J92" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K92" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L92" t="n">
         <v>4</v>
@@ -5234,7 +5234,7 @@
         <v>50</v>
       </c>
       <c r="N92" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="93">
@@ -5266,18 +5266,18 @@
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>Nanna</t>
+          <t>Anna</t>
         </is>
       </c>
       <c r="J93" t="n">
         <v>1</v>
       </c>
       <c r="K93" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L93" t="n">
         <v>4</v>
@@ -5286,7 +5286,7 @@
         <v>50</v>
       </c>
       <c r="N93" t="n">
-        <v>50</v>
+        <v>220</v>
       </c>
     </row>
     <row r="94">
@@ -5318,18 +5318,18 @@
       </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>Anna</t>
+          <t>Bergur</t>
         </is>
       </c>
       <c r="J94" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K94" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L94" t="n">
         <v>4</v>
@@ -5338,7 +5338,7 @@
         <v>50</v>
       </c>
       <c r="N94" t="n">
-        <v>220</v>
+        <v>100</v>
       </c>
     </row>
     <row r="95">
@@ -5370,15 +5370,15 @@
       </c>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J95" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K95" t="n">
         <v>0</v>
@@ -5390,7 +5390,7 @@
         <v>80</v>
       </c>
       <c r="N95" t="n">
-        <v>150</v>
+        <v>130</v>
       </c>
     </row>
     <row r="96">
@@ -5422,15 +5422,15 @@
       </c>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Össur</t>
         </is>
       </c>
       <c r="J96" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K96" t="n">
         <v>1</v>
@@ -5442,7 +5442,7 @@
         <v>40</v>
       </c>
       <c r="N96" t="n">
-        <v>180</v>
+        <v>90</v>
       </c>
     </row>
     <row r="97">
@@ -5474,11 +5474,11 @@
       </c>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J97" t="n">
@@ -5494,7 +5494,7 @@
         <v>40</v>
       </c>
       <c r="N97" t="n">
-        <v>90</v>
+        <v>40</v>
       </c>
     </row>
     <row r="98">
@@ -5526,18 +5526,18 @@
       </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="n">
+        <v>4</v>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Thelma</t>
+        </is>
+      </c>
+      <c r="J98" t="n">
+        <v>3</v>
+      </c>
+      <c r="K98" t="n">
         <v>5</v>
-      </c>
-      <c r="I98" t="inlineStr">
-        <is>
-          <t>Pétur</t>
-        </is>
-      </c>
-      <c r="J98" t="n">
-        <v>2</v>
-      </c>
-      <c r="K98" t="n">
-        <v>8</v>
       </c>
       <c r="L98" t="n">
         <v>3</v>
@@ -5546,7 +5546,7 @@
         <v>70</v>
       </c>
       <c r="N98" t="n">
-        <v>320</v>
+        <v>300</v>
       </c>
     </row>
     <row r="99">
@@ -5578,11 +5578,11 @@
       </c>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J99" t="n">
@@ -5598,7 +5598,7 @@
         <v>70</v>
       </c>
       <c r="N99" t="n">
-        <v>140</v>
+        <v>160</v>
       </c>
     </row>
     <row r="100">
@@ -5630,11 +5630,11 @@
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J100" t="n">
@@ -5650,7 +5650,7 @@
         <v>70</v>
       </c>
       <c r="N100" t="n">
-        <v>140</v>
+        <v>160</v>
       </c>
     </row>
     <row r="101">
@@ -5682,18 +5682,18 @@
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J101" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K101" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L101" t="n">
         <v>3</v>
@@ -5702,7 +5702,7 @@
         <v>70</v>
       </c>
       <c r="N101" t="n">
-        <v>270</v>
+        <v>320</v>
       </c>
     </row>
     <row r="102">
@@ -5734,18 +5734,18 @@
       </c>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J102" t="n">
         <v>2</v>
       </c>
       <c r="K102" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L102" t="n">
         <v>3</v>
@@ -5754,7 +5754,7 @@
         <v>70</v>
       </c>
       <c r="N102" t="n">
-        <v>320</v>
+        <v>310</v>
       </c>
     </row>
     <row r="103">
@@ -5786,18 +5786,18 @@
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K103" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L103" t="n">
         <v>3</v>
@@ -5806,7 +5806,7 @@
         <v>70</v>
       </c>
       <c r="N103" t="n">
-        <v>140</v>
+        <v>320</v>
       </c>
     </row>
     <row r="104">
@@ -5838,18 +5838,18 @@
       </c>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J104" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K104" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L104" t="n">
         <v>3</v>
@@ -5858,7 +5858,7 @@
         <v>70</v>
       </c>
       <c r="N104" t="n">
-        <v>310</v>
+        <v>320</v>
       </c>
     </row>
     <row r="105">
@@ -5890,18 +5890,18 @@
       </c>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Camilla</t>
+          <t>Ólafur</t>
         </is>
       </c>
       <c r="J105" t="n">
         <v>1</v>
       </c>
       <c r="K105" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="L105" t="n">
         <v>3</v>
@@ -5910,7 +5910,7 @@
         <v>70</v>
       </c>
       <c r="N105" t="n">
-        <v>320</v>
+        <v>290</v>
       </c>
     </row>
     <row r="106">
@@ -5942,18 +5942,18 @@
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>Ólafur</t>
+          <t>Anna</t>
         </is>
       </c>
       <c r="J106" t="n">
         <v>1</v>
       </c>
       <c r="K106" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L106" t="n">
         <v>3</v>
@@ -5962,7 +5962,7 @@
         <v>70</v>
       </c>
       <c r="N106" t="n">
-        <v>290</v>
+        <v>170</v>
       </c>
     </row>
     <row r="107">
@@ -5994,18 +5994,18 @@
       </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>Anna</t>
+          <t>Bergur</t>
         </is>
       </c>
       <c r="J107" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K107" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L107" t="n">
         <v>3</v>
@@ -6014,7 +6014,7 @@
         <v>70</v>
       </c>
       <c r="N107" t="n">
-        <v>290</v>
+        <v>310</v>
       </c>
     </row>
     <row r="108">
@@ -6057,7 +6057,7 @@
         <v>1</v>
       </c>
       <c r="K108" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L108" t="n">
         <v>3</v>
@@ -6098,11 +6098,11 @@
       </c>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J109" t="n">
@@ -6118,7 +6118,7 @@
         <v>90</v>
       </c>
       <c r="N109" t="n">
-        <v>250</v>
+        <v>260</v>
       </c>
     </row>
     <row r="110">
@@ -6150,18 +6150,18 @@
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Helgi</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J110" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K110" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L110" t="n">
         <v>4</v>
@@ -6202,18 +6202,18 @@
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="n">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Nanna</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J111" t="n">
         <v>1</v>
       </c>
       <c r="K111" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L111" t="n">
         <v>4</v>
@@ -6222,7 +6222,7 @@
         <v>100</v>
       </c>
       <c r="N111" t="n">
-        <v>150</v>
+        <v>170</v>
       </c>
     </row>
     <row r="112">
@@ -6254,18 +6254,18 @@
       </c>
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Bergur</t>
+          <t>Nanna</t>
         </is>
       </c>
       <c r="J112" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K112" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L112" t="n">
         <v>4</v>
@@ -6369,7 +6369,7 @@
         <v>3</v>
       </c>
       <c r="K114" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="L114" t="n">
         <v>4</v>
@@ -6378,7 +6378,7 @@
         <v>70</v>
       </c>
       <c r="N114" t="n">
-        <v>210</v>
+        <v>190</v>
       </c>
     </row>
     <row r="115">
@@ -6410,18 +6410,18 @@
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J115" t="n">
         <v>2</v>
       </c>
       <c r="K115" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L115" t="n">
         <v>4</v>
@@ -6430,7 +6430,7 @@
         <v>70</v>
       </c>
       <c r="N115" t="n">
-        <v>70</v>
+        <v>140</v>
       </c>
     </row>
     <row r="116">
@@ -6473,7 +6473,7 @@
         <v>2</v>
       </c>
       <c r="K116" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="L116" t="n">
         <v>4</v>
@@ -6482,7 +6482,7 @@
         <v>70</v>
       </c>
       <c r="N116" t="n">
-        <v>70</v>
+        <v>200</v>
       </c>
     </row>
     <row r="117">
@@ -6514,18 +6514,18 @@
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J117" t="n">
         <v>2</v>
       </c>
       <c r="K117" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L117" t="n">
         <v>4</v>
@@ -6534,7 +6534,7 @@
         <v>70</v>
       </c>
       <c r="N117" t="n">
-        <v>160</v>
+        <v>70</v>
       </c>
     </row>
     <row r="118">
@@ -6566,18 +6566,18 @@
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J118" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K118" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L118" t="n">
         <v>4</v>
@@ -6618,18 +6618,18 @@
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J119" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K119" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L119" t="n">
         <v>4</v>
@@ -6638,7 +6638,7 @@
         <v>70</v>
       </c>
       <c r="N119" t="n">
-        <v>170</v>
+        <v>70</v>
       </c>
     </row>
     <row r="120">
@@ -6670,18 +6670,18 @@
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J120" t="n">
         <v>2</v>
       </c>
       <c r="K120" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L120" t="n">
         <v>4</v>
@@ -6878,18 +6878,18 @@
       </c>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Pétur</t>
+          <t>Össur</t>
         </is>
       </c>
       <c r="J124" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K124" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="L124" t="n">
         <v>2</v>
@@ -6898,7 +6898,7 @@
         <v>70</v>
       </c>
       <c r="N124" t="n">
-        <v>250</v>
+        <v>230</v>
       </c>
     </row>
     <row r="125">
@@ -6930,18 +6930,18 @@
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J125" t="n">
         <v>2</v>
       </c>
       <c r="K125" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="L125" t="n">
         <v>2</v>
@@ -6950,7 +6950,7 @@
         <v>70</v>
       </c>
       <c r="N125" t="n">
-        <v>240</v>
+        <v>250</v>
       </c>
     </row>
     <row r="126">
@@ -6982,18 +6982,18 @@
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J126" t="n">
         <v>2</v>
       </c>
       <c r="K126" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L126" t="n">
         <v>2</v>
@@ -7034,18 +7034,18 @@
       </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J127" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K127" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L127" t="n">
         <v>2</v>
@@ -7054,7 +7054,7 @@
         <v>70</v>
       </c>
       <c r="N127" t="n">
-        <v>250</v>
+        <v>70</v>
       </c>
     </row>
     <row r="128">
@@ -7097,7 +7097,7 @@
         <v>2</v>
       </c>
       <c r="K128" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L128" t="n">
         <v>2</v>
@@ -7106,7 +7106,7 @@
         <v>70</v>
       </c>
       <c r="N128" t="n">
-        <v>70</v>
+        <v>240</v>
       </c>
     </row>
     <row r="129">
@@ -7138,18 +7138,18 @@
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J129" t="n">
         <v>2</v>
       </c>
       <c r="K129" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L129" t="n">
         <v>2</v>
@@ -7201,7 +7201,7 @@
         <v>2</v>
       </c>
       <c r="K130" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L130" t="n">
         <v>2</v>
@@ -7210,7 +7210,7 @@
         <v>70</v>
       </c>
       <c r="N130" t="n">
-        <v>160</v>
+        <v>70</v>
       </c>
     </row>
     <row r="131">
@@ -7242,18 +7242,18 @@
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J131" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K131" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L131" t="n">
         <v>2</v>
@@ -7294,18 +7294,18 @@
       </c>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J132" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K132" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L132" t="n">
         <v>2</v>
@@ -7314,7 +7314,7 @@
         <v>70</v>
       </c>
       <c r="N132" t="n">
-        <v>70</v>
+        <v>240</v>
       </c>
     </row>
     <row r="133">
@@ -7357,7 +7357,7 @@
         <v>1</v>
       </c>
       <c r="K133" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L133" t="n">
         <v>2</v>
@@ -7366,7 +7366,7 @@
         <v>70</v>
       </c>
       <c r="N133" t="n">
-        <v>220</v>
+        <v>260</v>
       </c>
     </row>
     <row r="134">
@@ -7409,7 +7409,7 @@
         <v>2</v>
       </c>
       <c r="K134" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L134" t="n">
         <v>2</v>
@@ -7418,7 +7418,7 @@
         <v>70</v>
       </c>
       <c r="N134" t="n">
-        <v>220</v>
+        <v>240</v>
       </c>
     </row>
     <row r="135">
@@ -7450,11 +7450,11 @@
       </c>
       <c r="G135" t="inlineStr"/>
       <c r="H135" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J135" t="n">
@@ -7470,7 +7470,7 @@
         <v>90</v>
       </c>
       <c r="N135" t="n">
-        <v>240</v>
+        <v>200</v>
       </c>
     </row>
     <row r="136">
@@ -7502,15 +7502,15 @@
       </c>
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Össur</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J136" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K136" t="n">
         <v>1</v>
@@ -7554,11 +7554,11 @@
       </c>
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J137" t="n">
@@ -7812,17 +7812,19 @@
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" t="n">
+        <v>1</v>
+      </c>
       <c r="L3" t="n">
         <v>1</v>
       </c>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+      <c r="N3" t="n">
+        <v>1</v>
+      </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
@@ -7830,9 +7832,7 @@
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr"/>
@@ -7855,52 +7855,56 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="n">
-        <v>1</v>
-      </c>
+      <c r="J4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
+      <c r="T4" t="n">
+        <v>1</v>
+      </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
+      <c r="AA4" t="n">
+        <v>1</v>
+      </c>
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
       <c r="AD4" t="inlineStr"/>
       <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="n">
-        <v>1</v>
-      </c>
+      <c r="AF4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr"/>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
-      <c r="E5" t="n">
-        <v>1</v>
-      </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
         <v>1</v>
@@ -7908,13 +7912,13 @@
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
+      <c r="U5" t="n">
+        <v>1</v>
+      </c>
       <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr"/>
@@ -7935,28 +7939,28 @@
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
       <c r="E6" t="inlineStr"/>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+      <c r="O6" t="n">
+        <v>1</v>
+      </c>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
-      <c r="S6" t="n">
-        <v>1</v>
-      </c>
+      <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="n">
         <v>1</v>
@@ -7966,9 +7970,7 @@
       <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="n">
-        <v>1</v>
-      </c>
+      <c r="AA6" t="inlineStr"/>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="inlineStr"/>
@@ -7979,19 +7981,17 @@
       <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" t="n">
-        <v>1</v>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
-      <c r="J7" t="n">
-        <v>1</v>
-      </c>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
         <v>1</v>
@@ -8000,21 +8000,21 @@
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
+      <c r="T7" t="n">
+        <v>1</v>
+      </c>
+      <c r="U7" t="n">
+        <v>1</v>
+      </c>
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="n">
-        <v>1</v>
-      </c>
+      <c r="AA7" t="inlineStr"/>
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr"/>
@@ -8026,11 +8026,11 @@
         <v>7</v>
       </c>
       <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
       <c r="D8" t="inlineStr"/>
-      <c r="E8" t="n">
-        <v>1</v>
-      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
@@ -8039,10 +8039,10 @@
         <v>1</v>
       </c>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" t="n">
-        <v>1</v>
-      </c>
-      <c r="M8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="n">
+        <v>1</v>
+      </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
@@ -8055,10 +8055,10 @@
       <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr"/>
-      <c r="Z8" t="inlineStr"/>
-      <c r="AA8" t="n">
-        <v>1</v>
-      </c>
+      <c r="Z8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA8" t="inlineStr"/>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr"/>
@@ -8071,11 +8071,11 @@
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
-      <c r="D9" t="n">
-        <v>1</v>
-      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
@@ -8084,9 +8084,7 @@
       </c>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
-      <c r="M9" t="n">
-        <v>1</v>
-      </c>
+      <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
@@ -8104,7 +8102,9 @@
       <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
-      <c r="AA9" t="inlineStr"/>
+      <c r="AA9" t="n">
+        <v>1</v>
+      </c>
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="inlineStr"/>
@@ -8123,23 +8123,23 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" t="n">
-        <v>1</v>
-      </c>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
       <c r="M10" t="n">
         <v>1</v>
       </c>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
+      <c r="Q10" t="n">
+        <v>1</v>
+      </c>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
-      <c r="T10" t="n">
-        <v>1</v>
-      </c>
+      <c r="T10" t="inlineStr"/>
       <c r="U10" t="n">
         <v>1</v>
       </c>
@@ -8164,72 +8164,72 @@
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="n">
-        <v>1</v>
-      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="n">
-        <v>1</v>
-      </c>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
+      <c r="S11" t="n">
+        <v>1</v>
+      </c>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr"/>
-      <c r="Z11" t="n">
-        <v>1</v>
-      </c>
+      <c r="Z11" t="inlineStr"/>
       <c r="AA11" t="inlineStr"/>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="inlineStr"/>
       <c r="AE11" t="inlineStr"/>
-      <c r="AF11" t="inlineStr"/>
+      <c r="AF11" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
         <v>11</v>
       </c>
       <c r="B12" t="inlineStr"/>
-      <c r="C12" t="n">
-        <v>1</v>
-      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
       <c r="L12" t="inlineStr"/>
-      <c r="M12" t="n">
-        <v>1</v>
-      </c>
+      <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
-      <c r="S12" t="n">
-        <v>1</v>
-      </c>
-      <c r="T12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="n">
+        <v>1</v>
+      </c>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
@@ -8252,42 +8252,42 @@
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
-      <c r="E13" t="n">
-        <v>1</v>
-      </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
-      <c r="K13" t="n">
-        <v>1</v>
-      </c>
-      <c r="L13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="n">
+        <v>1</v>
+      </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
+      <c r="Q13" t="n">
+        <v>1</v>
+      </c>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
-      <c r="T13" t="n">
-        <v>1</v>
-      </c>
-      <c r="U13" t="n">
-        <v>1</v>
-      </c>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr"/>
       <c r="X13" t="inlineStr"/>
       <c r="Y13" t="inlineStr"/>
       <c r="Z13" t="inlineStr"/>
-      <c r="AA13" t="inlineStr"/>
+      <c r="AA13" t="n">
+        <v>1</v>
+      </c>
       <c r="AB13" t="inlineStr"/>
       <c r="AC13" t="inlineStr"/>
       <c r="AD13" t="inlineStr"/>
       <c r="AE13" t="inlineStr"/>
-      <c r="AF13" t="inlineStr"/>
+      <c r="AF13" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -8296,20 +8296,22 @@
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
+      <c r="J14" t="n">
+        <v>1</v>
+      </c>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="n">
         <v>1</v>
       </c>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" t="n">
-        <v>1</v>
-      </c>
+      <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="n">
@@ -8341,7 +8343,9 @@
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
@@ -8352,9 +8356,7 @@
       </c>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
-      <c r="O15" t="n">
-        <v>1</v>
-      </c>
+      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="n">
         <v>1</v>
@@ -8367,10 +8369,10 @@
       <c r="W15" t="inlineStr"/>
       <c r="X15" t="inlineStr"/>
       <c r="Y15" t="inlineStr"/>
-      <c r="Z15" t="inlineStr"/>
-      <c r="AA15" t="n">
-        <v>1</v>
-      </c>
+      <c r="Z15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA15" t="inlineStr"/>
       <c r="AB15" t="inlineStr"/>
       <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="inlineStr"/>
@@ -8383,30 +8385,32 @@
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
-      <c r="D16" t="n">
-        <v>1</v>
-      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="n">
-        <v>1</v>
-      </c>
+      <c r="J16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="n">
-        <v>1</v>
-      </c>
+      <c r="M16" t="n">
+        <v>1</v>
+      </c>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
+      <c r="Q16" t="n">
+        <v>1</v>
+      </c>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
+      <c r="U16" t="n">
+        <v>1</v>
+      </c>
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
       <c r="X16" t="inlineStr"/>
@@ -8428,39 +8432,37 @@
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="n">
-        <v>1</v>
-      </c>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
-      <c r="K17" t="n">
-        <v>1</v>
-      </c>
-      <c r="L17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="n">
+        <v>1</v>
+      </c>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
+      <c r="N17" t="n">
+        <v>1</v>
+      </c>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
+      <c r="Q17" t="n">
+        <v>1</v>
+      </c>
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
-      <c r="T17" t="n">
-        <v>1</v>
-      </c>
-      <c r="U17" t="n">
-        <v>1</v>
-      </c>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr"/>
-      <c r="X17" t="n">
-        <v>1</v>
-      </c>
+      <c r="X17" t="inlineStr"/>
       <c r="Y17" t="inlineStr"/>
       <c r="Z17" t="inlineStr"/>
-      <c r="AA17" t="inlineStr"/>
+      <c r="AA17" t="n">
+        <v>1</v>
+      </c>
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="inlineStr"/>
@@ -8490,9 +8492,7 @@
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
-      <c r="S18" t="n">
-        <v>1</v>
-      </c>
+      <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr"/>
@@ -8506,7 +8506,9 @@
       <c r="AB18" t="inlineStr"/>
       <c r="AC18" t="inlineStr"/>
       <c r="AD18" t="inlineStr"/>
-      <c r="AE18" t="inlineStr"/>
+      <c r="AE18" t="n">
+        <v>1</v>
+      </c>
       <c r="AF18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -8514,11 +8516,11 @@
         <v>18</v>
       </c>
       <c r="B19" t="inlineStr"/>
-      <c r="C19" t="n">
-        <v>1</v>
-      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
@@ -8528,23 +8530,23 @@
       </c>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
-      <c r="M19" t="n">
-        <v>1</v>
-      </c>
+      <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
+      <c r="S19" t="n">
+        <v>1</v>
+      </c>
       <c r="T19" t="inlineStr"/>
-      <c r="U19" t="n">
-        <v>1</v>
-      </c>
+      <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr"/>
       <c r="X19" t="inlineStr"/>
-      <c r="Y19" t="inlineStr"/>
+      <c r="Y19" t="n">
+        <v>1</v>
+      </c>
       <c r="Z19" t="inlineStr"/>
       <c r="AA19" t="inlineStr"/>
       <c r="AB19" t="inlineStr"/>
@@ -8557,9 +8559,7 @@
       <c r="A20" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="n">
-        <v>1</v>
-      </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
@@ -8567,9 +8567,7 @@
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
-      <c r="J20" t="n">
-        <v>1</v>
-      </c>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -8578,7 +8576,9 @@
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
+      <c r="Q20" t="n">
+        <v>1</v>
+      </c>
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr"/>
@@ -8586,11 +8586,13 @@
       <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr"/>
       <c r="X20" t="inlineStr"/>
-      <c r="Y20" t="inlineStr"/>
-      <c r="Z20" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA20" t="inlineStr"/>
+      <c r="Y20" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z20" t="inlineStr"/>
+      <c r="AA20" t="n">
+        <v>1</v>
+      </c>
       <c r="AB20" t="inlineStr"/>
       <c r="AC20" t="inlineStr"/>
       <c r="AD20" t="inlineStr"/>
@@ -8610,9 +8612,7 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" t="n">
-        <v>1</v>
-      </c>
+      <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="n">
         <v>1</v>
@@ -8631,7 +8631,9 @@
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
-      <c r="X21" t="inlineStr"/>
+      <c r="X21" t="n">
+        <v>1</v>
+      </c>
       <c r="Y21" t="inlineStr"/>
       <c r="Z21" t="inlineStr"/>
       <c r="AA21" t="inlineStr"/>
@@ -8654,10 +8656,10 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="n">
-        <v>1</v>
-      </c>
+      <c r="I22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" t="inlineStr"/>
       <c r="K22" t="n">
         <v>1</v>
       </c>
@@ -8678,9 +8680,7 @@
       <c r="X22" t="inlineStr"/>
       <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="inlineStr"/>
-      <c r="AA22" t="n">
-        <v>1</v>
-      </c>
+      <c r="AA22" t="inlineStr"/>
       <c r="AB22" t="inlineStr"/>
       <c r="AC22" t="inlineStr"/>
       <c r="AD22" t="inlineStr"/>
@@ -8691,22 +8691,24 @@
       <c r="A23" t="n">
         <v>22</v>
       </c>
-      <c r="B23" t="n">
-        <v>1</v>
-      </c>
-      <c r="C23" t="inlineStr"/>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="n">
-        <v>1</v>
-      </c>
+      <c r="J23" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
+      <c r="M23" t="n">
+        <v>1</v>
+      </c>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
@@ -8719,17 +8721,15 @@
       <c r="W23" t="inlineStr"/>
       <c r="X23" t="inlineStr"/>
       <c r="Y23" t="inlineStr"/>
-      <c r="Z23" t="inlineStr"/>
-      <c r="AA23" t="n">
-        <v>1</v>
-      </c>
+      <c r="Z23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA23" t="inlineStr"/>
       <c r="AB23" t="inlineStr"/>
       <c r="AC23" t="inlineStr"/>
       <c r="AD23" t="inlineStr"/>
       <c r="AE23" t="inlineStr"/>
-      <c r="AF23" t="n">
-        <v>1</v>
-      </c>
+      <c r="AF23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -8745,9 +8745,7 @@
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" t="n">
-        <v>1</v>
-      </c>
+      <c r="J24" t="inlineStr"/>
       <c r="K24" t="n">
         <v>1</v>
       </c>
@@ -8781,17 +8779,19 @@
       <c r="A25" t="n">
         <v>24</v>
       </c>
-      <c r="B25" t="inlineStr"/>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" t="n">
-        <v>1</v>
-      </c>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="n">
         <v>1</v>
       </c>
@@ -8806,9 +8806,7 @@
         <v>1</v>
       </c>
       <c r="T25" t="inlineStr"/>
-      <c r="U25" t="n">
-        <v>1</v>
-      </c>
+      <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr"/>
       <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr"/>
@@ -8818,26 +8816,26 @@
       <c r="AB25" t="inlineStr"/>
       <c r="AC25" t="inlineStr"/>
       <c r="AD25" t="inlineStr"/>
-      <c r="AE25" t="n">
-        <v>1</v>
-      </c>
+      <c r="AE25" t="inlineStr"/>
       <c r="AF25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="n">
-        <v>1</v>
-      </c>
+      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
+      <c r="J26" t="n">
+        <v>1</v>
+      </c>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="n">
         <v>1</v>
@@ -8857,10 +8855,10 @@
       <c r="W26" t="inlineStr"/>
       <c r="X26" t="inlineStr"/>
       <c r="Y26" t="inlineStr"/>
-      <c r="Z26" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="n">
+        <v>1</v>
+      </c>
       <c r="AB26" t="inlineStr"/>
       <c r="AC26" t="inlineStr"/>
       <c r="AD26" t="inlineStr"/>
@@ -8885,18 +8883,20 @@
       <c r="K27" t="n">
         <v>1</v>
       </c>
-      <c r="L27" t="n">
-        <v>1</v>
-      </c>
+      <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
+      <c r="Q27" t="n">
+        <v>1</v>
+      </c>
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr"/>
-      <c r="U27" t="inlineStr"/>
+      <c r="U27" t="n">
+        <v>1</v>
+      </c>
       <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr"/>
@@ -8940,9 +8940,7 @@
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr"/>
-      <c r="U28" t="n">
-        <v>1</v>
-      </c>
+      <c r="U28" t="inlineStr"/>
       <c r="V28" t="inlineStr"/>
       <c r="W28" t="inlineStr"/>
       <c r="X28" t="inlineStr"/>
@@ -8963,15 +8961,15 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" t="n">
-        <v>1</v>
-      </c>
+      <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
@@ -9052,14 +9050,14 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" t="n">
-        <v>1</v>
-      </c>
+      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
+      <c r="J31" t="n">
+        <v>1</v>
+      </c>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="n">
         <v>1</v>
@@ -9096,7 +9094,9 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="n">
+        <v>1</v>
+      </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
@@ -9110,19 +9110,19 @@
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
+      <c r="S32" t="n">
+        <v>1</v>
+      </c>
       <c r="T32" t="inlineStr"/>
-      <c r="U32" t="inlineStr"/>
+      <c r="U32" t="n">
+        <v>1</v>
+      </c>
       <c r="V32" t="inlineStr"/>
       <c r="W32" t="inlineStr"/>
       <c r="X32" t="inlineStr"/>
-      <c r="Y32" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y32" t="inlineStr"/>
       <c r="Z32" t="inlineStr"/>
       <c r="AA32" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
lagaði hvernig json skjöl eru sótt
færði json skjöl í data möppuna - lagaði þannig að greedy ætti að sækja skjölin rétt núna
</commit_message>
<xml_diff>
--- a/03_26_schedule_results.xlsx
+++ b/03_26_schedule_results.xlsx
@@ -534,18 +534,18 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Thelma</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>3</v>
@@ -554,7 +554,7 @@
         <v>40</v>
       </c>
       <c r="N2" t="n">
-        <v>230</v>
+        <v>370</v>
       </c>
     </row>
     <row r="3">
@@ -586,18 +586,18 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L3" t="n">
         <v>3</v>
@@ -606,7 +606,7 @@
         <v>40</v>
       </c>
       <c r="N3" t="n">
-        <v>110</v>
+        <v>480</v>
       </c>
     </row>
     <row r="4">
@@ -638,15 +638,15 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -658,7 +658,7 @@
         <v>100</v>
       </c>
       <c r="N4" t="n">
-        <v>260</v>
+        <v>440</v>
       </c>
     </row>
     <row r="5">
@@ -690,18 +690,18 @@
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Helgi</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L5" t="n">
         <v>3</v>
@@ -710,7 +710,7 @@
         <v>80</v>
       </c>
       <c r="N5" t="n">
-        <v>250</v>
+        <v>470</v>
       </c>
     </row>
     <row r="6">
@@ -742,18 +742,18 @@
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Thelma</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L6" t="n">
         <v>3</v>
@@ -762,7 +762,7 @@
         <v>80</v>
       </c>
       <c r="N6" t="n">
-        <v>250</v>
+        <v>410</v>
       </c>
     </row>
     <row r="7">
@@ -794,11 +794,11 @@
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J7" t="n">
@@ -814,7 +814,7 @@
         <v>80</v>
       </c>
       <c r="N7" t="n">
-        <v>130</v>
+        <v>360</v>
       </c>
     </row>
     <row r="8">
@@ -846,11 +846,11 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J8" t="n">
@@ -866,7 +866,7 @@
         <v>80</v>
       </c>
       <c r="N8" t="n">
-        <v>270</v>
+        <v>470</v>
       </c>
     </row>
     <row r="9">
@@ -898,15 +898,15 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" t="n">
         <v>2</v>
@@ -918,7 +918,7 @@
         <v>80</v>
       </c>
       <c r="N9" t="n">
-        <v>270</v>
+        <v>470</v>
       </c>
     </row>
     <row r="10">
@@ -950,11 +950,11 @@
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Camilla</t>
+          <t>Anna</t>
         </is>
       </c>
       <c r="J10" t="n">
@@ -970,7 +970,7 @@
         <v>80</v>
       </c>
       <c r="N10" t="n">
-        <v>130</v>
+        <v>360</v>
       </c>
     </row>
     <row r="11">
@@ -1002,18 +1002,18 @@
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Pétur</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J11" t="n">
         <v>2</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L11" t="n">
         <v>3</v>
@@ -1022,7 +1022,7 @@
         <v>40</v>
       </c>
       <c r="N11" t="n">
-        <v>90</v>
+        <v>440</v>
       </c>
     </row>
     <row r="12">
@@ -1054,18 +1054,18 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Nanna</t>
+          <t>Bergur</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
         <v>3</v>
@@ -1074,7 +1074,7 @@
         <v>40</v>
       </c>
       <c r="N12" t="n">
-        <v>190</v>
+        <v>360</v>
       </c>
     </row>
     <row r="13">
@@ -1117,7 +1117,7 @@
         <v>3</v>
       </c>
       <c r="K13" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L13" t="n">
         <v>4</v>
@@ -1126,7 +1126,7 @@
         <v>70</v>
       </c>
       <c r="N13" t="n">
-        <v>170</v>
+        <v>340</v>
       </c>
     </row>
     <row r="14">
@@ -1178,7 +1178,7 @@
         <v>70</v>
       </c>
       <c r="N14" t="n">
-        <v>160</v>
+        <v>420</v>
       </c>
     </row>
     <row r="15">
@@ -1210,11 +1210,11 @@
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J15" t="n">
@@ -1230,7 +1230,7 @@
         <v>70</v>
       </c>
       <c r="N15" t="n">
-        <v>70</v>
+        <v>340</v>
       </c>
     </row>
     <row r="16">
@@ -1273,7 +1273,7 @@
         <v>2</v>
       </c>
       <c r="K16" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L16" t="n">
         <v>4</v>
@@ -1282,7 +1282,7 @@
         <v>70</v>
       </c>
       <c r="N16" t="n">
-        <v>70</v>
+        <v>480</v>
       </c>
     </row>
     <row r="17">
@@ -1314,18 +1314,18 @@
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L17" t="n">
         <v>4</v>
@@ -1334,7 +1334,7 @@
         <v>70</v>
       </c>
       <c r="N17" t="n">
-        <v>70</v>
+        <v>500</v>
       </c>
     </row>
     <row r="18">
@@ -1366,18 +1366,18 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J18" t="n">
         <v>2</v>
       </c>
       <c r="K18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L18" t="n">
         <v>4</v>
@@ -1386,7 +1386,7 @@
         <v>70</v>
       </c>
       <c r="N18" t="n">
-        <v>170</v>
+        <v>470</v>
       </c>
     </row>
     <row r="19">
@@ -1418,18 +1418,18 @@
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K19" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L19" t="n">
         <v>4</v>
@@ -1438,7 +1438,7 @@
         <v>70</v>
       </c>
       <c r="N19" t="n">
-        <v>170</v>
+        <v>530</v>
       </c>
     </row>
     <row r="20">
@@ -1470,18 +1470,18 @@
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
         <v>4</v>
@@ -1490,7 +1490,7 @@
         <v>70</v>
       </c>
       <c r="N20" t="n">
-        <v>170</v>
+        <v>330</v>
       </c>
     </row>
     <row r="21">
@@ -1522,18 +1522,18 @@
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J21" t="n">
         <v>2</v>
       </c>
       <c r="K21" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="L21" t="n">
         <v>4</v>
@@ -1542,7 +1542,7 @@
         <v>70</v>
       </c>
       <c r="N21" t="n">
-        <v>170</v>
+        <v>340</v>
       </c>
     </row>
     <row r="22">
@@ -1574,18 +1574,18 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Bergur</t>
+          <t>Camilla</t>
         </is>
       </c>
       <c r="J22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K22" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="L22" t="n">
         <v>4</v>
@@ -1594,7 +1594,7 @@
         <v>70</v>
       </c>
       <c r="N22" t="n">
-        <v>170</v>
+        <v>500</v>
       </c>
     </row>
     <row r="23">
@@ -1626,18 +1626,18 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Gunnar</t>
+          <t>Anna</t>
         </is>
       </c>
       <c r="J23" t="n">
         <v>1</v>
       </c>
       <c r="K23" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="L23" t="n">
         <v>4</v>
@@ -1646,7 +1646,7 @@
         <v>70</v>
       </c>
       <c r="N23" t="n">
-        <v>170</v>
+        <v>530</v>
       </c>
     </row>
     <row r="24">
@@ -1678,11 +1678,11 @@
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Ólafur</t>
+          <t>Nanna</t>
         </is>
       </c>
       <c r="J24" t="n">
@@ -1698,7 +1698,7 @@
         <v>100</v>
       </c>
       <c r="N24" t="n">
-        <v>100</v>
+        <v>420</v>
       </c>
     </row>
     <row r="25">
@@ -1750,7 +1750,7 @@
         <v>80</v>
       </c>
       <c r="N25" t="n">
-        <v>130</v>
+        <v>350</v>
       </c>
     </row>
     <row r="26">
@@ -1782,11 +1782,11 @@
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J26" t="n">
@@ -1802,7 +1802,7 @@
         <v>80</v>
       </c>
       <c r="N26" t="n">
-        <v>80</v>
+        <v>340</v>
       </c>
     </row>
     <row r="27">
@@ -1834,15 +1834,15 @@
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Ólafur</t>
         </is>
       </c>
       <c r="J27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -1854,7 +1854,7 @@
         <v>80</v>
       </c>
       <c r="N27" t="n">
-        <v>150</v>
+        <v>440</v>
       </c>
     </row>
     <row r="28">
@@ -1886,11 +1886,11 @@
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J28" t="n">
@@ -1906,7 +1906,7 @@
         <v>90</v>
       </c>
       <c r="N28" t="n">
-        <v>260</v>
+        <v>480</v>
       </c>
     </row>
     <row r="29">
@@ -1938,18 +1938,18 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Össur</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K29" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L29" t="n">
         <v>3.5</v>
@@ -1958,7 +1958,7 @@
         <v>50</v>
       </c>
       <c r="N29" t="n">
-        <v>280</v>
+        <v>420</v>
       </c>
     </row>
     <row r="30">
@@ -1990,18 +1990,18 @@
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J30" t="n">
         <v>2</v>
       </c>
       <c r="K30" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L30" t="n">
         <v>3.5</v>
@@ -2010,7 +2010,7 @@
         <v>50</v>
       </c>
       <c r="N30" t="n">
-        <v>190</v>
+        <v>490</v>
       </c>
     </row>
     <row r="31">
@@ -2042,18 +2042,18 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J31" t="n">
         <v>2</v>
       </c>
       <c r="K31" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L31" t="n">
         <v>3.5</v>
@@ -2062,7 +2062,7 @@
         <v>50</v>
       </c>
       <c r="N31" t="n">
-        <v>130</v>
+        <v>510</v>
       </c>
     </row>
     <row r="32">
@@ -2094,18 +2094,18 @@
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J32" t="n">
         <v>2</v>
       </c>
       <c r="K32" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L32" t="n">
         <v>3.5</v>
@@ -2114,7 +2114,7 @@
         <v>50</v>
       </c>
       <c r="N32" t="n">
-        <v>270</v>
+        <v>410</v>
       </c>
     </row>
     <row r="33">
@@ -2146,18 +2146,18 @@
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J33" t="n">
         <v>2</v>
       </c>
       <c r="K33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L33" t="n">
         <v>3.5</v>
@@ -2166,7 +2166,7 @@
         <v>50</v>
       </c>
       <c r="N33" t="n">
-        <v>250</v>
+        <v>430</v>
       </c>
     </row>
     <row r="34">
@@ -2198,18 +2198,18 @@
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K34" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L34" t="n">
         <v>3.5</v>
@@ -2218,7 +2218,7 @@
         <v>50</v>
       </c>
       <c r="N34" t="n">
-        <v>290</v>
+        <v>380</v>
       </c>
     </row>
     <row r="35">
@@ -2250,18 +2250,18 @@
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J35" t="n">
         <v>2</v>
       </c>
       <c r="K35" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L35" t="n">
         <v>3.5</v>
@@ -2270,7 +2270,7 @@
         <v>50</v>
       </c>
       <c r="N35" t="n">
-        <v>200</v>
+        <v>520</v>
       </c>
     </row>
     <row r="36">
@@ -2302,15 +2302,15 @@
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K36" t="n">
         <v>7</v>
@@ -2322,7 +2322,7 @@
         <v>50</v>
       </c>
       <c r="N36" t="n">
-        <v>270</v>
+        <v>540</v>
       </c>
     </row>
     <row r="37">
@@ -2354,18 +2354,18 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K37" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L37" t="n">
         <v>3.5</v>
@@ -2374,7 +2374,7 @@
         <v>50</v>
       </c>
       <c r="N37" t="n">
-        <v>190</v>
+        <v>540</v>
       </c>
     </row>
     <row r="38">
@@ -2406,18 +2406,18 @@
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Nanna</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K38" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L38" t="n">
         <v>3.5</v>
@@ -2426,7 +2426,7 @@
         <v>50</v>
       </c>
       <c r="N38" t="n">
-        <v>290</v>
+        <v>540</v>
       </c>
     </row>
     <row r="39">
@@ -2458,18 +2458,18 @@
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Anna</t>
+          <t>Gunnar</t>
         </is>
       </c>
       <c r="J39" t="n">
         <v>1</v>
       </c>
       <c r="K39" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L39" t="n">
         <v>3.5</v>
@@ -2478,7 +2478,7 @@
         <v>50</v>
       </c>
       <c r="N39" t="n">
-        <v>270</v>
+        <v>550</v>
       </c>
     </row>
     <row r="40">
@@ -2510,18 +2510,18 @@
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Ásdís</t>
+          <t>Össur</t>
         </is>
       </c>
       <c r="J40" t="n">
         <v>3</v>
       </c>
       <c r="K40" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L40" t="n">
         <v>4</v>
@@ -2530,7 +2530,7 @@
         <v>50</v>
       </c>
       <c r="N40" t="n">
-        <v>50</v>
+        <v>540</v>
       </c>
     </row>
     <row r="41">
@@ -2562,18 +2562,18 @@
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Helgi</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J41" t="n">
+        <v>2</v>
+      </c>
+      <c r="K41" t="n">
         <v>3</v>
-      </c>
-      <c r="K41" t="n">
-        <v>8</v>
       </c>
       <c r="L41" t="n">
         <v>4</v>
@@ -2582,7 +2582,7 @@
         <v>50</v>
       </c>
       <c r="N41" t="n">
-        <v>50</v>
+        <v>330</v>
       </c>
     </row>
     <row r="42">
@@ -2614,18 +2614,18 @@
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Össur</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K42" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L42" t="n">
         <v>4</v>
@@ -2634,7 +2634,7 @@
         <v>50</v>
       </c>
       <c r="N42" t="n">
-        <v>50</v>
+        <v>310</v>
       </c>
     </row>
     <row r="43">
@@ -2666,18 +2666,18 @@
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Thelma</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K43" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L43" t="n">
         <v>4</v>
@@ -2686,7 +2686,7 @@
         <v>50</v>
       </c>
       <c r="N43" t="n">
-        <v>50</v>
+        <v>530</v>
       </c>
     </row>
     <row r="44">
@@ -2718,18 +2718,18 @@
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Pétur</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J44" t="n">
         <v>2</v>
       </c>
       <c r="K44" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L44" t="n">
         <v>4</v>
@@ -2738,7 +2738,7 @@
         <v>50</v>
       </c>
       <c r="N44" t="n">
-        <v>50</v>
+        <v>330</v>
       </c>
     </row>
     <row r="45">
@@ -2770,18 +2770,18 @@
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J45" t="n">
         <v>2</v>
       </c>
       <c r="K45" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L45" t="n">
         <v>4</v>
@@ -2790,7 +2790,7 @@
         <v>50</v>
       </c>
       <c r="N45" t="n">
-        <v>50</v>
+        <v>330</v>
       </c>
     </row>
     <row r="46">
@@ -2822,18 +2822,18 @@
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K46" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L46" t="n">
         <v>4</v>
@@ -2842,7 +2842,7 @@
         <v>50</v>
       </c>
       <c r="N46" t="n">
-        <v>50</v>
+        <v>490</v>
       </c>
     </row>
     <row r="47">
@@ -2874,18 +2874,18 @@
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J47" t="n">
         <v>2</v>
       </c>
       <c r="K47" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L47" t="n">
         <v>4</v>
@@ -2894,7 +2894,7 @@
         <v>50</v>
       </c>
       <c r="N47" t="n">
-        <v>50</v>
+        <v>330</v>
       </c>
     </row>
     <row r="48">
@@ -2926,18 +2926,18 @@
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K48" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L48" t="n">
         <v>4</v>
@@ -2946,7 +2946,7 @@
         <v>50</v>
       </c>
       <c r="N48" t="n">
-        <v>50</v>
+        <v>320</v>
       </c>
     </row>
     <row r="49">
@@ -2978,18 +2978,18 @@
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Ólafur</t>
         </is>
       </c>
       <c r="J49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K49" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L49" t="n">
         <v>4</v>
@@ -2998,7 +2998,7 @@
         <v>50</v>
       </c>
       <c r="N49" t="n">
-        <v>50</v>
+        <v>490</v>
       </c>
     </row>
     <row r="50">
@@ -3030,18 +3030,18 @@
       </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Bergur</t>
         </is>
       </c>
       <c r="J50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K50" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L50" t="n">
         <v>4</v>
@@ -3050,7 +3050,7 @@
         <v>50</v>
       </c>
       <c r="N50" t="n">
-        <v>50</v>
+        <v>320</v>
       </c>
     </row>
     <row r="51">
@@ -3082,11 +3082,11 @@
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Anna</t>
+          <t>Camilla</t>
         </is>
       </c>
       <c r="J51" t="n">
@@ -3102,7 +3102,7 @@
         <v>100</v>
       </c>
       <c r="N51" t="n">
-        <v>100</v>
+        <v>430</v>
       </c>
     </row>
     <row r="52">
@@ -3154,7 +3154,7 @@
         <v>50</v>
       </c>
       <c r="N52" t="n">
-        <v>100</v>
+        <v>390</v>
       </c>
     </row>
     <row r="53">
@@ -3197,7 +3197,7 @@
         <v>2</v>
       </c>
       <c r="K53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L53" t="n">
         <v>4</v>
@@ -3206,7 +3206,7 @@
         <v>50</v>
       </c>
       <c r="N53" t="n">
-        <v>90</v>
+        <v>370</v>
       </c>
     </row>
     <row r="54">
@@ -3238,18 +3238,18 @@
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J54" t="n">
         <v>2</v>
       </c>
       <c r="K54" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L54" t="n">
         <v>4</v>
@@ -3258,7 +3258,7 @@
         <v>50</v>
       </c>
       <c r="N54" t="n">
-        <v>120</v>
+        <v>560</v>
       </c>
     </row>
     <row r="55">
@@ -3290,18 +3290,18 @@
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K55" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="L55" t="n">
         <v>4</v>
@@ -3310,7 +3310,7 @@
         <v>50</v>
       </c>
       <c r="N55" t="n">
-        <v>220</v>
+        <v>390</v>
       </c>
     </row>
     <row r="56">
@@ -3342,18 +3342,18 @@
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J56" t="n">
         <v>2</v>
       </c>
       <c r="K56" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L56" t="n">
         <v>4</v>
@@ -3362,7 +3362,7 @@
         <v>50</v>
       </c>
       <c r="N56" t="n">
-        <v>120</v>
+        <v>350</v>
       </c>
     </row>
     <row r="57">
@@ -3394,15 +3394,15 @@
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="J57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K57" t="n">
         <v>8</v>
@@ -3414,7 +3414,7 @@
         <v>50</v>
       </c>
       <c r="N57" t="n">
-        <v>200</v>
+        <v>580</v>
       </c>
     </row>
     <row r="58">
@@ -3446,18 +3446,18 @@
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J58" t="n">
         <v>2</v>
       </c>
       <c r="K58" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L58" t="n">
         <v>4</v>
@@ -3466,7 +3466,7 @@
         <v>50</v>
       </c>
       <c r="N58" t="n">
-        <v>120</v>
+        <v>390</v>
       </c>
     </row>
     <row r="59">
@@ -3498,18 +3498,18 @@
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J59" t="n">
         <v>2</v>
       </c>
       <c r="K59" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L59" t="n">
         <v>4</v>
@@ -3518,7 +3518,7 @@
         <v>50</v>
       </c>
       <c r="N59" t="n">
-        <v>50</v>
+        <v>390</v>
       </c>
     </row>
     <row r="60">
@@ -3550,18 +3550,18 @@
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Camilla</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K60" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L60" t="n">
         <v>4</v>
@@ -3570,7 +3570,7 @@
         <v>50</v>
       </c>
       <c r="N60" t="n">
-        <v>50</v>
+        <v>390</v>
       </c>
     </row>
     <row r="61">
@@ -3602,18 +3602,18 @@
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Bergur</t>
+          <t>Nanna</t>
         </is>
       </c>
       <c r="J61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K61" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L61" t="n">
         <v>4</v>
@@ -3622,7 +3622,7 @@
         <v>50</v>
       </c>
       <c r="N61" t="n">
-        <v>50</v>
+        <v>320</v>
       </c>
     </row>
     <row r="62">
@@ -3654,18 +3654,18 @@
       </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Gunnar</t>
+          <t>Anna</t>
         </is>
       </c>
       <c r="J62" t="n">
         <v>1</v>
       </c>
       <c r="K62" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L62" t="n">
         <v>4</v>
@@ -3674,7 +3674,7 @@
         <v>50</v>
       </c>
       <c r="N62" t="n">
-        <v>220</v>
+        <v>580</v>
       </c>
     </row>
     <row r="63">
@@ -3706,11 +3706,11 @@
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J63" t="n">
@@ -3726,7 +3726,7 @@
         <v>80</v>
       </c>
       <c r="N63" t="n">
-        <v>150</v>
+        <v>470</v>
       </c>
     </row>
     <row r="64">
@@ -3758,18 +3758,18 @@
       </c>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Thelma</t>
+          <t>Ásdís</t>
         </is>
       </c>
       <c r="J64" t="n">
         <v>3</v>
       </c>
       <c r="K64" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L64" t="n">
         <v>4</v>
@@ -3778,7 +3778,7 @@
         <v>70</v>
       </c>
       <c r="N64" t="n">
-        <v>120</v>
+        <v>420</v>
       </c>
     </row>
     <row r="65">
@@ -3810,18 +3810,18 @@
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Harpa</t>
+          <t>Thelma</t>
         </is>
       </c>
       <c r="J65" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K65" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L65" t="n">
         <v>4</v>
@@ -3830,7 +3830,7 @@
         <v>70</v>
       </c>
       <c r="N65" t="n">
-        <v>70</v>
+        <v>330</v>
       </c>
     </row>
     <row r="66">
@@ -3862,18 +3862,18 @@
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J66" t="n">
         <v>2</v>
       </c>
       <c r="K66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L66" t="n">
         <v>4</v>
@@ -3882,7 +3882,7 @@
         <v>70</v>
       </c>
       <c r="N66" t="n">
-        <v>70</v>
+        <v>330</v>
       </c>
     </row>
     <row r="67">
@@ -3914,18 +3914,18 @@
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K67" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L67" t="n">
         <v>4</v>
@@ -3934,7 +3934,7 @@
         <v>70</v>
       </c>
       <c r="N67" t="n">
-        <v>70</v>
+        <v>340</v>
       </c>
     </row>
     <row r="68">
@@ -3966,18 +3966,18 @@
       </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Gunnar</t>
         </is>
       </c>
       <c r="J68" t="n">
         <v>1</v>
       </c>
       <c r="K68" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L68" t="n">
         <v>4</v>
@@ -3986,7 +3986,7 @@
         <v>70</v>
       </c>
       <c r="N68" t="n">
-        <v>140</v>
+        <v>330</v>
       </c>
     </row>
     <row r="69">
@@ -4018,18 +4018,18 @@
       </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Helgi</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J69" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K69" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L69" t="n">
         <v>4.5</v>
@@ -4038,7 +4038,7 @@
         <v>100</v>
       </c>
       <c r="N69" t="n">
-        <v>270</v>
+        <v>480</v>
       </c>
     </row>
     <row r="70">
@@ -4070,18 +4070,18 @@
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J70" t="n">
         <v>2</v>
       </c>
       <c r="K70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L70" t="n">
         <v>4.5</v>
@@ -4090,7 +4090,7 @@
         <v>100</v>
       </c>
       <c r="N70" t="n">
-        <v>270</v>
+        <v>490</v>
       </c>
     </row>
     <row r="71">
@@ -4122,11 +4122,11 @@
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Pétur</t>
+          <t>Jóna</t>
         </is>
       </c>
       <c r="J71" t="n">
@@ -4142,7 +4142,7 @@
         <v>100</v>
       </c>
       <c r="N71" t="n">
-        <v>260</v>
+        <v>490</v>
       </c>
     </row>
     <row r="72">
@@ -4185,7 +4185,7 @@
         <v>3</v>
       </c>
       <c r="K72" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L72" t="n">
         <v>3.5</v>
@@ -4194,7 +4194,7 @@
         <v>50</v>
       </c>
       <c r="N72" t="n">
-        <v>250</v>
+        <v>470</v>
       </c>
     </row>
     <row r="73">
@@ -4226,18 +4226,18 @@
       </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Thelma</t>
         </is>
       </c>
       <c r="J73" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K73" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="L73" t="n">
         <v>3.5</v>
@@ -4246,7 +4246,7 @@
         <v>50</v>
       </c>
       <c r="N73" t="n">
-        <v>170</v>
+        <v>530</v>
       </c>
     </row>
     <row r="74">
@@ -4278,18 +4278,18 @@
       </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K74" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L74" t="n">
         <v>3.5</v>
@@ -4298,7 +4298,7 @@
         <v>50</v>
       </c>
       <c r="N74" t="n">
-        <v>270</v>
+        <v>520</v>
       </c>
     </row>
     <row r="75">
@@ -4341,7 +4341,7 @@
         <v>2</v>
       </c>
       <c r="K75" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L75" t="n">
         <v>3.5</v>
@@ -4350,7 +4350,7 @@
         <v>50</v>
       </c>
       <c r="N75" t="n">
-        <v>170</v>
+        <v>530</v>
       </c>
     </row>
     <row r="76">
@@ -4393,7 +4393,7 @@
         <v>2</v>
       </c>
       <c r="K76" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L76" t="n">
         <v>3.5</v>
@@ -4402,7 +4402,7 @@
         <v>50</v>
       </c>
       <c r="N76" t="n">
-        <v>250</v>
+        <v>380</v>
       </c>
     </row>
     <row r="77">
@@ -4445,7 +4445,7 @@
         <v>2</v>
       </c>
       <c r="K77" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L77" t="n">
         <v>3.5</v>
@@ -4454,7 +4454,7 @@
         <v>50</v>
       </c>
       <c r="N77" t="n">
-        <v>250</v>
+        <v>380</v>
       </c>
     </row>
     <row r="78">
@@ -4486,18 +4486,18 @@
       </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J78" t="n">
         <v>2</v>
       </c>
       <c r="K78" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L78" t="n">
         <v>3.5</v>
@@ -4506,7 +4506,7 @@
         <v>50</v>
       </c>
       <c r="N78" t="n">
-        <v>170</v>
+        <v>440</v>
       </c>
     </row>
     <row r="79">
@@ -4538,18 +4538,18 @@
       </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Máni</t>
         </is>
       </c>
       <c r="J79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K79" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L79" t="n">
         <v>3.5</v>
@@ -4558,7 +4558,7 @@
         <v>50</v>
       </c>
       <c r="N79" t="n">
-        <v>290</v>
+        <v>530</v>
       </c>
     </row>
     <row r="80">
@@ -4590,18 +4590,18 @@
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J80" t="n">
         <v>1</v>
       </c>
       <c r="K80" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L80" t="n">
         <v>3.5</v>
@@ -4610,7 +4610,7 @@
         <v>50</v>
       </c>
       <c r="N80" t="n">
-        <v>250</v>
+        <v>540</v>
       </c>
     </row>
     <row r="81">
@@ -4642,18 +4642,18 @@
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Camilla</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K81" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L81" t="n">
         <v>3.5</v>
@@ -4662,7 +4662,7 @@
         <v>50</v>
       </c>
       <c r="N81" t="n">
-        <v>250</v>
+        <v>380</v>
       </c>
     </row>
     <row r="82">
@@ -4694,11 +4694,11 @@
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Ólafur</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J82" t="n">
@@ -4714,7 +4714,7 @@
         <v>50</v>
       </c>
       <c r="N82" t="n">
-        <v>150</v>
+        <v>370</v>
       </c>
     </row>
     <row r="83">
@@ -4766,7 +4766,7 @@
         <v>100</v>
       </c>
       <c r="N83" t="n">
-        <v>100</v>
+        <v>430</v>
       </c>
     </row>
     <row r="84">
@@ -4798,18 +4798,18 @@
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J84" t="n">
         <v>2</v>
       </c>
       <c r="K84" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L84" t="n">
         <v>4</v>
@@ -4818,7 +4818,7 @@
         <v>50</v>
       </c>
       <c r="N84" t="n">
-        <v>180</v>
+        <v>420</v>
       </c>
     </row>
     <row r="85">
@@ -4850,18 +4850,18 @@
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Björk</t>
+          <t>Freyja</t>
         </is>
       </c>
       <c r="J85" t="n">
         <v>2</v>
       </c>
       <c r="K85" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L85" t="n">
         <v>4</v>
@@ -4870,7 +4870,7 @@
         <v>50</v>
       </c>
       <c r="N85" t="n">
-        <v>220</v>
+        <v>390</v>
       </c>
     </row>
     <row r="86">
@@ -4902,18 +4902,18 @@
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Björk</t>
         </is>
       </c>
       <c r="J86" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K86" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="L86" t="n">
         <v>4</v>
@@ -4922,7 +4922,7 @@
         <v>50</v>
       </c>
       <c r="N86" t="n">
-        <v>220</v>
+        <v>540</v>
       </c>
     </row>
     <row r="87">
@@ -4954,18 +4954,18 @@
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K87" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="L87" t="n">
         <v>4</v>
@@ -4974,7 +4974,7 @@
         <v>50</v>
       </c>
       <c r="N87" t="n">
-        <v>100</v>
+        <v>580</v>
       </c>
     </row>
     <row r="88">
@@ -5006,18 +5006,18 @@
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Inga</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J88" t="n">
         <v>2</v>
       </c>
       <c r="K88" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="L88" t="n">
         <v>4</v>
@@ -5026,7 +5026,7 @@
         <v>50</v>
       </c>
       <c r="N88" t="n">
-        <v>100</v>
+        <v>580</v>
       </c>
     </row>
     <row r="89">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J89" t="n">
@@ -5078,7 +5078,7 @@
         <v>50</v>
       </c>
       <c r="N89" t="n">
-        <v>100</v>
+        <v>400</v>
       </c>
     </row>
     <row r="90">
@@ -5110,11 +5110,11 @@
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Ylfa</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J90" t="n">
@@ -5130,7 +5130,7 @@
         <v>50</v>
       </c>
       <c r="N90" t="n">
-        <v>100</v>
+        <v>390</v>
       </c>
     </row>
     <row r="91">
@@ -5162,18 +5162,18 @@
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>Jóna</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J91" t="n">
         <v>2</v>
       </c>
       <c r="K91" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L91" t="n">
         <v>4</v>
@@ -5182,7 +5182,7 @@
         <v>50</v>
       </c>
       <c r="N91" t="n">
-        <v>100</v>
+        <v>390</v>
       </c>
     </row>
     <row r="92">
@@ -5214,11 +5214,11 @@
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>Nanna</t>
+          <t>Camilla</t>
         </is>
       </c>
       <c r="J92" t="n">
@@ -5234,7 +5234,7 @@
         <v>50</v>
       </c>
       <c r="N92" t="n">
-        <v>50</v>
+        <v>330</v>
       </c>
     </row>
     <row r="93">
@@ -5266,18 +5266,18 @@
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>Anna</t>
+          <t>Ólafur</t>
         </is>
       </c>
       <c r="J93" t="n">
         <v>1</v>
       </c>
       <c r="K93" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L93" t="n">
         <v>4</v>
@@ -5286,7 +5286,7 @@
         <v>50</v>
       </c>
       <c r="N93" t="n">
-        <v>220</v>
+        <v>540</v>
       </c>
     </row>
     <row r="94">
@@ -5329,7 +5329,7 @@
         <v>2</v>
       </c>
       <c r="K94" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L94" t="n">
         <v>4</v>
@@ -5338,7 +5338,7 @@
         <v>50</v>
       </c>
       <c r="N94" t="n">
-        <v>100</v>
+        <v>410</v>
       </c>
     </row>
     <row r="95">
@@ -5390,7 +5390,7 @@
         <v>80</v>
       </c>
       <c r="N95" t="n">
-        <v>130</v>
+        <v>460</v>
       </c>
     </row>
     <row r="96">
@@ -5442,7 +5442,7 @@
         <v>40</v>
       </c>
       <c r="N96" t="n">
-        <v>90</v>
+        <v>350</v>
       </c>
     </row>
     <row r="97">
@@ -5494,7 +5494,7 @@
         <v>40</v>
       </c>
       <c r="N97" t="n">
-        <v>40</v>
+        <v>320</v>
       </c>
     </row>
     <row r="98">
@@ -5526,18 +5526,18 @@
       </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>Thelma</t>
+          <t>Ásdís</t>
         </is>
       </c>
       <c r="J98" t="n">
         <v>3</v>
       </c>
       <c r="K98" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L98" t="n">
         <v>3</v>
@@ -5546,7 +5546,7 @@
         <v>70</v>
       </c>
       <c r="N98" t="n">
-        <v>300</v>
+        <v>540</v>
       </c>
     </row>
     <row r="99">
@@ -5578,18 +5578,18 @@
       </c>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>Pétur</t>
+          <t>Helgi</t>
         </is>
       </c>
       <c r="J99" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K99" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="L99" t="n">
         <v>3</v>
@@ -5598,7 +5598,7 @@
         <v>70</v>
       </c>
       <c r="N99" t="n">
-        <v>160</v>
+        <v>540</v>
       </c>
     </row>
     <row r="100">
@@ -5630,18 +5630,18 @@
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>Unnur</t>
+          <t>Össur</t>
         </is>
       </c>
       <c r="J100" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K100" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L100" t="n">
         <v>3</v>
@@ -5650,7 +5650,7 @@
         <v>70</v>
       </c>
       <c r="N100" t="n">
-        <v>160</v>
+        <v>490</v>
       </c>
     </row>
     <row r="101">
@@ -5682,18 +5682,18 @@
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J101" t="n">
         <v>2</v>
       </c>
       <c r="K101" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L101" t="n">
         <v>3</v>
@@ -5702,7 +5702,7 @@
         <v>70</v>
       </c>
       <c r="N101" t="n">
-        <v>320</v>
+        <v>490</v>
       </c>
     </row>
     <row r="102">
@@ -5734,11 +5734,11 @@
       </c>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J102" t="n">
@@ -5754,7 +5754,7 @@
         <v>70</v>
       </c>
       <c r="N102" t="n">
-        <v>310</v>
+        <v>490</v>
       </c>
     </row>
     <row r="103">
@@ -5786,18 +5786,18 @@
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J103" t="n">
         <v>2</v>
       </c>
       <c r="K103" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="L103" t="n">
         <v>3</v>
@@ -5806,7 +5806,7 @@
         <v>70</v>
       </c>
       <c r="N103" t="n">
-        <v>320</v>
+        <v>380</v>
       </c>
     </row>
     <row r="104">
@@ -5838,18 +5838,18 @@
       </c>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="n">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Erla</t>
         </is>
       </c>
       <c r="J104" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K104" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L104" t="n">
         <v>3</v>
@@ -5858,7 +5858,7 @@
         <v>70</v>
       </c>
       <c r="N104" t="n">
-        <v>320</v>
+        <v>360</v>
       </c>
     </row>
     <row r="105">
@@ -5890,18 +5890,18 @@
       </c>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Ólafur</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K105" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L105" t="n">
         <v>3</v>
@@ -5910,7 +5910,7 @@
         <v>70</v>
       </c>
       <c r="N105" t="n">
-        <v>290</v>
+        <v>540</v>
       </c>
     </row>
     <row r="106">
@@ -5942,11 +5942,11 @@
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>Anna</t>
+          <t>Ólafur</t>
         </is>
       </c>
       <c r="J106" t="n">
@@ -5962,7 +5962,7 @@
         <v>70</v>
       </c>
       <c r="N106" t="n">
-        <v>170</v>
+        <v>360</v>
       </c>
     </row>
     <row r="107">
@@ -6005,7 +6005,7 @@
         <v>2</v>
       </c>
       <c r="K107" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L107" t="n">
         <v>3</v>
@@ -6014,7 +6014,7 @@
         <v>70</v>
       </c>
       <c r="N107" t="n">
-        <v>310</v>
+        <v>480</v>
       </c>
     </row>
     <row r="108">
@@ -6057,7 +6057,7 @@
         <v>1</v>
       </c>
       <c r="K108" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L108" t="n">
         <v>3</v>
@@ -6066,7 +6066,7 @@
         <v>70</v>
       </c>
       <c r="N108" t="n">
-        <v>290</v>
+        <v>500</v>
       </c>
     </row>
     <row r="109">
@@ -6098,11 +6098,11 @@
       </c>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>Máni</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J109" t="n">
@@ -6118,7 +6118,7 @@
         <v>90</v>
       </c>
       <c r="N109" t="n">
-        <v>260</v>
+        <v>470</v>
       </c>
     </row>
     <row r="110">
@@ -6161,7 +6161,7 @@
         <v>1</v>
       </c>
       <c r="K110" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L110" t="n">
         <v>4</v>
@@ -6170,7 +6170,7 @@
         <v>100</v>
       </c>
       <c r="N110" t="n">
-        <v>170</v>
+        <v>460</v>
       </c>
     </row>
     <row r="111">
@@ -6202,11 +6202,11 @@
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J111" t="n">
@@ -6222,7 +6222,7 @@
         <v>100</v>
       </c>
       <c r="N111" t="n">
-        <v>170</v>
+        <v>470</v>
       </c>
     </row>
     <row r="112">
@@ -6254,18 +6254,18 @@
       </c>
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Nanna</t>
+          <t>Anna</t>
         </is>
       </c>
       <c r="J112" t="n">
         <v>1</v>
       </c>
       <c r="K112" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L112" t="n">
         <v>4</v>
@@ -6274,7 +6274,7 @@
         <v>100</v>
       </c>
       <c r="N112" t="n">
-        <v>150</v>
+        <v>460</v>
       </c>
     </row>
     <row r="113">
@@ -6306,18 +6306,18 @@
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>Ásdís</t>
+          <t>Thelma</t>
         </is>
       </c>
       <c r="J113" t="n">
         <v>3</v>
       </c>
       <c r="K113" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L113" t="n">
         <v>4</v>
@@ -6326,7 +6326,7 @@
         <v>70</v>
       </c>
       <c r="N113" t="n">
-        <v>200</v>
+        <v>480</v>
       </c>
     </row>
     <row r="114">
@@ -6358,18 +6358,18 @@
       </c>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>Thelma</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J114" t="n">
+        <v>2</v>
+      </c>
+      <c r="K114" t="n">
         <v>3</v>
-      </c>
-      <c r="K114" t="n">
-        <v>5</v>
       </c>
       <c r="L114" t="n">
         <v>4</v>
@@ -6378,7 +6378,7 @@
         <v>70</v>
       </c>
       <c r="N114" t="n">
-        <v>190</v>
+        <v>400</v>
       </c>
     </row>
     <row r="115">
@@ -6410,18 +6410,18 @@
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="n">
+        <v>9</v>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Freyja</t>
+        </is>
+      </c>
+      <c r="J115" t="n">
+        <v>2</v>
+      </c>
+      <c r="K115" t="n">
         <v>7</v>
-      </c>
-      <c r="I115" t="inlineStr">
-        <is>
-          <t>Harpa</t>
-        </is>
-      </c>
-      <c r="J115" t="n">
-        <v>2</v>
-      </c>
-      <c r="K115" t="n">
-        <v>3</v>
       </c>
       <c r="L115" t="n">
         <v>4</v>
@@ -6430,7 +6430,7 @@
         <v>70</v>
       </c>
       <c r="N115" t="n">
-        <v>140</v>
+        <v>540</v>
       </c>
     </row>
     <row r="116">
@@ -6462,18 +6462,18 @@
       </c>
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Davíð</t>
         </is>
       </c>
       <c r="J116" t="n">
         <v>2</v>
       </c>
       <c r="K116" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L116" t="n">
         <v>4</v>
@@ -6482,7 +6482,7 @@
         <v>70</v>
       </c>
       <c r="N116" t="n">
-        <v>200</v>
+        <v>540</v>
       </c>
     </row>
     <row r="117">
@@ -6514,18 +6514,18 @@
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>Rakel</t>
+          <t>Laufey</t>
         </is>
       </c>
       <c r="J117" t="n">
         <v>2</v>
       </c>
       <c r="K117" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="L117" t="n">
         <v>4</v>
@@ -6534,7 +6534,7 @@
         <v>70</v>
       </c>
       <c r="N117" t="n">
-        <v>70</v>
+        <v>540</v>
       </c>
     </row>
     <row r="118">
@@ -6566,18 +6566,18 @@
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Davíð</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="J118" t="n">
         <v>2</v>
       </c>
       <c r="K118" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L118" t="n">
         <v>4</v>
@@ -6586,7 +6586,7 @@
         <v>70</v>
       </c>
       <c r="N118" t="n">
-        <v>70</v>
+        <v>340</v>
       </c>
     </row>
     <row r="119">
@@ -6618,18 +6618,18 @@
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Úlfur</t>
         </is>
       </c>
       <c r="J119" t="n">
         <v>1</v>
       </c>
       <c r="K119" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L119" t="n">
         <v>4</v>
@@ -6638,7 +6638,7 @@
         <v>70</v>
       </c>
       <c r="N119" t="n">
-        <v>70</v>
+        <v>550</v>
       </c>
     </row>
     <row r="120">
@@ -6670,18 +6670,18 @@
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Kata</t>
+          <t>Inga</t>
         </is>
       </c>
       <c r="J120" t="n">
         <v>2</v>
       </c>
       <c r="K120" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L120" t="n">
         <v>4</v>
@@ -6690,7 +6690,7 @@
         <v>70</v>
       </c>
       <c r="N120" t="n">
-        <v>170</v>
+        <v>340</v>
       </c>
     </row>
     <row r="121">
@@ -6722,18 +6722,18 @@
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Silja</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="J121" t="n">
         <v>1</v>
       </c>
       <c r="K121" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L121" t="n">
         <v>4</v>
@@ -6742,7 +6742,7 @@
         <v>70</v>
       </c>
       <c r="N121" t="n">
-        <v>200</v>
+        <v>340</v>
       </c>
     </row>
     <row r="122">
@@ -6785,7 +6785,7 @@
         <v>1</v>
       </c>
       <c r="K122" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L122" t="n">
         <v>4</v>
@@ -6794,7 +6794,7 @@
         <v>70</v>
       </c>
       <c r="N122" t="n">
-        <v>200</v>
+        <v>570</v>
       </c>
     </row>
     <row r="123">
@@ -6826,18 +6826,18 @@
       </c>
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>Ólafur</t>
+          <t>Nanna</t>
         </is>
       </c>
       <c r="J123" t="n">
         <v>1</v>
       </c>
       <c r="K123" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L123" t="n">
         <v>4</v>
@@ -6846,7 +6846,7 @@
         <v>70</v>
       </c>
       <c r="N123" t="n">
-        <v>220</v>
+        <v>490</v>
       </c>
     </row>
     <row r="124">
@@ -6878,18 +6878,18 @@
       </c>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Össur</t>
+          <t>Pétur</t>
         </is>
       </c>
       <c r="J124" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K124" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L124" t="n">
         <v>2</v>
@@ -6898,7 +6898,7 @@
         <v>70</v>
       </c>
       <c r="N124" t="n">
-        <v>230</v>
+        <v>560</v>
       </c>
     </row>
     <row r="125">
@@ -6930,18 +6930,18 @@
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Vala</t>
+          <t>Unnur</t>
         </is>
       </c>
       <c r="J125" t="n">
         <v>2</v>
       </c>
       <c r="K125" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L125" t="n">
         <v>2</v>
@@ -6950,7 +6950,7 @@
         <v>70</v>
       </c>
       <c r="N125" t="n">
-        <v>250</v>
+        <v>560</v>
       </c>
     </row>
     <row r="126">
@@ -6982,18 +6982,18 @@
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Freyja</t>
+          <t>Harpa</t>
         </is>
       </c>
       <c r="J126" t="n">
         <v>2</v>
       </c>
       <c r="K126" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L126" t="n">
         <v>2</v>
@@ -7002,7 +7002,7 @@
         <v>70</v>
       </c>
       <c r="N126" t="n">
-        <v>240</v>
+        <v>510</v>
       </c>
     </row>
     <row r="127">
@@ -7034,18 +7034,18 @@
       </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Lísa</t>
+          <t>Vala</t>
         </is>
       </c>
       <c r="J127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K127" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L127" t="n">
         <v>2</v>
@@ -7054,7 +7054,7 @@
         <v>70</v>
       </c>
       <c r="N127" t="n">
-        <v>70</v>
+        <v>590</v>
       </c>
     </row>
     <row r="128">
@@ -7086,18 +7086,18 @@
       </c>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Erla</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="J128" t="n">
         <v>2</v>
       </c>
       <c r="K128" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="L128" t="n">
         <v>2</v>
@@ -7106,7 +7106,7 @@
         <v>70</v>
       </c>
       <c r="N128" t="n">
-        <v>240</v>
+        <v>580</v>
       </c>
     </row>
     <row r="129">
@@ -7138,18 +7138,18 @@
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Laufey</t>
+          <t>Lísa</t>
         </is>
       </c>
       <c r="J129" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K129" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L129" t="n">
         <v>2</v>
@@ -7158,7 +7158,7 @@
         <v>70</v>
       </c>
       <c r="N129" t="n">
-        <v>70</v>
+        <v>340</v>
       </c>
     </row>
     <row r="130">
@@ -7190,18 +7190,18 @@
       </c>
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Rakel</t>
         </is>
       </c>
       <c r="J130" t="n">
         <v>2</v>
       </c>
       <c r="K130" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="L130" t="n">
         <v>2</v>
@@ -7210,7 +7210,7 @@
         <v>70</v>
       </c>
       <c r="N130" t="n">
-        <v>70</v>
+        <v>570</v>
       </c>
     </row>
     <row r="131">
@@ -7242,18 +7242,18 @@
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Úlfur</t>
+          <t>Kata</t>
         </is>
       </c>
       <c r="J131" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K131" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L131" t="n">
         <v>2</v>
@@ -7262,7 +7262,7 @@
         <v>70</v>
       </c>
       <c r="N131" t="n">
-        <v>240</v>
+        <v>340</v>
       </c>
     </row>
     <row r="132">
@@ -7305,7 +7305,7 @@
         <v>2</v>
       </c>
       <c r="K132" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L132" t="n">
         <v>2</v>
@@ -7314,7 +7314,7 @@
         <v>70</v>
       </c>
       <c r="N132" t="n">
-        <v>240</v>
+        <v>340</v>
       </c>
     </row>
     <row r="133">
@@ -7346,18 +7346,18 @@
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Nanna</t>
+          <t>Silja</t>
         </is>
       </c>
       <c r="J133" t="n">
         <v>1</v>
       </c>
       <c r="K133" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="L133" t="n">
         <v>2</v>
@@ -7366,7 +7366,7 @@
         <v>70</v>
       </c>
       <c r="N133" t="n">
-        <v>260</v>
+        <v>540</v>
       </c>
     </row>
     <row r="134">
@@ -7409,7 +7409,7 @@
         <v>2</v>
       </c>
       <c r="K134" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="L134" t="n">
         <v>2</v>
@@ -7418,7 +7418,7 @@
         <v>70</v>
       </c>
       <c r="N134" t="n">
-        <v>240</v>
+        <v>550</v>
       </c>
     </row>
     <row r="135">
@@ -7450,11 +7450,11 @@
       </c>
       <c r="G135" t="inlineStr"/>
       <c r="H135" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Ylfa</t>
         </is>
       </c>
       <c r="J135" t="n">
@@ -7470,7 +7470,7 @@
         <v>90</v>
       </c>
       <c r="N135" t="n">
-        <v>200</v>
+        <v>470</v>
       </c>
     </row>
     <row r="136">
@@ -7522,7 +7522,7 @@
         <v>100</v>
       </c>
       <c r="N136" t="n">
-        <v>170</v>
+        <v>440</v>
       </c>
     </row>
     <row r="137">
@@ -7574,7 +7574,7 @@
         <v>100</v>
       </c>
       <c r="N137" t="n">
-        <v>170</v>
+        <v>440</v>
       </c>
     </row>
   </sheetData>
@@ -7768,11 +7768,11 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="n">
-        <v>1</v>
-      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
+      <c r="M2" t="n">
+        <v>1</v>
+      </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
@@ -7782,14 +7782,14 @@
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" t="n">
+        <v>1</v>
+      </c>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="n">
-        <v>1</v>
-      </c>
+      <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
@@ -7801,7 +7801,9 @@
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
@@ -7812,23 +7814,21 @@
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="n">
-        <v>1</v>
-      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
         <v>1</v>
       </c>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="n">
-        <v>1</v>
-      </c>
+      <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
+      <c r="U3" t="n">
+        <v>1</v>
+      </c>
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr"/>
@@ -7855,9 +7855,7 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" t="n">
-        <v>1</v>
-      </c>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="n">
         <v>1</v>
       </c>
@@ -7872,15 +7870,15 @@
       <c r="T4" t="n">
         <v>1</v>
       </c>
-      <c r="U4" t="inlineStr"/>
+      <c r="U4" t="n">
+        <v>1</v>
+      </c>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="n">
-        <v>1</v>
-      </c>
+      <c r="AA4" t="inlineStr"/>
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
       <c r="AD4" t="inlineStr"/>
@@ -7902,9 +7900,7 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="n">
-        <v>1</v>
-      </c>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
         <v>1</v>
@@ -7912,13 +7908,13 @@
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
+      <c r="Q5" t="n">
+        <v>1</v>
+      </c>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
-      <c r="U5" t="n">
-        <v>1</v>
-      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr"/>
@@ -7937,11 +7933,11 @@
       <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
       <c r="C6" t="inlineStr"/>
-      <c r="D6" t="n">
-        <v>1</v>
-      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
@@ -7954,13 +7950,13 @@
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
-      <c r="O6" t="n">
-        <v>1</v>
-      </c>
+      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
+      <c r="S6" t="n">
+        <v>1</v>
+      </c>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="n">
         <v>1</v>
@@ -7970,7 +7966,9 @@
       <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
+      <c r="AA6" t="n">
+        <v>1</v>
+      </c>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="inlineStr"/>
@@ -7981,9 +7979,7 @@
       <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="n">
-        <v>1</v>
-      </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
@@ -7991,7 +7987,9 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
         <v>1</v>
@@ -8014,7 +8012,9 @@
       <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr"/>
+      <c r="AA7" t="n">
+        <v>1</v>
+      </c>
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr"/>
@@ -8026,20 +8026,20 @@
         <v>7</v>
       </c>
       <c r="B8" t="inlineStr"/>
-      <c r="C8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
-      <c r="J8" t="n">
-        <v>1</v>
-      </c>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
       <c r="M8" t="n">
         <v>1</v>
       </c>
@@ -8058,7 +8058,9 @@
       <c r="Z8" t="n">
         <v>1</v>
       </c>
-      <c r="AA8" t="inlineStr"/>
+      <c r="AA8" t="n">
+        <v>1</v>
+      </c>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr"/>
@@ -8072,31 +8074,31 @@
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="n">
-        <v>1</v>
-      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" t="n">
-        <v>1</v>
-      </c>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" t="n">
+        <v>1</v>
+      </c>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
+      <c r="Q9" t="n">
+        <v>1</v>
+      </c>
       <c r="R9" t="inlineStr"/>
-      <c r="S9" t="n">
-        <v>1</v>
-      </c>
+      <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
-      <c r="U9" t="n">
-        <v>1</v>
-      </c>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr"/>
@@ -8116,7 +8118,9 @@
         <v>9</v>
       </c>
       <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
@@ -8125,32 +8129,28 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
-      <c r="L10" t="n">
-        <v>1</v>
-      </c>
+      <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
         <v>1</v>
       </c>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
+      <c r="S10" t="n">
+        <v>1</v>
+      </c>
       <c r="T10" t="inlineStr"/>
-      <c r="U10" t="n">
-        <v>1</v>
-      </c>
+      <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr"/>
-      <c r="Z10" t="inlineStr"/>
-      <c r="AA10" t="n">
-        <v>1</v>
-      </c>
+      <c r="Z10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA10" t="inlineStr"/>
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="inlineStr"/>
@@ -8164,10 +8164,10 @@
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
-      <c r="E11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
@@ -8230,15 +8230,17 @@
       <c r="T12" t="n">
         <v>1</v>
       </c>
-      <c r="U12" t="inlineStr"/>
+      <c r="U12" t="n">
+        <v>1</v>
+      </c>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
       <c r="X12" t="inlineStr"/>
       <c r="Y12" t="inlineStr"/>
-      <c r="Z12" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="n">
+        <v>1</v>
+      </c>
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr"/>
       <c r="AD12" t="inlineStr"/>
@@ -8249,7 +8251,9 @@
       <c r="A13" t="n">
         <v>12</v>
       </c>
-      <c r="B13" t="inlineStr"/>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
@@ -8258,19 +8262,19 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="n">
-        <v>1</v>
-      </c>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr"/>
+      <c r="S13" t="n">
+        <v>1</v>
+      </c>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr"/>
@@ -8307,9 +8311,7 @@
         <v>1</v>
       </c>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" t="n">
-        <v>1</v>
-      </c>
+      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
@@ -8318,17 +8320,19 @@
         <v>1</v>
       </c>
       <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
+      <c r="S14" t="n">
+        <v>1</v>
+      </c>
       <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr"/>
+      <c r="U14" t="n">
+        <v>1</v>
+      </c>
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
       <c r="X14" t="inlineStr"/>
       <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="inlineStr"/>
-      <c r="AA14" t="n">
-        <v>1</v>
-      </c>
+      <c r="AA14" t="inlineStr"/>
       <c r="AB14" t="inlineStr"/>
       <c r="AC14" t="inlineStr"/>
       <c r="AD14" t="inlineStr"/>
@@ -8342,18 +8346,20 @@
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="n">
-        <v>1</v>
-      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="n">
-        <v>1</v>
-      </c>
+      <c r="J15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
@@ -8369,10 +8375,10 @@
       <c r="W15" t="inlineStr"/>
       <c r="X15" t="inlineStr"/>
       <c r="Y15" t="inlineStr"/>
-      <c r="Z15" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="n">
+        <v>1</v>
+      </c>
       <c r="AB15" t="inlineStr"/>
       <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="inlineStr"/>
@@ -8391,14 +8397,12 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" t="n">
-        <v>1</v>
-      </c>
-      <c r="K16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="n">
+        <v>1</v>
+      </c>
       <c r="L16" t="inlineStr"/>
-      <c r="M16" t="n">
-        <v>1</v>
-      </c>
+      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
@@ -8408,12 +8412,12 @@
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr"/>
-      <c r="U16" t="n">
-        <v>1</v>
-      </c>
+      <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
+      <c r="X16" t="n">
+        <v>1</v>
+      </c>
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="n">
         <v>1</v>
@@ -8432,7 +8436,9 @@
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
@@ -8443,26 +8449,24 @@
         <v>1</v>
       </c>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="n">
-        <v>1</v>
-      </c>
+      <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
+      <c r="S17" t="n">
+        <v>1</v>
+      </c>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr"/>
       <c r="X17" t="inlineStr"/>
       <c r="Y17" t="inlineStr"/>
-      <c r="Z17" t="inlineStr"/>
-      <c r="AA17" t="n">
-        <v>1</v>
-      </c>
+      <c r="Z17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA17" t="inlineStr"/>
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="inlineStr"/>
@@ -8473,9 +8477,7 @@
       <c r="A18" t="n">
         <v>17</v>
       </c>
-      <c r="B18" t="n">
-        <v>1</v>
-      </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
@@ -8490,32 +8492,36 @@
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
+      <c r="Q18" t="n">
+        <v>1</v>
+      </c>
       <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
+      <c r="S18" t="n">
+        <v>1</v>
+      </c>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr"/>
       <c r="W18" t="inlineStr"/>
       <c r="X18" t="inlineStr"/>
       <c r="Y18" t="inlineStr"/>
-      <c r="Z18" t="inlineStr"/>
-      <c r="AA18" t="n">
-        <v>1</v>
-      </c>
+      <c r="Z18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA18" t="inlineStr"/>
       <c r="AB18" t="inlineStr"/>
       <c r="AC18" t="inlineStr"/>
       <c r="AD18" t="inlineStr"/>
-      <c r="AE18" t="n">
-        <v>1</v>
-      </c>
+      <c r="AE18" t="inlineStr"/>
       <c r="AF18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
         <v>18</v>
       </c>
-      <c r="B19" t="inlineStr"/>
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
@@ -8525,20 +8531,18 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
-      <c r="J19" t="n">
-        <v>1</v>
-      </c>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
+      <c r="L19" t="n">
+        <v>1</v>
+      </c>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
-      <c r="S19" t="n">
-        <v>1</v>
-      </c>
+      <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr"/>
@@ -8562,23 +8566,25 @@
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
+      <c r="J20" t="n">
+        <v>1</v>
+      </c>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
-      <c r="M20" t="n">
-        <v>1</v>
-      </c>
-      <c r="N20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="n">
+        <v>1</v>
+      </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr"/>
@@ -8586,13 +8592,11 @@
       <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr"/>
       <c r="X20" t="inlineStr"/>
-      <c r="Y20" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z20" t="inlineStr"/>
-      <c r="AA20" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y20" t="inlineStr"/>
+      <c r="Z20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA20" t="inlineStr"/>
       <c r="AB20" t="inlineStr"/>
       <c r="AC20" t="inlineStr"/>
       <c r="AD20" t="inlineStr"/>
@@ -8612,28 +8616,28 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
+      <c r="I21" t="n">
+        <v>1</v>
+      </c>
       <c r="J21" t="inlineStr"/>
-      <c r="K21" t="n">
-        <v>1</v>
-      </c>
-      <c r="L21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="n">
+        <v>1</v>
+      </c>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
+      <c r="Q21" t="n">
+        <v>1</v>
+      </c>
       <c r="R21" t="inlineStr"/>
-      <c r="S21" t="n">
-        <v>1</v>
-      </c>
+      <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
-      <c r="X21" t="n">
-        <v>1</v>
-      </c>
+      <c r="X21" t="inlineStr"/>
       <c r="Y21" t="inlineStr"/>
       <c r="Z21" t="inlineStr"/>
       <c r="AA21" t="inlineStr"/>
@@ -8648,21 +8652,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="n">
-        <v>1</v>
-      </c>
+      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="n">
-        <v>1</v>
-      </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="n">
-        <v>1</v>
-      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
@@ -8679,7 +8681,9 @@
       <c r="W22" t="inlineStr"/>
       <c r="X22" t="inlineStr"/>
       <c r="Y22" t="inlineStr"/>
-      <c r="Z22" t="inlineStr"/>
+      <c r="Z22" t="n">
+        <v>1</v>
+      </c>
       <c r="AA22" t="inlineStr"/>
       <c r="AB22" t="inlineStr"/>
       <c r="AC22" t="inlineStr"/>
@@ -8691,28 +8695,28 @@
       <c r="A23" t="n">
         <v>22</v>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="n">
-        <v>1</v>
-      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" t="n">
-        <v>1</v>
-      </c>
-      <c r="K23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="n">
+        <v>1</v>
+      </c>
       <c r="L23" t="inlineStr"/>
-      <c r="M23" t="n">
-        <v>1</v>
-      </c>
+      <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
+      <c r="Q23" t="n">
+        <v>1</v>
+      </c>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr"/>
@@ -8735,9 +8739,7 @@
       <c r="A24" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="n">
-        <v>1</v>
-      </c>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
@@ -8745,30 +8747,32 @@
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="n">
-        <v>1</v>
-      </c>
-      <c r="L24" t="inlineStr"/>
+      <c r="J24" t="n">
+        <v>1</v>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="n">
+        <v>1</v>
+      </c>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
+      <c r="N24" t="n">
+        <v>1</v>
+      </c>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
-      <c r="S24" t="n">
-        <v>1</v>
-      </c>
+      <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr"/>
       <c r="W24" t="inlineStr"/>
       <c r="X24" t="inlineStr"/>
       <c r="Y24" t="inlineStr"/>
-      <c r="Z24" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="n">
+        <v>1</v>
+      </c>
       <c r="AB24" t="inlineStr"/>
       <c r="AC24" t="inlineStr"/>
       <c r="AD24" t="inlineStr"/>
@@ -8779,14 +8783,10 @@
       <c r="A25" t="n">
         <v>24</v>
       </c>
-      <c r="B25" t="n">
-        <v>1</v>
-      </c>
+      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="n">
-        <v>1</v>
-      </c>
+      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
@@ -8800,13 +8800,15 @@
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
+      <c r="Q25" t="n">
+        <v>1</v>
+      </c>
       <c r="R25" t="inlineStr"/>
-      <c r="S25" t="n">
-        <v>1</v>
-      </c>
+      <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
+      <c r="U25" t="n">
+        <v>1</v>
+      </c>
       <c r="V25" t="inlineStr"/>
       <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr"/>
@@ -8816,7 +8818,9 @@
       <c r="AB25" t="inlineStr"/>
       <c r="AC25" t="inlineStr"/>
       <c r="AD25" t="inlineStr"/>
-      <c r="AE25" t="inlineStr"/>
+      <c r="AE25" t="n">
+        <v>1</v>
+      </c>
       <c r="AF25" t="inlineStr"/>
     </row>
     <row r="26">
@@ -8826,9 +8830,7 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="n">
-        <v>1</v>
-      </c>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
@@ -8842,13 +8844,13 @@
       </c>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
+      <c r="O26" t="n">
+        <v>1</v>
+      </c>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
-      <c r="S26" t="n">
-        <v>1</v>
-      </c>
+      <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="inlineStr"/>
@@ -8869,9 +8871,7 @@
       <c r="A27" t="n">
         <v>26</v>
       </c>
-      <c r="B27" t="n">
-        <v>1</v>
-      </c>
+      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
@@ -8894,17 +8894,17 @@
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr"/>
-      <c r="U27" t="n">
-        <v>1</v>
-      </c>
+      <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr"/>
-      <c r="Y27" t="inlineStr"/>
-      <c r="Z27" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA27" t="inlineStr"/>
+      <c r="Y27" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="n">
+        <v>1</v>
+      </c>
       <c r="AB27" t="inlineStr"/>
       <c r="AC27" t="inlineStr"/>
       <c r="AD27" t="inlineStr"/>
@@ -8916,11 +8916,11 @@
         <v>27</v>
       </c>
       <c r="B28" t="inlineStr"/>
-      <c r="C28" t="n">
-        <v>1</v>
-      </c>
+      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
@@ -8934,11 +8934,11 @@
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr"/>
-      <c r="S28" t="inlineStr"/>
+      <c r="S28" t="n">
+        <v>1</v>
+      </c>
       <c r="T28" t="inlineStr"/>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="inlineStr"/>
@@ -8961,38 +8961,38 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
-      <c r="D29" t="n">
-        <v>1</v>
-      </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
+      <c r="J29" t="n">
+        <v>1</v>
+      </c>
       <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
+      <c r="L29" t="n">
+        <v>1</v>
+      </c>
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr"/>
-      <c r="S29" t="n">
-        <v>1</v>
-      </c>
+      <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="inlineStr"/>
       <c r="W29" t="inlineStr"/>
       <c r="X29" t="inlineStr"/>
-      <c r="Y29" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z29" t="inlineStr"/>
-      <c r="AA29" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA29" t="inlineStr"/>
       <c r="AB29" t="inlineStr"/>
       <c r="AC29" t="inlineStr"/>
       <c r="AD29" t="inlineStr"/>
@@ -9006,25 +9006,27 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
-      <c r="E30" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
+      <c r="K30" t="n">
+        <v>1</v>
+      </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
-      <c r="S30" t="inlineStr"/>
+      <c r="S30" t="n">
+        <v>1</v>
+      </c>
       <c r="T30" t="inlineStr"/>
       <c r="U30" t="n">
         <v>1</v>
@@ -9033,9 +9035,7 @@
       <c r="W30" t="inlineStr"/>
       <c r="X30" t="inlineStr"/>
       <c r="Y30" t="inlineStr"/>
-      <c r="Z30" t="n">
-        <v>1</v>
-      </c>
+      <c r="Z30" t="inlineStr"/>
       <c r="AA30" t="inlineStr"/>
       <c r="AB30" t="inlineStr"/>
       <c r="AC30" t="inlineStr"/>
@@ -9048,16 +9048,18 @@
         <v>30</v>
       </c>
       <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="n">
+        <v>1</v>
+      </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
-      <c r="J31" t="n">
-        <v>1</v>
-      </c>
+      <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="n">
         <v>1</v>
@@ -9068,17 +9070,15 @@
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
-      <c r="S31" t="n">
-        <v>1</v>
-      </c>
+      <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr"/>
-      <c r="U31" t="n">
-        <v>1</v>
-      </c>
+      <c r="U31" t="inlineStr"/>
       <c r="V31" t="inlineStr"/>
       <c r="W31" t="inlineStr"/>
       <c r="X31" t="inlineStr"/>
-      <c r="Y31" t="inlineStr"/>
+      <c r="Y31" t="n">
+        <v>1</v>
+      </c>
       <c r="Z31" t="inlineStr"/>
       <c r="AA31" t="inlineStr"/>
       <c r="AB31" t="inlineStr"/>
@@ -9093,19 +9093,19 @@
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="n">
-        <v>1</v>
-      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="n">
-        <v>1</v>
-      </c>
+      <c r="K32" t="n">
+        <v>1</v>
+      </c>
+      <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
@@ -9140,19 +9140,19 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
-      <c r="E33" t="n">
-        <v>1</v>
-      </c>
+      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
+      <c r="J33" t="n">
+        <v>1</v>
+      </c>
       <c r="K33" t="inlineStr"/>
-      <c r="L33" t="n">
-        <v>1</v>
-      </c>
-      <c r="M33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="n">
+        <v>1</v>
+      </c>
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>

</xml_diff>